<commit_message>
chore(artifacts): rebuild after live-render verification
Net data unchanged (verification write was reverted); refreshes the export timestamp and change log.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -555,7 +555,7 @@
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
-          <t>04 Closed</t>
+          <t>01 Open</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -2927,7 +2927,11 @@
           <t>Director, Marketing DS</t>
         </is>
       </c>
-      <c r="C34" t="inlineStr"/>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
@@ -4565,7 +4569,11 @@
           <t>Senior Director, Marketing Science</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr"/>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr">
         <is>
@@ -4575,7 +4583,7 @@
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>03 Applied</t>
         </is>
       </c>
       <c r="H56" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after Built In source and reprioritization
143 -> 188 tracker rows from the first run with Built In wired in and the 100-role cap.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V144"/>
+  <dimension ref="A1:V189"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4968,11 +4968,11 @@
         </is>
       </c>
       <c r="Q61" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>Manager-level individual contributor in brand/advocacy marketing; candidate is a Senior Director running a measurement team — both level and function are off. Customer marketing is about case studies, references, and customer advocacy narratives, not causal measurement or forecasting. The candidate has never built customer-story or advocacy programs; his entire track record is quantitative infrastructure behind marketing decisions, not marketing communications itself. Gaps: No customer advocacy/case-study experience; Function is brand storytelling, not measurement science; Manager title is a level below his current Senior Director scope</t>
+          <t>Manager-level IC role — a step down from the candidate's current Senior Director title and a different function (customer/lifecycle marketing). Customer marketing (case studies, advocacy, industry-vertical customer programs) has no overlap with measurement science or causal inference. It's also a management-level title, below where the candidate sits now. Gaps: No customer marketing/advocacy experience; Title level is a downgrade</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
@@ -5034,11 +5034,11 @@
         </is>
       </c>
       <c r="Q62" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>Field marketing (event/regional campaign execution) is a different discipline entirely from marketing science leadership. Field marketing leads run regional events, pipeline campaigns, and sales-marketing alignment for a vertical — none of which appears in the candidate's background. His public-sector-adjacent experience (Fortune 500 B2B program at Samsung) is about segmentation and measurement, not event/campaign execution. Gaps: No field/event marketing execution experience; No public sector go-to-market background; Function mismatch: campaign execution vs. measurement science</t>
+          <t>Field marketing is an events/pipeline function, unrelated to the candidate's causal measurement track regardless of title level. Field marketing for public sector is about event programs, regional campaigns, and sales-pipeline generation. The candidate has no public-sector GTM or field-marketing background. Gaps: No field/events marketing experience; No public sector domain exposure</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
@@ -5100,11 +5100,11 @@
         </is>
       </c>
       <c r="Q63" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>Manager-level field marketing in a region (APAC/Singapore) the candidate has no footprint in; step down in level and unrelated function. Same function mismatch as the public sector field marketing role, compounded by a geographic relocation to Singapore with no stated candidate presence there. Nothing in the resume touches regional campaign marketing. Gaps: No APAC market experience; No field marketing execution background; Manager level is below current scope</t>
+          <t>Manager-level, wrong function, wrong geography (Singapore) — candidate is NYC-based and has no APAC GTM experience. Same field-marketing mismatch as the public-sector version, compounded by a location and regional-market fit problem. Gaps: No field marketing background; No APAC market experience; Location mismatch</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
@@ -5166,11 +5166,11 @@
         </is>
       </c>
       <c r="Q64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>Software engineering IC role — entirely different skill set and career track. This is a hands-on front-end engineering job (building marketing site/web experiences). The candidate is a data science leader with no front-end engineering background. Gaps: No front-end engineering experience; No web development portfolio; Completely different discipline</t>
+          <t>Wrong track entirely — this is a software engineering IC role (front-end dev), not a data science or measurement position. The candidate manages data science/measurement teams and writes Python for modeling, not production front-end code. Even his 'shipped a forecasting app' work was likely built with an app/eng partner, not hand-coded UI work by him. Gaps: No front-end engineering background (React/JS/etc.); Function is software engineering, not data science</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
@@ -5232,11 +5232,11 @@
         </is>
       </c>
       <c r="Q65" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>"Head of" title suggests real seniority, but the function — community management/enterprise advocacy — is not measurement science and not the candidate's track. Community leadership is about relationship-building, forums, events, and enterprise customer engagement programs. The candidate has managed data science and measurement teams, not community or membership programs, and nothing in his history shows community-building work. Gaps: No community management or developer-relations experience; Function is relationship/engagement-driven, not analytical; No evidence of running member/community programs</t>
+          <t>'Head of' is a senior title, but the function — community management — is unrelated to measurement science or data leadership. Community marketing (developer/customer community programs, forums, events) doesn't touch causal inference, MMM, or attribution. This would be a full discipline change, not a step up or lateral in the candidate's actual expertise. Gaps: No community management experience; No overlap with measurement/causal skill set</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
@@ -5298,11 +5298,11 @@
         </is>
       </c>
       <c r="Q66" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>Lead-level but in co-marketing/alliance function — a track the candidate has never worked in. Partner marketing for cloud (AWS/GCP/Azure co-sell and joint go-to-market) requires alliance management and channel marketing experience. The candidate's entire career is inward-facing measurement and data science, not partner/channel marketing. Gaps: No cloud alliance/partner marketing experience; No co-marketing or channel program background; Domain is partnerships, not causal measurement</t>
+          <t>Lead-level fits seniority-wise, but partner/alliance marketing (AWS/GCP co-marketing) is a distinct function with no relation to measurement science. Partner marketing is about joint GTM motions with cloud hyperscalers — a channel/alliances discipline. Nothing in the candidate's résumé touches partner co-marketing. Gaps: No partner/alliance marketing experience; No cloud channel GTM background</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
@@ -5364,11 +5364,11 @@
         </is>
       </c>
       <c r="Q67" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>Manager-level partner marketing execution role — both a level and function mismatch. This role coordinates partner-tied product launches, a marketing-operations/comms function with no overlap in the candidate's measurement-science background. Gaps: No launch marketing or partner coordination experience; Manager level below current Senior Director scope; No relevant domain overlap</t>
+          <t>Manager-level, same partner-marketing function mismatch as the Lead version, plus a level downgrade. Launch-focused partner marketing coordination has nothing to do with measurement science, and Manager is below the candidate's current scope. Gaps: No partner marketing experience; Title level downgrade</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
@@ -5430,11 +5430,11 @@
         </is>
       </c>
       <c r="Q68" t="n">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>Lead-level title is level-appropriate, but product marketing/GTM strategy is a distinct discipline (positioning, messaging, launch strategy) from marketing science measurement. There's a surface overlap in the phrase "GTM strategy," but this role is about product positioning, narrative, and launch planning for a product line — not causal measurement, forecasting, or experimentation infrastructure. The candidate has never owned product marketing messaging or launch strategy. Gaps: No product marketing/positioning experience; No messaging or narrative-development background; Measurement expertise doesn't translate directly to GTM storytelling</t>
+          <t>Lead-level title is fine, but this is product marketing, a completely different function from data science/measurement leadership. Product marketing GTM strategy is about positioning, messaging, and launch strategy — not causal inference, MMM, or measurement infrastructure. The candidate has zero product marketing background; this is pure function drift off a keyword match on 'GTM.' Gaps: No product marketing experience (positioning, messaging, launch playbooks); No enterprise SaaS GTM strategy track record</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
@@ -5496,11 +5496,11 @@
         </is>
       </c>
       <c r="Q69" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>Manager-level product marketing IC — level and function both misaligned. Same function mismatch as the Lead version above (positioning/messaging vs. measurement), compounded by a manager-level title that is a step down from Senior Director. Gaps: No product marketing experience; Manager title below current level; No messaging/positioning track record</t>
+          <t>Manager-level IC/PMM role — both a level step down from current Senior Director and a track change into product marketing. Same function mismatch as the GTM Lead role, compounded by a lower seniority band. No basis in the resume for product marketing management. Gaps: No product marketing background; Level is below current title</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
@@ -5562,11 +5562,11 @@
         </is>
       </c>
       <c r="Q70" t="n">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>Lead-level is title-appropriate, but solutions marketing (translating technical capability into vertical value props) is a different discipline than measurement science. Solutions marketing is customer-facing technical storytelling for a vertical, not analytics or experimentation work. The candidate's public-sector-adjacent B2B experience (Samsung) was in segmentation and measurement, not solution positioning or sales enablement content. Gaps: No solutions/technical marketing experience; No public sector domain background; Function is narrative/enablement, not measurement</t>
+          <t>Lead-level title is roughly in range, but solutions marketing (translating product capability into sector value props/sales enablement) is a marketing-comms function, not a measurement or data science role. There's a thin conceptual echo — the candidate does translate technical capability into commercial value — but the actual deliverables here (sales enablement content, positioning, competitive narratives) are outside his experience. Public sector is also a new vertical for him. Gaps: No solutions marketing/sales enablement content experience; No public sector domain background</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
@@ -5632,7 +5632,7 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>Manager-level solutions marketing in a vertical (cybersecurity) with no candidate domain background — level and function mismatch. Requires cybersecurity domain fluency and solutions/technical marketing skill, neither of which appears anywhere in the candidate's history. Gaps: No cybersecurity domain expertise; No solutions marketing experience; Manager level below current scope</t>
+          <t>Manager-level is a downgrade from Senior Director, and cybersecurity solutions marketing is a different domain and function. No cybersecurity domain experience and no solutions-marketing/content background. Overlap is essentially zero beyond 'technical enough to talk to a technical buyer.' Gaps: No cybersecurity domain expertise; No solutions marketing experience; Level downgrade</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
@@ -5698,7 +5698,7 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>Manager-level solutions marketing in a vertical (healthcare/science) unrelated to candidate's ad-tech/retail/CPG measurement background. No healthcare or life-sciences domain experience, and the function (solutions marketing) is not measurement science regardless of vertical. Gaps: No healthcare/science domain experience; No solutions marketing background; Manager level below current scope</t>
+          <t>Manager-level downgrade; healthcare/science solutions marketing is a different domain and function from measurement science. No healthcare/life-sciences domain background and no solutions marketing experience. The role wants a domain-fluent content/positioning marketer, not a causal-inference practitioner. Gaps: No healthcare/science domain expertise; No solutions marketing background</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
@@ -5760,11 +5760,11 @@
         </is>
       </c>
       <c r="Q73" t="n">
-        <v>55</v>
+        <v>30</v>
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>Lead-level strategy/ops role is a lateral-to-slightly-different track from Senior Director measurement leadership — plausible if the role leans analytical/forecasting rather than pure program management. This is the one role in the batch with genuine surface logic: the candidate has built forecasting suites, backtesting harnesses, and self-serve planning tools that materially reduced ad-hoc requests from a marketing org — exactly the kind of operational/analytical backbone a Strategy &amp; Ops team needs. The risk is that "Strategy &amp; Ops" at a company like Anthropic often skews toward headcount planning, budget administration, and cross-functional coordination rather than causal measurement, which would waste his core differentiation. Gaps: Unclear if role is analytically-driven (forecasting/planning models) vs. pure operations/coordination; No enterprise SaaS marketing org experience specifically; Would need to confirm the role isn't a generalist chief-of-staff function</t>
+          <t>Lead-level is roughly in range with the candidate's Director/Senior Director track, but this is marketing operations (planning, systems, headcount, process), not measurement science. There's real adjacency — the candidate has built forecasting models, backtesting harnesses, and self-serve planning tools, which is the kind of rigor a marketing strategy &amp; ops function wants. But the role is about running the marketing org's operating cadence, budget/headcount planning, and tooling decisions, not producing causal measurement — a genuine function shift even if the analytical muscle transfers. Gaps: No experience running marketing org operating rhythms/budget-headcount planning as a discipline; No direct marketing-ops tooling (Marketo/Asana/etc.) experience</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
@@ -5826,11 +5826,11 @@
         </is>
       </c>
       <c r="Q74" t="n">
-        <v>48</v>
+        <v>30</v>
       </c>
       <c r="R74" t="inlineStr">
         <is>
-          <t>Lead-level strategy/ops, broader marketing org scope than the enterprise-specific version — same track tension between operations/coordination vs. genuine analytical ownership. Similar logic to the enterprise-marketing variant but less targeted: without the enterprise-marketing specificity, this could skew further toward general program management and comms cadence work, which is a weaker match for a measurement-science background. Still worth a look given the forecasting/tooling overlap, but likely more generalist than the enterprise version. Gaps: Broader/vaguer scope than the enterprise variant makes true overlap harder to gauge; Risk of being a pure operations/PM role with no analytical component; No direct marketing-org-wide strategy experience outside client-facing measurement</t>
+          <t>Same read as the enterprise-marketing variant — level is plausible, function is marketing ops, not measurement science. Same adjacency-but-not-match as the enterprise version: strong forecasting/process background, but the role centers on marketing operating rhythm and resourcing, not causal measurement work. Gaps: No marketing-org operations background specifically; Not clear if this is measurement-adjacent or pure biz-ops</t>
         </is>
       </c>
       <c r="S74" t="inlineStr">
@@ -5892,11 +5892,11 @@
         </is>
       </c>
       <c r="Q75" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="R75" t="inlineStr">
         <is>
-          <t>Director level is a fair title match for a Senior Director; martech/innovation function partially overlaps with the candidate's self-serve tooling and measurement infrastructure work, but core martech-stack ownership (CDP, ad-tech vendor management) isn't proven on his resume. The candidate has real credibility building self-serve tooling and forecasting apps that reduced dependency on the data science team, which is the spirit of "marketing technology innovation." But this role likely centers on martech stack architecture, vendor evaluation, and tooling rollout rather than causal measurement or MMM, which is his real differentiator — so it's a plausible adjacent move, not a clean match. Gaps: No direct martech stack ownership (CDP/marketing automation platform administration) on resume; Unclear overlap between 'innovation' mandate and his measurement/forecasting specialty; Would be moving from client/brand-facing measurement work to Pinterest's internal marketing org tooling</t>
+          <t>Director level matches the candidate's track record exactly (current Senior Director, prior Director titles) — the best level match in this batch. This is the one role in the batch with plausible real overlap: MarTech/measurement tooling could mean owning experimentation infrastructure, self-serve analytics, or attribution stack — all things the candidate has actually built. But the JD excerpt given is just the title, so it's unverified whether this is measurement/analytics-adjacent or pure CRM/campaign-tooling and vendor management, which would be a much weaker match. Gaps: JD detail is too thin to confirm it's a measurement/analytics role vs. pure martech stack/vendor ops; No direct experience owning a MarTech vendor stack (CDP, campaign tools) as the core job, only as an adjacent input to measurement work</t>
         </is>
       </c>
       <c r="S75" t="inlineStr">
@@ -5962,7 +5962,7 @@
       </c>
       <c r="R76" t="inlineStr">
         <is>
-          <t>"Head of" is a senior title, but business marketing in a specific country market (in-market brand/advertiser marketing) is a different function and geography entirely. This role is in-market revenue/brand marketing leadership for Australia — advertiser-facing brand campaigns and local market growth, not measurement science, with no stated candidate presence or experience in the APAC region. Gaps: No in-market/regional business marketing experience; No Australia/APAC footprint; Function is brand/revenue marketing, not causal measurement</t>
+          <t>'Head of' is senior, but this is a P&amp;L/sales-marketing leadership role for a regional ad business, not a measurement science function, and it's in Sydney. Business marketing leadership in a specific geography is a commercial/sales-support leadership role, not a data science or measurement role. Also a relocation to Australia the candidate hasn't signaled interest in. Gaps: No regional business marketing/commercial leadership experience; Location requires relocation to Sydney</t>
         </is>
       </c>
       <c r="S76" t="inlineStr">
@@ -6024,11 +6024,11 @@
         </is>
       </c>
       <c r="Q77" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="R77" t="inlineStr">
         <is>
-          <t>Lead-level PMM title sounds senior, but it's a pure product marketing track — candidate has zero PMM experience at any level. This role is about crafting positioning, narrative, and sales enablement for Pinterest's ad products — a marketing communications function, not measurement science or causal analytics. Nothing in the candidate's decade of MMM/forecasting/segmentation work transfers here. Gaps: No product marketing / messaging / GTM narrative experience; No sales-enablement or product launch marketing background</t>
+          <t>'Lead' + 'Manager' is an IC/senior-IC product marketing title — a track change from the candidate's people-management, measurement-science path. Ads product marketing is about positioning and go-to-market for Pinterest's ad products — sales narratives, launch messaging, competitive positioning — not measurement or causal inference, even though it's ads-adjacent. Gaps: No product marketing experience (positioning, launch narratives, sales collateral); Track change from management to PMM IC work</t>
         </is>
       </c>
       <c r="S77" t="inlineStr">
@@ -6090,11 +6090,11 @@
         </is>
       </c>
       <c r="Q78" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="R78" t="inlineStr">
         <is>
-          <t>"Sr." PMM is a mid-level IC title in a function the candidate has never worked in. Ads Delivery PMM is about explaining delivery/optimization mechanics to advertisers and internal sales — a technical marketing communications role, not data science or measurement. No overlap with the candidate's causal/forecasting background. Gaps: No PMM experience; No ad-delivery/optimization product knowledge</t>
+          <t>Right level band (Sr. Manager) but wrong function entirely — this is product marketing, not measurement science. Ads Product Marketing Manager roles own positioning, sales enablement, and go-to-market narratives for an ad product, not causal measurement or data science. Candidate has zero product marketing experience on the resume. Gaps: No product marketing / positioning experience; No ads-product GTM narrative-building background</t>
         </is>
       </c>
       <c r="S78" t="inlineStr">
@@ -6156,16 +6156,16 @@
         </is>
       </c>
       <c r="Q79" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="R79" t="inlineStr">
         <is>
-          <t>"Sr. Data Scientist" is an IC rung, likely below Staff/Principal — candidate currently manages a team as Senior Director, so this is a track change (manager → IC) and probably a level step-down. Domain is the closest overlap in this batch — marketing data science, forecasting, measurement — but the role is hands-on IC work, not strategy/leadership. Taking it would mean giving up team ownership and executive stakeholder scope the candidate has built over the last two years. Gaps: Level/track mismatch: IC 'Sr' vs current people-manager Senior Director scope; Unclear if role has any leadership or roadmap-ownership component</t>
+          <t>IC 'Sr.' data scientist seat — a track and title step down from candidate's current Senior Director, people-manager role. Domain matches well (marketing data science), and Pinterest's marketing DS org almost certainly touches MMM/incrementality. But the candidate has spent the last 3+ years managing teams of 4-5 and owning strategy, not writing production models solo as an IC. Gaps: IC vs. manager track reversal; Title/level below current Senior Director seat</t>
         </is>
       </c>
       <c r="S79" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>skip</t>
         </is>
       </c>
       <c r="T79" t="inlineStr">
@@ -6230,7 +6230,7 @@
       </c>
       <c r="R80" t="inlineStr">
         <is>
-          <t>Systems/infrastructure engineering IC role — wrong function and wrong track entirely. This is a software/systems engineering role supporting internal sales and marketing tooling. Candidate is a data science/measurement leader, not an infrastructure or platform engineer. Gaps: No systems engineering background; No production infra/ops experience</t>
+          <t>Systems/infrastructure engineering role — no overlap with candidate's data science and measurement track. This is a sales/marketing systems (likely CRM/MarTech infrastructure or internal tooling) engineering role. Nothing in the resume — Python/SQL/Databricks for modeling — substitutes for systems engineering. Gaps: No systems/infrastructure engineering background; Not a measurement or data science role at all</t>
         </is>
       </c>
       <c r="S80" t="inlineStr">
@@ -6292,11 +6292,11 @@
         </is>
       </c>
       <c r="Q81" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="R81" t="inlineStr">
         <is>
-          <t>Staff Software Engineer is a senior IC engineering title — right level of seniority, completely wrong discipline. This requires production software engineering chops (shipping code at Staff level) for growth/performance marketing systems. Candidate's technical work is data science and analytics (Python/SQL/Tableau), not software engineering. Gaps: No software engineering track record; No experience shipping production engineering systems at Staff level</t>
+          <t>Staff Software Engineer is a pure senior IC engineering track — unrelated to the candidate's data science/analytics leadership track. This requires production software engineering chops (shipping code at Staff level), not statistical modeling or measurement leadership. Candidate's stack experience (scikit-learn, SQL, Tableau) doesn't indicate software engineering depth. Gaps: No software engineering track record; Wrong function — growth engineering, not measurement science</t>
         </is>
       </c>
       <c r="S81" t="inlineStr">
@@ -6358,11 +6358,11 @@
         </is>
       </c>
       <c r="Q82" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="R82" t="inlineStr">
         <is>
-          <t>Country Lead is a GM/business-leadership title, not a measurement or data science role — different track and function. This is a market-leadership role running Reddit's UK commercial/marketing business — sales, partnerships, market strategy — not causal measurement or analytics. Candidate has never run a commercial P&amp;L or country business unit. Gaps: No P&amp;L / country-GM experience; No sales/business-leadership track record</t>
+          <t>Country-level commercial/sales leadership role — a different function (ad sales/business leadership) despite a senior title. Country Lead for Business Marketing at a platform typically means owning ad sales, agency relationships, and revenue for a market — not measurement or data science. Candidate has no sales leadership or P&amp;L ownership on the resume. Gaps: No ad sales / commercial leadership experience; No UK market or country-lead P&amp;L experience</t>
         </is>
       </c>
       <c r="S82" t="inlineStr">
@@ -6424,11 +6424,11 @@
         </is>
       </c>
       <c r="Q83" t="n">
-        <v>22</v>
+        <v>38</v>
       </c>
       <c r="R83" t="inlineStr">
         <is>
-          <t>Right seniority band on paper (senior technical/customer-facing), but Applied AI Architect roles typically demand hands-on LLM/agent engineering depth the resume doesn't demonstrate; Singapore location also has no evident connection to candidate. Candidate's Arjentic bullet mentions 'custom agentic solutions' but with no technical detail — nowhere near the depth of production LLM/agent building Anthropic typically hires for. This is an aspirational target role, but the resume as written doesn't support it. Gaps: No demonstrated hands-on LLM/agent engineering track record; No Singapore/APAC connection or relocation signal</t>
+          <t>Title matches a stated career-goal target, but this Singapore-based role is a technical solutions-architecture/pre-sales seat, not a measurement science leadership role, and relocation is a real barrier. The candidate lists 'Applied AI Architect' as a target role, but this JD is almost certainly hands-on LLM/API solution engineering for enterprise customers — a different skill set from the classical ML/causal-inference/MMM toolkit on the resume. Arjentic's 'custom agentic solutions' work is the only real anchor point, and it's thin next to what this role likely demands. Gaps: No demonstrated hands-on LLM application/agent engineering depth at production scale; Singapore location vs. NY base — relocation not indicated as acceptable; Track shift from data science leadership to technical pre-sales/deployment IC work</t>
         </is>
       </c>
       <c r="S83" t="inlineStr">
@@ -6494,11 +6494,11 @@
         </is>
       </c>
       <c r="Q84" t="n">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="R84" t="inlineStr">
         <is>
-          <t>Right general seniority band, wrong vertical domain — no life sciences background at all. This requires deep life sciences domain fluency (clinical, pharma, research workflows) layered on applied AI engineering. Candidate has neither the life sciences domain nor the engineering depth this role needs. Gaps: No life sciences/pharma/biotech domain experience; Same LLM/agent engineering depth gap as other Architect roles</t>
+          <t>Same engineering-heavy Applied AI Architect track mismatch, compounded by a life sciences domain the candidate only touches tangentially (Lilly MMM work was marketing, not clinical/scientific). The Lilly engagement was a pharma marketing measurement project, not life sciences R&amp;D or clinical deployment context, so the domain overlap is thinner than it looks. Combined with the same hands-on AI engineering gap and a London relocation, this is a stretch. Gaps: Life sciences domain is marketing-adjacent only, not clinical/scientific; No hands-on AI solutions engineering evidence; London relocation</t>
         </is>
       </c>
       <c r="S84" t="inlineStr">
@@ -6564,11 +6564,11 @@
         </is>
       </c>
       <c r="Q85" t="n">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="R85" t="inlineStr">
         <is>
-          <t>Right seniority band, wrong domain — no cybersecurity background. This requires cyber domain expertise (threat modeling, security operations) plus applied AI engineering. Candidate's background is marketing measurement science; there's no cyber experience to draw on. NYC location is workable but doesn't offset the domain gap. Gaps: No cybersecurity domain experience; Same engineering-depth gap as other Architect roles</t>
+          <t>Domain is a hard mismatch — no cybersecurity background anywhere in the resume. This vertical requires deep cyber domain fluency (threat detection, security operations) to deploy Claude meaningfully for security customers. Nothing in the candidate's marketing/measurement background transfers. Gaps: No cybersecurity domain experience; No hands-on AI solutions engineering background</t>
         </is>
       </c>
       <c r="S85" t="inlineStr">
@@ -6634,11 +6634,11 @@
         </is>
       </c>
       <c r="Q86" t="n">
-        <v>18</v>
+        <v>35</v>
       </c>
       <c r="R86" t="inlineStr">
         <is>
-          <t>Right seniority band; vertical (digital-native/tech companies) is a closer stretch given candidate's ad-tech/media background, but engineering depth and Munich location are both real gaps. Candidate's media/ad-tech client exposure is a tangential plus for the 'digital natives' vertical, but the role's core ask — deep applied AI/agent engineering with enterprise customers — isn't supported by the resume, and there's no Germany connection. Gaps: No hands-on LLM/agent engineering depth; No Germany/EU relocation signal or language</t>
+          <t>Same track/domain gap as the Singapore Applied AI Architect role, with a Munich location adding another relocation barrier. Nominal title match to a career goal, but the resume shows no evidence of the hands-on LLM/agent deployment engineering this role requires, and it's a track change from measurement science leadership to technical solutions engineering. Gaps: No hands-on LLM/agentic engineering track record at this depth; Munich location — relocation not established; 'Digital Natives Business' segment suggests a specific vertical fluency (fast-growing tech/startups) not reflected in the resume</t>
         </is>
       </c>
       <c r="S86" t="inlineStr">
@@ -6704,11 +6704,11 @@
         </is>
       </c>
       <c r="Q87" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="R87" t="inlineStr">
         <is>
-          <t>Right seniority band; function is partnerships/BD-flavored applied AI, a further drift from candidate's measurement science track, plus Bangalore location mismatch. This blends applied AI engineering with partner/BD relationship management — candidate has neither the engineering depth nor a partnerships track record, and there's no India connection. Gaps: No partnerships/BD experience; No engineering depth or India location fit</t>
+          <t>IC technical-partnerships role; also a track change off the candidate's management line, with no seniority cue in the JD to offset the location and function mismatches. Partnerships-flavored Applied AI Architect roles skew toward technical enablement of ISVs/SIs — a BD-adjacent, partner-facing engineering function distinct from direct client measurement delivery. Bangalore location has no connection to the candidate's NYC-based, US-market career. Gaps: No partnerships/channel-enablement experience — candidate's work has been direct client delivery, not partner-technical-enablement; Bangalore location mismatch with no visible relocation basis; Same hands-on engineering gap as the other two Architect roles</t>
         </is>
       </c>
       <c r="S87" t="inlineStr">
@@ -6774,11 +6774,11 @@
         </is>
       </c>
       <c r="Q88" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="R88" t="inlineStr">
         <is>
-          <t>Right seniority band, entirely wrong domain — national security/public sector work typically requires clearance and government-sector background, neither of which the candidate has. This is a specialized vertical requiring security clearance eligibility and public-sector/defense domain fluency. Candidate's entire career is commercial marketing measurement — no plausible bridge here. Gaps: No security clearance or public-sector background; No national security domain knowledge</t>
+          <t>Hard domain mismatch — public sector/national security requires clearances and government context the candidate has never worked in. Nothing in the resume touches government, defense, or public-sector work, and this role almost certainly requires a security clearance or clearance-eligibility. Pure keyword-only overlap ('Applied AI Architect' title) with none of the substance. Gaps: No public sector / national security experience; Likely requires security clearance the candidate doesn't have</t>
         </is>
       </c>
       <c r="S88" t="inlineStr">
@@ -6844,11 +6844,11 @@
         </is>
       </c>
       <c r="Q89" t="n">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="R89" t="inlineStr">
         <is>
-          <t>Right seniority band and NYC location fits, but this is still an IC-flavored hands-on applied engineering role, and the resume doesn't evidence the LLM/agent building depth Anthropic hires for at this bar. Of the Architect postings this is the most logistically plausible (NYC) and the vertical is generalist rather than domain-locked, but 'Applied AI Architect' at Anthropic is a deeply technical builder role — candidate's stack is data science/analytics tooling, not production AI engineering, and the resume gives no concrete evidence of building/deploying LLM agent systems. Gaps: No demonstrated hands-on LLM/agent engineering portfolio; Career track has been people-management, not individual technical building</t>
+          <t>Startup-vertical solutions engineering, SF/NYC-based (location fits) but same fundamental engineering-track mismatch. Candidate's Arjentic role is itself a small independent studio, which shows some startup-adjacent comfort, but this role wants someone hands-on building and shipping AI solutions fast for startup customers — not measurement strategy. No evidence of that build velocity or engineering depth in the resume. Gaps: No hands-on AI solutions engineering track record; Startup customer-deployment experience unproven</t>
         </is>
       </c>
       <c r="S89" t="inlineStr">
@@ -6918,7 +6918,7 @@
       </c>
       <c r="R90" t="inlineStr">
         <is>
-          <t>Right seniority band and NYC/SF/Seattle location fits; enterprise-tech vertical maps loosely onto candidate's experience with large enterprise stakeholders (Gap, Samsung), but it's still a hands-on engineering role the resume doesn't back up. This is the best-aligned Architect posting for the candidate on paper — enterprise stakeholder navigation is a real strength — but the job is fundamentally a technical AI engineering/deployment role, and nothing in the resume shows the candidate has built or shipped LLM/agent systems at the depth this bar requires. Gaps: No hands-on LLM/agent engineering track record; Would need to reposition from measurement-science leader to technical AI builder</t>
+          <t>Right altitude (senior/staff IC or leadership-adjacent) but wrong track — this is a technical AI-deployment/solutions-architecture seat, not a measurement or marketing-science role. Candidate's 'Field CTO / Head AI Solutions' aspiration points at roles like this, but the actual work is architecting Claude deployments for enterprise customers — a technical AI infrastructure/solutions-engineering skill set the candidate hasn't practiced. His experience is building MMM/attribution/segmentation models and leading measurement teams, not designing LLM integration architectures. Gaps: No hands-on LLM/AI deployment or solutions-architecture experience; No evidence of technical enterprise AI implementation work, only marketing analytics infra</t>
         </is>
       </c>
       <c r="S90" t="inlineStr">
@@ -6984,11 +6984,11 @@
         </is>
       </c>
       <c r="Q91" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R91" t="inlineStr">
         <is>
-          <t>Straight engineering IC role — both a track change (manager → engineer) and a domain mismatch, plus Tokyo location. Applied AI Engineer is a hands-on software/ML engineering role. Candidate has never worked as a software engineer, and there's no Japan connection. Gaps: No software/ML engineering background; No Japan relocation signal or language</t>
+          <t>IC engineering role; candidate is a people-manager/data-science director, not a hands-on AI engineer — and Tokyo location doesn't match candidate base. This is a builder/engineer seat requiring direct AI application development, not marketing measurement or causal inference. Nothing in the resume points to shipping AI engineering deliverables. Gaps: No software/AI engineering track record; Location mismatch (Tokyo)</t>
         </is>
       </c>
       <c r="S91" t="inlineStr">
@@ -7054,11 +7054,11 @@
         </is>
       </c>
       <c r="Q92" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="R92" t="inlineStr">
         <is>
-          <t>Engineering IC role (track change from people-manager) compounded by a life sciences domain the candidate has no experience in; NYC/SF location is the only thing that fits. Requires production engineering skill plus life sciences domain fluency — candidate has neither. Even with the right city, this isn't close. Gaps: No software/ML engineering background; No life sciences domain experience</t>
+          <t>IC engineering role in a domain (life sciences) with zero overlap to candidate's marketing/media measurement background. Both the function (hands-on engineering) and the domain (life sciences) are outside the candidate's experience, which is entirely marketing/media measurement and audience modeling. Gaps: No life sciences domain experience; No applied engineering background</t>
         </is>
       </c>
       <c r="S92" t="inlineStr">
@@ -7124,11 +7124,11 @@
         </is>
       </c>
       <c r="Q93" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="R93" t="inlineStr">
         <is>
-          <t>IC engineering role; candidate is a Senior Director/consultant, not a hands-on production software engineer — a track and level mismatch in both directions. This is a build-and-ship engineering seat requiring production coding for customer integrations. Candidate's Python is analytical (sklearn/statsmodels/SQL), not application engineering, and nothing on the resume shows shipping customer-facing software. Gaps: No production software engineering background; No LLM/agent-building track record; Paris location with no stated relocation</t>
+          <t>Engineer-level IC role is a clear step down from Senior Director and a track change into hands-on engineering — not a fit regardless of domain. Below current level and off-track from data science/measurement leadership into deployment engineering; the Paris location adds a further mismatch. This reads as keyword overlap on 'Applied AI' only. Gaps: Level mismatch — Engineer is below Director/Senior Director; No hands-on software/AI engineering deployment experience at the required depth; Paris location</t>
         </is>
       </c>
       <c r="S93" t="inlineStr">
@@ -7194,11 +7194,11 @@
         </is>
       </c>
       <c r="Q94" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R94" t="inlineStr">
         <is>
-          <t>Same IC engineering track mismatch as the Paris variant; location is better but the core skills gap is unchanged. Requires hands-on engineering delivery, not measurement strategy or team leadership. Candidate's value is in causal/statistical modeling and stakeholder-facing analytics leadership, not writing production integration code. Gaps: No production software engineering portfolio; No evidence of API/infra-level AI engineering work</t>
+          <t>IC engineering role — candidate's track is management/measurement strategy, not hands-on AI engineering. Right city (NY is listed) but wrong function: this seat wants someone building and deploying AI systems directly, whereas the candidate's value is in causal measurement design and leading teams that productionize forecasting/segmentation models — adjacent but not the same skill. Gaps: No direct AI application engineering experience; Resume shows model consumption/oversight, not building AI product integrations</t>
         </is>
       </c>
       <c r="S94" t="inlineStr">
@@ -7268,7 +7268,7 @@
       </c>
       <c r="R95" t="inlineStr">
         <is>
-          <t>Deep ML research/engineering IC role — no overlap with candidate's applied marketing science background. This role sits in model research/engineering, effectively a different discipline than applied marketing measurement. Nothing in the resume points to research-engineering depth (no papers, no model architecture work, no infra-scale ML). Gaps: No research engineering or ML infrastructure experience; No publications or research artifacts</t>
+          <t>Research engineering IC role — far outside candidate's applied marketing-science background. This is a research-engineering seat, almost certainly requiring strong ML research/engineering chops (not marketing measurement, MMM, or attribution). No signal in the resume supports this. Gaps: No ML research or engineering publication/build history; Function is fundamentally different from marketing science leadership</t>
         </is>
       </c>
       <c r="S95" t="inlineStr">
@@ -7334,7 +7334,7 @@
       </c>
       <c r="R96" t="inlineStr">
         <is>
-          <t>Wrong domain entirely (security architecture) and wrong location (London) — not a track candidate should pursue. Security architecture requires a security engineering background the resume does not contain at all. This is pure keyword noise relative to candidate's actual expertise. Gaps: No security engineering/architecture experience anywhere on resume</t>
+          <t>Security architecture is a completely different specialty; no track or domain overlap. Nothing in the candidate's background touches security architecture. This is a pure keyword-only match on 'Applied AI' and should be disregarded. Gaps: No security background; No architecture engineering background; Location mismatch (London)</t>
         </is>
       </c>
       <c r="S96" t="inlineStr">
@@ -7400,11 +7400,11 @@
         </is>
       </c>
       <c r="Q97" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="R97" t="inlineStr">
         <is>
-          <t>Strategist/advisory track loosely matches candidate's consulting experience, but domain is generalist enterprise AI adoption, not measurement science, and location (London) doesn't match. Candidate has genuine client-advisory chops (fractional analytics leadership, Arjentic consulting) and executive-facing communication skill, but this role wants a broad AI-adoption strategist for EMEA enterprise accounts, not a marketing measurement specialist. The domain pivot is real, not just keyword overlap, but unproven at this scope. Gaps: No demonstrated general enterprise AI strategy work beyond marketing/media; London-based role vs. NY-based candidate; No public evidence of technical AI fluency outside of classic ML/stats</t>
+          <t>Plausible altitude (strategist/customer-facing, closer to candidate's consulting/leadership experience) but wrong region and still an AI-deployment strategy role, not measurement science. Of the Anthropic postings, 'Strategist' is the closest in shape to the candidate's consulting and cross-functional leadership work, but it's about driving AI adoption/strategy for enterprise customers in EMEA, not marketing measurement or causal inference — and the location (London) doesn't match. Gaps: No direct AI-adoption consulting experience; EMEA location mismatch; Domain is general AI strategy, not measurement/marketing science</t>
         </is>
       </c>
       <c r="S97" t="inlineStr">
@@ -7470,11 +7470,11 @@
         </is>
       </c>
       <c r="Q98" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R98" t="inlineStr">
         <is>
-          <t>Developer-relations/evangelism IC role — different track (technical community-building) than candidate's client/analytics leadership track. Evangelism roles need live coding demos and startup-developer credibility. Candidate has no developer-relations, conference-speaking-to-engineers, or open-source track record. Gaps: No developer relations or technical evangelism experience; No public code/demo portfolio</t>
+          <t>Developer-relations/evangelism track — not the candidate's people-manager/measurement-science track. This role wants someone embedded in the startup/developer ecosystem doing technical evangelism, a fundamentally different function from measurement science leadership. No signal of dev-relations or startup-ecosystem engagement in the resume. Gaps: No developer relations or technical evangelism experience; No startup ecosystem engagement track record</t>
         </is>
       </c>
       <c r="S98" t="inlineStr">
@@ -7540,11 +7540,11 @@
         </is>
       </c>
       <c r="Q99" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="R99" t="inlineStr">
         <is>
-          <t>Plain 'Data Scientist' IC title is a level drop from Senior Director/Principal Consultant, and the domain (internal engineering metrics) is unrelated to marketing measurement. This is an internal-facing DS role measuring engineering/developer workflows, not commercial/marketing causal inference. Candidate's causal and experimentation skills don't transfer to this specific domain, and the title is a step down. Gaps: No developer-productivity or engineering-metrics domain experience; Title/level is an IC step down from current scope</t>
+          <t>IC data scientist role in a domain (internal dev tooling/productivity metrics) distinct from marketing measurement, and below candidate's management level. The experimentation/causal-inference muscle is relevant in the abstract, but this role measures internal engineering productivity, not commercial/marketing outcomes — a genuine domain switch, and titled as an individual contributor rather than a leadership seat. Gaps: No developer-productivity or engineering-metrics domain experience; IC vs. manager track mismatch</t>
         </is>
       </c>
       <c r="S99" t="inlineStr">
@@ -7606,11 +7606,11 @@
         </is>
       </c>
       <c r="Q100" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="R100" t="inlineStr">
         <is>
-          <t>IC role in AI policy research — both level and domain are off for a marketing science leader. Policy data science involves AI governance/safety research questions, not commercial measurement. Nothing in the resume touches policy, governance, or safety research. Gaps: No policy or AI governance research background; Domain has zero overlap with marketing/media measurement</t>
+          <t>IC data scientist role in policy analytics — no domain or track overlap with candidate's marketing science leadership background. Policy-focused data science (e.g., AI safety/governance analysis) shares almost no surface with marketing measurement, MMM, or attribution work. This is a keyword-only match on 'Data Scientist.' Gaps: No policy or governance analytics experience; Domain entirely unrelated to marketing/commercial measurement</t>
         </is>
       </c>
       <c r="S100" t="inlineStr">
@@ -7672,16 +7672,16 @@
         </is>
       </c>
       <c r="Q101" t="n">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="R101" t="inlineStr">
         <is>
-          <t>Plain IC 'Data Scientist' title is a real step down from Senior Director/Principal Consultant, even though the experimentation angle is the closest domain overlap in this batch. Product data science does involve causal inference and experimentation, which is genuinely in the candidate's wheelhouse, but the title and scope point to an individual-contributor product-analytics role, not measurement leadership. It's the same skill applied to product metrics rather than marketing/media outcomes. Gaps: Title/level is an IC step down from current people-manager scope; No product-analytics (vs. marketing-analytics) domain experience; No B2C product experimentation portfolio specifically</t>
+          <t>Closest domain overlap (product experimentation/causal inference) of the batch, but still an IC data scientist role — a step down from candidate's current Director/team-lead track. Product data science involves A/B testing and causal methods the candidate has real depth in, but the role is almost certainly an individual-contributor seat measuring product usage/feature impact, not marketing/commercial measurement, and would mean giving up his management scope. Gaps: Track change from manager to IC; Domain shift from marketing/media measurement to product analytics; No direct product-metrics/product-experimentation portfolio to point to</t>
         </is>
       </c>
       <c r="S101" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>research</t>
         </is>
       </c>
       <c r="T101" t="inlineStr">
@@ -7738,11 +7738,11 @@
         </is>
       </c>
       <c r="Q102" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="R102" t="inlineStr">
         <is>
-          <t>IC trust-and-safety data science role — domain and level both mismatched. Safeguards work is about abuse/misuse detection and model safety analytics, unrelated to marketing measurement or causal commercial modeling. Gaps: No trust &amp; safety, abuse-detection, or content-moderation analytics experience</t>
+          <t>Title comparison is moot — this is a Trust &amp; Safety / misuse-analytics function, not marketing measurement, so level match doesn't rescue a domain mismatch this wide. Everything on this resume is commercial marketing measurement — MMM, attribution, propensity, segmentation — for retail, CPG, and consumer electronics clients. 'Safeguards' at an AI lab means quantifying model misuse, policy violations, and harm mitigation, a different discipline with different stakeholders, methods, and success metrics. Gaps: No trust &amp; safety, content moderation, or misuse/risk analytics experience anywhere in the work history; No AI safety domain exposure — candidate's causal/experimentation work is entirely commercial (revenue, ROI, budget allocation); Function is risk/policy analytics, not GTM-facing measurement science</t>
         </is>
       </c>
       <c r="S102" t="inlineStr">
@@ -8999,7 +8999,7 @@
       <c r="F121" t="inlineStr"/>
       <c r="G121" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H121" t="inlineStr"/>
@@ -10562,6 +10562,2978 @@
       <c r="U144" t="inlineStr"/>
       <c r="V144" t="inlineStr"/>
     </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>B2B Marketing Lead, India</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr"/>
+      <c r="D145" t="inlineStr"/>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F145" t="inlineStr"/>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H145" t="inlineStr"/>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr"/>
+      <c r="K145" t="inlineStr"/>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/2e127590-8604-4901-ac38-8dfd8e9e255f</t>
+        </is>
+      </c>
+      <c r="M145" t="inlineStr"/>
+      <c r="N145" t="inlineStr"/>
+      <c r="O145" t="inlineStr"/>
+      <c r="P145" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q145" t="n">
+        <v>12</v>
+      </c>
+      <c r="R145" t="inlineStr">
+        <is>
+          <t>Regional B2B marketing lead is a GTM/marketing execution role, not measurement science, at any level. This is a full-stack B2B marketer role owning India GTM, partner and developer programs, and sales enablement. Nothing in the candidate's background is enterprise regional marketing leadership; the causal inference/MMM skill set doesn't transfer here. Gaps: No regional B2B marketing/GTM experience; No India market or sales-led GTM background</t>
+        </is>
+      </c>
+      <c r="S145" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T145" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U145" t="inlineStr"/>
+      <c r="V145" t="inlineStr"/>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Business Operations Manager, Business Marketing</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr"/>
+      <c r="D146" t="inlineStr"/>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F146" t="inlineStr"/>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H146" t="inlineStr"/>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr"/>
+      <c r="K146" t="inlineStr"/>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/2df4df3a-7ac6-42f2-b8ec-d471627a80c8</t>
+        </is>
+      </c>
+      <c r="M146" t="inlineStr"/>
+      <c r="N146" t="inlineStr"/>
+      <c r="O146" t="inlineStr"/>
+      <c r="P146" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q146" t="n">
+        <v>22</v>
+      </c>
+      <c r="R146" t="inlineStr">
+        <is>
+          <t>Ops/strategy manager role inside a marketing org — adjacent function, not a measurement science leadership seat. The role touches 'measurement and organizational learning' but is really strategy &amp; operations support (cadences, portfolio/resource management) for a marketing team, not causal measurement work. Candidate's Director-level measurement leadership doesn't map onto a Biz Ops Manager function. Gaps: No marketing strategy/ops (planning cadences, resourcing) experience; Role is operations support, not owning measurement methodology</t>
+        </is>
+      </c>
+      <c r="S146" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T146" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U146" t="inlineStr"/>
+      <c r="V146" t="inlineStr"/>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Consumer Marketing Lead, Korea</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr"/>
+      <c r="D147" t="inlineStr"/>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F147" t="inlineStr"/>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H147" t="inlineStr"/>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr"/>
+      <c r="K147" t="inlineStr"/>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/2e035bad-8691-4efc-839e-a21b41b7e6fc</t>
+        </is>
+      </c>
+      <c r="M147" t="inlineStr"/>
+      <c r="N147" t="inlineStr"/>
+      <c r="O147" t="inlineStr"/>
+      <c r="P147" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q147" t="n">
+        <v>8</v>
+      </c>
+      <c r="R147" t="inlineStr">
+        <is>
+          <t>Senior regional consumer marketing lead — right seniority word, completely wrong function and market fit. Requires deep Korean cultural/market fluency and full-stack consumer marketing craft (brand, media, launches). No overlap with causal measurement or marketing science. Gaps: No Korea market experience or language/cultural fluency; No consumer brand marketing background</t>
+        </is>
+      </c>
+      <c r="S147" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T147" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U147" t="inlineStr"/>
+      <c r="V147" t="inlineStr"/>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Consumer Marketing Manager, Japan</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr"/>
+      <c r="D148" t="inlineStr"/>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F148" t="inlineStr"/>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H148" t="inlineStr"/>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr"/>
+      <c r="K148" t="inlineStr"/>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/19755930-3377-49c2-949c-192629eb4119</t>
+        </is>
+      </c>
+      <c r="M148" t="inlineStr"/>
+      <c r="N148" t="inlineStr"/>
+      <c r="O148" t="inlineStr"/>
+      <c r="P148" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q148" t="n">
+        <v>6</v>
+      </c>
+      <c r="R148" t="inlineStr">
+        <is>
+          <t>Manager reporting into a Japan Marketing Lead — junior to candidate's current Director level and a different function. Hands-on execution role for locally relevant consumer campaigns in Japan; requires Japanese market fluency and campaign execution skills the candidate doesn't have. Gaps: No Japan market or language experience; No hands-on consumer campaign execution background</t>
+        </is>
+      </c>
+      <c r="S148" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T148" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U148" t="inlineStr"/>
+      <c r="V148" t="inlineStr"/>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Content Marketing Manager, Demand Generation</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr"/>
+      <c r="D149" t="inlineStr"/>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F149" t="inlineStr"/>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H149" t="inlineStr"/>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr"/>
+      <c r="K149" t="inlineStr"/>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/67c67c36-e710-4f21-bd9c-759eb72cfabf</t>
+        </is>
+      </c>
+      <c r="M149" t="inlineStr"/>
+      <c r="N149" t="inlineStr"/>
+      <c r="O149" t="inlineStr"/>
+      <c r="P149" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q149" t="n">
+        <v>6</v>
+      </c>
+      <c r="R149" t="inlineStr">
+        <is>
+          <t>IC content/editorial manager role — unrelated track and level to candidate's measurement leadership background. This is a narrative/content production role (editorial, demos, launches) partnering with product marketing. No causal inference, MMM, or measurement science content. Gaps: No content/editorial marketing production experience; No demand-gen content background</t>
+        </is>
+      </c>
+      <c r="S149" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T149" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U149" t="inlineStr"/>
+      <c r="V149" t="inlineStr"/>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Data Engineer, Core Experimentation</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr"/>
+      <c r="D150" t="inlineStr"/>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F150" t="inlineStr"/>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H150" t="inlineStr"/>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr"/>
+      <c r="K150" t="inlineStr"/>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/2796d32a-9f7c-4008-a2c5-50dd53b0f2fe</t>
+        </is>
+      </c>
+      <c r="M150" t="inlineStr"/>
+      <c r="N150" t="inlineStr"/>
+      <c r="O150" t="inlineStr"/>
+      <c r="P150" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q150" t="n">
+        <v>20</v>
+      </c>
+      <c r="R150" t="inlineStr">
+        <is>
+          <t>Software/data engineering IC role building experimentation infrastructure — a track change from candidate's data science leadership into engineering. Statsig's experimentation platform work is domain-adjacent (experimentation, causal inference infra) but this specific role is data engineering — building and operating pipelines/systems at software-engineering rigor, not designing or leading measurement methodology. Candidate's Python/SQL is analyst-tooling level, not platform engineering. Gaps: No data/software engineering background building production experimentation infrastructure; Would be an IC engineering role, a step down and sideways from Director-level science leadership</t>
+        </is>
+      </c>
+      <c r="S150" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T150" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U150" t="inlineStr"/>
+      <c r="V150" t="inlineStr"/>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Data Scientist, Core Experimentation</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr"/>
+      <c r="D151" t="inlineStr"/>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F151" t="inlineStr"/>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H151" t="inlineStr"/>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr"/>
+      <c r="K151" t="inlineStr"/>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/e90a44a7-fc2e-49bf-aec4-d43b9e3d8e92</t>
+        </is>
+      </c>
+      <c r="M151" t="inlineStr"/>
+      <c r="N151" t="inlineStr"/>
+      <c r="O151" t="inlineStr"/>
+      <c r="P151" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q151" t="n">
+        <v>38</v>
+      </c>
+      <c r="R151" t="inlineStr">
+        <is>
+          <t>Senior IC data scientist role — a track change from people-manager back to individual contributor, likely at a much higher technical bar than agency marketing science. This is the one role in the batch with genuine domain overlap: causal inference and experimentation methodology are core to the candidate's actual expertise. But the work is product/feature experimentation for a frontier AI platform (statistical rigor, platform-scale engineering) rather than marketing measurement, and it's an IC seat while the candidate currently leads a team of 5 as Senior Director. Gaps: Product/feature experimentation platform work differs from marketing MMM/attribution focus; IC role is a track and likely level step down from current people-management scope; No evidence of software engineering rigor needed for platform-scale experimentation systems</t>
+        </is>
+      </c>
+      <c r="S151" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T151" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U151" t="inlineStr"/>
+      <c r="V151" t="inlineStr"/>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Developer Marketing Lead, APAC</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr"/>
+      <c r="D152" t="inlineStr"/>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F152" t="inlineStr"/>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H152" t="inlineStr"/>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr"/>
+      <c r="K152" t="inlineStr"/>
+      <c r="L152" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/98eec6be-1d69-406d-88ba-3cb43f3fcbd7</t>
+        </is>
+      </c>
+      <c r="M152" t="inlineStr"/>
+      <c r="N152" t="inlineStr"/>
+      <c r="O152" t="inlineStr"/>
+      <c r="P152" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q152" t="n">
+        <v>8</v>
+      </c>
+      <c r="R152" t="inlineStr">
+        <is>
+          <t>Senior regional developer marketing lead — wrong function, no developer-audience marketing background. Requires deep technical-audience marketing craft (developer trust, ecosystem activation) across APAC. No connection to measurement science or causal work. Gaps: No developer marketing experience; No APAC regional marketing background</t>
+        </is>
+      </c>
+      <c r="S152" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T152" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U152" t="inlineStr"/>
+      <c r="V152" t="inlineStr"/>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Engineering Manager, Core Experimentation</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr"/>
+      <c r="D153" t="inlineStr"/>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F153" t="inlineStr"/>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H153" t="inlineStr"/>
+      <c r="I153" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J153" t="inlineStr"/>
+      <c r="K153" t="inlineStr"/>
+      <c r="L153" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/eda0d516-94bd-4257-9679-aded0d709fba</t>
+        </is>
+      </c>
+      <c r="M153" t="inlineStr"/>
+      <c r="N153" t="inlineStr"/>
+      <c r="O153" t="inlineStr"/>
+      <c r="P153" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q153" t="n">
+        <v>10</v>
+      </c>
+      <c r="R153" t="inlineStr">
+        <is>
+          <t>Engineering management of software engineers — a completely different management track from data science/measurement leadership. This role manages engineers building the Statsig experimentation platform itself; it requires an engineering management background, not marketing science or data science leadership. Gaps: No software engineering management experience; No platform/infrastructure engineering background</t>
+        </is>
+      </c>
+      <c r="S153" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T153" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U153" t="inlineStr"/>
+      <c r="V153" t="inlineStr"/>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Field Marketing Lead, APAC</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr"/>
+      <c r="D154" t="inlineStr"/>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F154" t="inlineStr"/>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H154" t="inlineStr"/>
+      <c r="I154" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J154" t="inlineStr"/>
+      <c r="K154" t="inlineStr"/>
+      <c r="L154" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/ca869798-6dbc-4673-b15c-a7d00e49630b</t>
+        </is>
+      </c>
+      <c r="M154" t="inlineStr"/>
+      <c r="N154" t="inlineStr"/>
+      <c r="O154" t="inlineStr"/>
+      <c r="P154" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q154" t="inlineStr"/>
+      <c r="R154" t="inlineStr"/>
+      <c r="S154" t="inlineStr"/>
+      <c r="T154" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U154" t="inlineStr"/>
+      <c r="V154" t="inlineStr"/>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Growth - Digital Marketing (Business)</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr"/>
+      <c r="D155" t="inlineStr"/>
+      <c r="E155" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F155" t="inlineStr"/>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H155" t="inlineStr"/>
+      <c r="I155" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J155" t="inlineStr"/>
+      <c r="K155" t="inlineStr"/>
+      <c r="L155" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/079ba35a-b4fa-42a3-92bb-dc31de99d9e3</t>
+        </is>
+      </c>
+      <c r="M155" t="inlineStr"/>
+      <c r="N155" t="inlineStr"/>
+      <c r="O155" t="inlineStr"/>
+      <c r="P155" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q155" t="n">
+        <v>14</v>
+      </c>
+      <c r="R155" t="inlineStr">
+        <is>
+          <t>Senior paid-channel growth marketing leader role — GTM/performance marketing track, not measurement science. This is a performance marketing leadership role (SEM, paid social, programmatic) for B2B self-serve and sales-assisted growth. Candidate has no paid channel management background; overlap is limited to generic 'data-driven' language. Gaps: No paid media/performance marketing channel management experience; No B2B growth funnel ownership background</t>
+        </is>
+      </c>
+      <c r="S155" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T155" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U155" t="inlineStr"/>
+      <c r="V155" t="inlineStr"/>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Growth - Digital Marketing (Consumer)</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr"/>
+      <c r="D156" t="inlineStr"/>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F156" t="inlineStr"/>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H156" t="inlineStr"/>
+      <c r="I156" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J156" t="inlineStr"/>
+      <c r="K156" t="inlineStr"/>
+      <c r="L156" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/b00e0207-d65f-4445-87d5-798f6c895dec</t>
+        </is>
+      </c>
+      <c r="M156" t="inlineStr"/>
+      <c r="N156" t="inlineStr"/>
+      <c r="O156" t="inlineStr"/>
+      <c r="P156" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q156" t="n">
+        <v>12</v>
+      </c>
+      <c r="R156" t="inlineStr">
+        <is>
+          <t>Senior consumer paid-marketing leader — same performance marketing track mismatch as the B2B growth role. Requires hands-on ownership of paid channel strategy and execution across global consumer markets. No fit with causal measurement/marketing science background. Gaps: No paid media channel ownership experience; No consumer growth marketing background</t>
+        </is>
+      </c>
+      <c r="S156" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T156" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U156" t="inlineStr"/>
+      <c r="V156" t="inlineStr"/>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Growth - Digital Marketing (Enterprise)</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr"/>
+      <c r="D157" t="inlineStr"/>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F157" t="inlineStr"/>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H157" t="inlineStr"/>
+      <c r="I157" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J157" t="inlineStr"/>
+      <c r="K157" t="inlineStr"/>
+      <c r="L157" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/2b9fa1aa-d844-4aa5-a762-6ac9bbb27d33</t>
+        </is>
+      </c>
+      <c r="M157" t="inlineStr"/>
+      <c r="N157" t="inlineStr"/>
+      <c r="O157" t="inlineStr"/>
+      <c r="P157" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q157" t="n">
+        <v>14</v>
+      </c>
+      <c r="R157" t="inlineStr">
+        <is>
+          <t>Senior enterprise paid-marketing/ABM leader — GTM/demand-gen track, not measurement science. Focused on ABM and paid demand gen for complex enterprise buying journeys; candidate's background is in measurement strategy, not campaign/channel execution or ABM program ownership. Gaps: No ABM or enterprise paid demand-gen experience; No channel strategy ownership background</t>
+        </is>
+      </c>
+      <c r="S157" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T157" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U157" t="inlineStr"/>
+      <c r="V157" t="inlineStr"/>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Growth Marketing, Creative and Ad Operations</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr"/>
+      <c r="D158" t="inlineStr"/>
+      <c r="E158" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H158" t="inlineStr"/>
+      <c r="I158" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J158" t="inlineStr"/>
+      <c r="K158" t="inlineStr"/>
+      <c r="L158" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/1ae64ddb-505f-4ad2-a731-3a857e94edee</t>
+        </is>
+      </c>
+      <c r="M158" t="inlineStr"/>
+      <c r="N158" t="inlineStr"/>
+      <c r="O158" t="inlineStr"/>
+      <c r="P158" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q158" t="n">
+        <v>6</v>
+      </c>
+      <c r="R158" t="inlineStr">
+        <is>
+          <t>Creative/ad ops execution role — unrelated function and track. This role is about creative production and ad operations workflows, not measurement or causal analysis. Gaps: No creative/ad operations experience; No relevant execution background</t>
+        </is>
+      </c>
+      <c r="S158" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T158" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U158" t="inlineStr"/>
+      <c r="V158" t="inlineStr"/>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Growth Marketing Manager, SMB Ads</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr"/>
+      <c r="D159" t="inlineStr"/>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F159" t="inlineStr"/>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H159" t="inlineStr"/>
+      <c r="I159" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J159" t="inlineStr"/>
+      <c r="K159" t="inlineStr"/>
+      <c r="L159" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/dc503400-f7a8-4ad4-b50b-b33d2d12cc2d</t>
+        </is>
+      </c>
+      <c r="M159" t="inlineStr"/>
+      <c r="N159" t="inlineStr"/>
+      <c r="O159" t="inlineStr"/>
+      <c r="P159" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q159" t="n">
+        <v>8</v>
+      </c>
+      <c r="R159" t="inlineStr">
+        <is>
+          <t>Manager-level execution role for SMB advertiser growth — junior to candidate's current level and a different function. Hands-on growth program execution for small-business advertisers; not a measurement science or strategy seat, and 'Manager' here sits below candidate's current Senior Director scope. Gaps: No SMB/advertiser growth marketing experience; Role level is below candidate's current title and scope</t>
+        </is>
+      </c>
+      <c r="S159" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T159" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U159" t="inlineStr"/>
+      <c r="V159" t="inlineStr"/>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Head of Ads Enterprise Marketing</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr"/>
+      <c r="D160" t="inlineStr"/>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F160" t="inlineStr"/>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H160" t="inlineStr"/>
+      <c r="I160" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J160" t="inlineStr"/>
+      <c r="K160" t="inlineStr"/>
+      <c r="L160" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/a7f4ec2e-e93f-4f81-892a-cd8381f347fe</t>
+        </is>
+      </c>
+      <c r="M160" t="inlineStr"/>
+      <c r="N160" t="inlineStr"/>
+      <c r="O160" t="inlineStr"/>
+      <c r="P160" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q160" t="n">
+        <v>18</v>
+      </c>
+      <c r="R160" t="inlineStr">
+        <is>
+          <t>Head-level leadership title matches candidate's seniority, but the function is ads monetization/GTM marketing, not measurement science. This is a marketing leadership role defining monetization strategy and GTM for OpenAI's ads business — leadership altitude fits, but the domain is ads product marketing and sales partnership, not causal measurement, MMM, or experimentation. Gaps: No ads/monetization product marketing experience; No GTM leadership track record outside measurement science</t>
+        </is>
+      </c>
+      <c r="S160" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T160" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U160" t="inlineStr"/>
+      <c r="V160" t="inlineStr"/>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Head of Marketing Technology (MarTech)</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr"/>
+      <c r="D161" t="inlineStr"/>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F161" t="inlineStr"/>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H161" t="inlineStr"/>
+      <c r="I161" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J161" t="inlineStr"/>
+      <c r="K161" t="inlineStr"/>
+      <c r="L161" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/50ab21f6-475d-4911-984d-7d2727e72ea1</t>
+        </is>
+      </c>
+      <c r="M161" t="inlineStr"/>
+      <c r="N161" t="inlineStr"/>
+      <c r="O161" t="inlineStr"/>
+      <c r="P161" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q161" t="n">
+        <v>30</v>
+      </c>
+      <c r="R161" t="inlineStr">
+        <is>
+          <t>Head-level title lines up with Director seniority, but this is a MarTech/marketing-ops infrastructure lead, not a measurement science role — different function at the right level. Candidate has adjacent CDP/marketing-data-infrastructure experience (Samsung enterprise CDP, product+engineering roadmap ownership) but this role is about building the operating model, systems, and agentic workflows behind marketing execution — not causal measurement, MMM, or experimentation. It's a stack-and-ops job wearing an AI wrapper. Gaps: No marketing ops/tooling-architecture track record (vs. measurement/analytics track); JD wants IT/Security/Eng systems ownership, not causal inference or forecasting</t>
+        </is>
+      </c>
+      <c r="S161" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T161" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U161" t="inlineStr"/>
+      <c r="V161" t="inlineStr"/>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Industry Product Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr"/>
+      <c r="D162" t="inlineStr"/>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F162" t="inlineStr"/>
+      <c r="G162" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H162" t="inlineStr"/>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J162" t="inlineStr"/>
+      <c r="K162" t="inlineStr"/>
+      <c r="L162" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/0e078d07-fb0b-4893-b90a-f50e413f3e13</t>
+        </is>
+      </c>
+      <c r="M162" t="inlineStr"/>
+      <c r="N162" t="inlineStr"/>
+      <c r="O162" t="inlineStr"/>
+      <c r="P162" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q162" t="n">
+        <v>15</v>
+      </c>
+      <c r="R162" t="inlineStr">
+        <is>
+          <t>Manager-level IC product marketing role — wrong track (PMM, not measurement) and a step down from Senior Director. This is narrative and positioning work for industry verticals, not measurement, causal inference, or experimentation. Candidate's resume has zero product marketing or messaging experience. Gaps: No product marketing or narrative-building experience; Function is GTM storytelling, not measurement science</t>
+        </is>
+      </c>
+      <c r="S162" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T162" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U162" t="inlineStr"/>
+      <c r="V162" t="inlineStr"/>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Integrated Marketing Lead, Brand &amp; Policy</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr"/>
+      <c r="D163" t="inlineStr"/>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F163" t="inlineStr"/>
+      <c r="G163" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H163" t="inlineStr"/>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J163" t="inlineStr"/>
+      <c r="K163" t="inlineStr"/>
+      <c r="L163" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/9e39d2ba-2076-4f44-9e07-c8520e9d5cdb</t>
+        </is>
+      </c>
+      <c r="M163" t="inlineStr"/>
+      <c r="N163" t="inlineStr"/>
+      <c r="O163" t="inlineStr"/>
+      <c r="P163" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q163" t="n">
+        <v>12</v>
+      </c>
+      <c r="R163" t="inlineStr">
+        <is>
+          <t>Lead-level title but a brand/policy comms role — wrong function entirely. This is reputation and policy narrative work sitting between Comms, Global Affairs, and Creative. Nothing in the candidate's background (causal measurement, MMM, forecasting) applies here. Gaps: No brand/policy communications background; No experience partnering with Global Affairs or Comms</t>
+        </is>
+      </c>
+      <c r="S163" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T163" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U163" t="inlineStr"/>
+      <c r="V163" t="inlineStr"/>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Integrated Marketing Manager, Developers</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr"/>
+      <c r="D164" t="inlineStr"/>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F164" t="inlineStr"/>
+      <c r="G164" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H164" t="inlineStr"/>
+      <c r="I164" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J164" t="inlineStr"/>
+      <c r="K164" t="inlineStr"/>
+      <c r="L164" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/39256344-0da0-4a5d-bd65-5438d94f7738</t>
+        </is>
+      </c>
+      <c r="M164" t="inlineStr"/>
+      <c r="N164" t="inlineStr"/>
+      <c r="O164" t="inlineStr"/>
+      <c r="P164" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q164" t="n">
+        <v>12</v>
+      </c>
+      <c r="R164" t="inlineStr">
+        <is>
+          <t>Manager-level IC integrated marketing role — track and level mismatch (people-manager Director into an execution-focused IC marketing seat). Campaign/launch execution for a developer audience. No measurement, causal inference, or MMM component; candidate has no developer-relations or campaign-management background. Gaps: No integrated campaign execution experience; No developer-audience marketing background</t>
+        </is>
+      </c>
+      <c r="S164" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T164" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U164" t="inlineStr"/>
+      <c r="V164" t="inlineStr"/>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Integrated Marketing Manager, Product &amp; Model Launches</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr"/>
+      <c r="D165" t="inlineStr"/>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F165" t="inlineStr"/>
+      <c r="G165" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H165" t="inlineStr"/>
+      <c r="I165" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J165" t="inlineStr"/>
+      <c r="K165" t="inlineStr"/>
+      <c r="L165" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/c5d0b0d2-7f17-4981-b224-adb1414c5158</t>
+        </is>
+      </c>
+      <c r="M165" t="inlineStr"/>
+      <c r="N165" t="inlineStr"/>
+      <c r="O165" t="inlineStr"/>
+      <c r="P165" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q165" t="n">
+        <v>12</v>
+      </c>
+      <c r="R165" t="inlineStr">
+        <is>
+          <t>Same as above — IC campaign manager role, level and function mismatch. This is launch-campaign strategy and execution across product/model releases, not measurement or causal analysis. No overlap with candidate's actual skill set. Gaps: No launch/campaign management experience; No product marketing background</t>
+        </is>
+      </c>
+      <c r="S165" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T165" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U165" t="inlineStr"/>
+      <c r="V165" t="inlineStr"/>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Lifecycle Marketing Manager, SMB Ads</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr"/>
+      <c r="D166" t="inlineStr"/>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F166" t="inlineStr"/>
+      <c r="G166" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H166" t="inlineStr"/>
+      <c r="I166" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J166" t="inlineStr"/>
+      <c r="K166" t="inlineStr"/>
+      <c r="L166" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/31f7b3d9-eb5f-4e70-98ab-9115dd153993</t>
+        </is>
+      </c>
+      <c r="M166" t="inlineStr"/>
+      <c r="N166" t="inlineStr"/>
+      <c r="O166" t="inlineStr"/>
+      <c r="P166" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q166" t="n">
+        <v>22</v>
+      </c>
+      <c r="R166" t="inlineStr">
+        <is>
+          <t>Manager-level IC lifecycle marketing role — track mismatch (people-manager into hands-on CRM/lifecycle execution) and a step down from Director. Mentions experimentation and Data Science partnership, which is the only real overlap, but the job is owning lifecycle/CRM programs for SMB advertisers, not designing or owning measurement methodology. Candidate has no lifecycle marketing or ads-product ownership experience. Gaps: No lifecycle/CRM program ownership; Role is ads-product growth, not measurement leadership</t>
+        </is>
+      </c>
+      <c r="S166" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T166" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U166" t="inlineStr"/>
+      <c r="V166" t="inlineStr"/>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Marketing Scientist - EMEA (London)</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr"/>
+      <c r="D167" t="inlineStr"/>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F167" t="inlineStr"/>
+      <c r="G167" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H167" t="inlineStr"/>
+      <c r="I167" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J167" t="inlineStr"/>
+      <c r="K167" t="inlineStr"/>
+      <c r="L167" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/aa55ee20-b904-44c1-8cc7-d9160fc8b341</t>
+        </is>
+      </c>
+      <c r="M167" t="inlineStr"/>
+      <c r="N167" t="inlineStr"/>
+      <c r="O167" t="inlineStr"/>
+      <c r="P167" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q167" t="n">
+        <v>45</v>
+      </c>
+      <c r="R167" t="inlineStr">
+        <is>
+          <t>Title reads as an IC 'Scientist' role — likely below Senior Director level, and it's in London while candidate is NY-based; the domain (data-driven market/monetization strategy) is the closest overlap in this batch but is skewed toward pricing/monetization research rather than media measurement/MMM/incrementality. This is the only role in the batch with 'Marketing Scientist' in the title and a data-driven, cross-functional analytics mandate. But the JD emphasizes monetization strategy and market dynamics, not the causal media measurement (MMM, MTA, geo-lift) that is the candidate's actual specialty, and the level/location both look like a step down and a relocation ask. Gaps: Location mismatch (London vs. NY, no relocation signal); Title suggests IC scientist, not a Director-level leadership seat; JD leans monetization/pricing science, not media MMM/incrementality</t>
+        </is>
+      </c>
+      <c r="S167" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="T167" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U167" t="inlineStr"/>
+      <c r="V167" t="inlineStr"/>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Partner Marketing Manager, Ads</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr"/>
+      <c r="D168" t="inlineStr"/>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F168" t="inlineStr"/>
+      <c r="G168" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H168" t="inlineStr"/>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J168" t="inlineStr"/>
+      <c r="K168" t="inlineStr"/>
+      <c r="L168" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/66fa2750-ca23-4a3e-8970-dfe7bac97d01</t>
+        </is>
+      </c>
+      <c r="M168" t="inlineStr"/>
+      <c r="N168" t="inlineStr"/>
+      <c r="O168" t="inlineStr"/>
+      <c r="P168" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q168" t="n">
+        <v>12</v>
+      </c>
+      <c r="R168" t="inlineStr">
+        <is>
+          <t>Manager-level IC partnerships role — wrong function and a step down. Ecosystem/partner enablement for ads measurement and agency partners, not a measurement science or analytics role itself. Candidate has no partner marketing experience. Gaps: No partner/ecosystem marketing background; Role is partnerships management, not analytics</t>
+        </is>
+      </c>
+      <c r="S168" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T168" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U168" t="inlineStr"/>
+      <c r="V168" t="inlineStr"/>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Partner Marketing Manager, AWS</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr"/>
+      <c r="D169" t="inlineStr"/>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F169" t="inlineStr"/>
+      <c r="G169" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H169" t="inlineStr"/>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J169" t="inlineStr"/>
+      <c r="K169" t="inlineStr"/>
+      <c r="L169" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/73f27385-2b31-49da-bc57-92e6f194c73e</t>
+        </is>
+      </c>
+      <c r="M169" t="inlineStr"/>
+      <c r="N169" t="inlineStr"/>
+      <c r="O169" t="inlineStr"/>
+      <c r="P169" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q169" t="n">
+        <v>10</v>
+      </c>
+      <c r="R169" t="inlineStr">
+        <is>
+          <t>Manager-level IC partner marketing role — wrong function and level. Cloud co-sell/GTM partnership management with AWS. No measurement or causal inference component at all. Gaps: No cloud partner/co-sell marketing experience; Function is partnerships, not analytics</t>
+        </is>
+      </c>
+      <c r="S169" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T169" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U169" t="inlineStr"/>
+      <c r="V169" t="inlineStr"/>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Partner Marketing Manager, GCP &amp; Oracle</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr"/>
+      <c r="D170" t="inlineStr"/>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F170" t="inlineStr"/>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr"/>
+      <c r="I170" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J170" t="inlineStr"/>
+      <c r="K170" t="inlineStr"/>
+      <c r="L170" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/f352f3e4-491c-4f6a-a7b6-68292283702d</t>
+        </is>
+      </c>
+      <c r="M170" t="inlineStr"/>
+      <c r="N170" t="inlineStr"/>
+      <c r="O170" t="inlineStr"/>
+      <c r="P170" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q170" t="n">
+        <v>10</v>
+      </c>
+      <c r="R170" t="inlineStr">
+        <is>
+          <t>Same as AWS partner role — IC partnerships, wrong function/level. Identical mismatch to the AWS partner marketing manager role, just a different cloud partner portfolio. Gaps: No cloud partner marketing experience; Function is partnerships, not measurement</t>
+        </is>
+      </c>
+      <c r="S170" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T170" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U170" t="inlineStr"/>
+      <c r="V170" t="inlineStr"/>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Partner Marketing Manager, Hardware</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr"/>
+      <c r="D171" t="inlineStr"/>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F171" t="inlineStr"/>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr"/>
+      <c r="I171" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J171" t="inlineStr"/>
+      <c r="K171" t="inlineStr"/>
+      <c r="L171" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/958eecd4-7446-445c-ae93-62c38436aa22</t>
+        </is>
+      </c>
+      <c r="M171" t="inlineStr"/>
+      <c r="N171" t="inlineStr"/>
+      <c r="O171" t="inlineStr"/>
+      <c r="P171" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q171" t="n">
+        <v>10</v>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>IC partner marketing role, wrong function/level. Hardware partner marketing execution — no measurement, causal inference, or analytics content. Gaps: No hardware partner marketing experience; Function is partnerships, not analytics</t>
+        </is>
+      </c>
+      <c r="S171" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T171" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U171" t="inlineStr"/>
+      <c r="V171" t="inlineStr"/>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Partner Marketing Manager, Technology Partners &amp; ISVs</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr"/>
+      <c r="D172" t="inlineStr"/>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr"/>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr"/>
+      <c r="I172" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J172" t="inlineStr"/>
+      <c r="K172" t="inlineStr"/>
+      <c r="L172" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/333ebd68-cc1d-4706-8d0a-07f3e50d7bfd</t>
+        </is>
+      </c>
+      <c r="M172" t="inlineStr"/>
+      <c r="N172" t="inlineStr"/>
+      <c r="O172" t="inlineStr"/>
+      <c r="P172" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q172" t="n">
+        <v>10</v>
+      </c>
+      <c r="R172" t="inlineStr">
+        <is>
+          <t>IC partner marketing role, wrong function/level. ISV/technology partner GTM management — same mismatch pattern as the other partner marketing roles. Gaps: No ISV/technology partner marketing experience; Function is partnerships, not analytics</t>
+        </is>
+      </c>
+      <c r="S172" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T172" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U172" t="inlineStr"/>
+      <c r="V172" t="inlineStr"/>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Product Manager, Safety Measurement</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr"/>
+      <c r="D173" t="inlineStr"/>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr"/>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr"/>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J173" t="inlineStr"/>
+      <c r="K173" t="inlineStr"/>
+      <c r="L173" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/fbc7ebaf-3a26-406d-9ff6-f166f3e246a2</t>
+        </is>
+      </c>
+      <c r="M173" t="inlineStr"/>
+      <c r="N173" t="inlineStr"/>
+      <c r="O173" t="inlineStr"/>
+      <c r="P173" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q173" t="n">
+        <v>18</v>
+      </c>
+      <c r="R173" t="inlineStr">
+        <is>
+          <t>PM-track role in AI safety, not marketing/GTM measurement — domain drift despite the 'measurement' keyword. This measures harm and safeguard efficacy for frontier model safety, a completely different discipline from marketing measurement science (MMM, attribution, incrementality). Surface keyword match only. Gaps: No AI safety/red-teaming background; Not a product management track</t>
+        </is>
+      </c>
+      <c r="S173" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T173" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U173" t="inlineStr"/>
+      <c r="V173" t="inlineStr"/>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Product Marketing Lead, API Models &amp; Research</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr"/>
+      <c r="D174" t="inlineStr"/>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr"/>
+      <c r="I174" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J174" t="inlineStr"/>
+      <c r="K174" t="inlineStr"/>
+      <c r="L174" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/38388825-65f9-46c5-b5f4-c783d1fb17d4</t>
+        </is>
+      </c>
+      <c r="M174" t="inlineStr"/>
+      <c r="N174" t="inlineStr"/>
+      <c r="O174" t="inlineStr"/>
+      <c r="P174" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q174" t="n">
+        <v>18</v>
+      </c>
+      <c r="R174" t="inlineStr">
+        <is>
+          <t>Lead-level seniority is a plausible level match, but the function (product marketing/narrative) is not measurement science. Senior PMM role translating research/model capability into market narrative and GTM strategy. Candidate has never done product marketing, positioning, or narrative work — the resume is entirely measurement and data science delivery. Gaps: No product marketing or narrative-strategy experience; No direct research-to-market translation background</t>
+        </is>
+      </c>
+      <c r="S174" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T174" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U174" t="inlineStr"/>
+      <c r="V174" t="inlineStr"/>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Product Marketing Lead, ChatGPT Work</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr"/>
+      <c r="D175" t="inlineStr"/>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr"/>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr"/>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J175" t="inlineStr"/>
+      <c r="K175" t="inlineStr"/>
+      <c r="L175" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/d45d6005-ad46-4c3c-8cfc-d312bffe01d5</t>
+        </is>
+      </c>
+      <c r="M175" t="inlineStr"/>
+      <c r="N175" t="inlineStr"/>
+      <c r="O175" t="inlineStr"/>
+      <c r="P175" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q175" t="n">
+        <v>18</v>
+      </c>
+      <c r="R175" t="inlineStr">
+        <is>
+          <t>Lead-level seniority matches, but function (product marketing strategy/narrative) does not. Owning strategy and narrative for a product line is a PMM leadership job, not a measurement/causal inference job. No overlap beyond seniority level. Gaps: No product marketing leadership experience; No narrative/positioning track record</t>
+        </is>
+      </c>
+      <c r="S175" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T175" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U175" t="inlineStr"/>
+      <c r="V175" t="inlineStr"/>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Product Marketing Lead, Executive Engagement</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr"/>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr"/>
+      <c r="I176" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J176" t="inlineStr"/>
+      <c r="K176" t="inlineStr"/>
+      <c r="L176" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/3c5ebd43-1f83-422b-9e44-94b96bc8e4e0</t>
+        </is>
+      </c>
+      <c r="M176" t="inlineStr"/>
+      <c r="N176" t="inlineStr"/>
+      <c r="O176" t="inlineStr"/>
+      <c r="P176" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q176" t="n">
+        <v>20</v>
+      </c>
+      <c r="R176" t="inlineStr">
+        <is>
+          <t>Lead-level seniority is plausible, but this is executive-briefing/narrative PMM work, not measurement. The only faint overlap is that candidate has presented model outputs and rationale to planning/strategy stakeholders (Gap Inc. work), but this role is fundamentally about crafting executive-facing product narrative, not building or owning measurement systems. Gaps: No product marketing or executive-narrative background; Not a measurement/analytics role despite senior level</t>
+        </is>
+      </c>
+      <c r="S176" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T176" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U176" t="inlineStr"/>
+      <c r="V176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Product Marketing Manager, Cybersecurity</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr"/>
+      <c r="D177" t="inlineStr"/>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr"/>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr"/>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J177" t="inlineStr"/>
+      <c r="K177" t="inlineStr"/>
+      <c r="L177" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/9c990e11-a5fb-4c6d-ab83-ede32839e78e</t>
+        </is>
+      </c>
+      <c r="M177" t="inlineStr"/>
+      <c r="N177" t="inlineStr"/>
+      <c r="O177" t="inlineStr"/>
+      <c r="P177" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q177" t="n">
+        <v>8</v>
+      </c>
+      <c r="R177" t="inlineStr">
+        <is>
+          <t>Product marketing IC role; candidate has never done product marketing, this is a function change not a level change. This is a cybersecurity go-to-market/narrative role for product marketers, not a measurement or data science position. Nothing in the candidate's causal inference, MMM, or forecasting background maps to positioning and field enablement for a security product line. Gaps: No product marketing experience; No cybersecurity domain background</t>
+        </is>
+      </c>
+      <c r="S177" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T177" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U177" t="inlineStr"/>
+      <c r="V177" t="inlineStr"/>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Product Marketing Manager, IT Admin and Governance</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr"/>
+      <c r="D178" t="inlineStr"/>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr"/>
+      <c r="I178" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J178" t="inlineStr"/>
+      <c r="K178" t="inlineStr"/>
+      <c r="L178" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/c6cb3f11-8e1f-4e34-b407-6a3327e39f2e</t>
+        </is>
+      </c>
+      <c r="M178" t="inlineStr"/>
+      <c r="N178" t="inlineStr"/>
+      <c r="O178" t="inlineStr"/>
+      <c r="P178" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q178" t="n">
+        <v>8</v>
+      </c>
+      <c r="R178" t="inlineStr">
+        <is>
+          <t>Product marketing IC role; wrong function entirely for this candidate. Owning the admin/governance experience messaging for ChatGPT Work and Codex is product marketing, not measurement science. There's no attribution, incrementality, or causal inference component here at all. Gaps: No product marketing background; No IT admin/governance domain experience</t>
+        </is>
+      </c>
+      <c r="S178" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T178" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U178" t="inlineStr"/>
+      <c r="V178" t="inlineStr"/>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Product Marketing Manager, Research &amp; Safety</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr"/>
+      <c r="D179" t="inlineStr"/>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr"/>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr"/>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J179" t="inlineStr"/>
+      <c r="K179" t="inlineStr"/>
+      <c r="L179" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/f630d886-76d4-4492-a06b-7c6a34d05b8f</t>
+        </is>
+      </c>
+      <c r="M179" t="inlineStr"/>
+      <c r="N179" t="inlineStr"/>
+      <c r="O179" t="inlineStr"/>
+      <c r="P179" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q179" t="n">
+        <v>8</v>
+      </c>
+      <c r="R179" t="inlineStr">
+        <is>
+          <t>Product marketing IC role; not this candidate's track. Research &amp; Safety PMM is about translating research narrative into market-facing messaging, not measurement, experimentation design, or causal analysis. Pure function drift. Gaps: No product marketing experience; No research communications background</t>
+        </is>
+      </c>
+      <c r="S179" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T179" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U179" t="inlineStr"/>
+      <c r="V179" t="inlineStr"/>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Program Manager, Business Marketing</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr"/>
+      <c r="D180" t="inlineStr"/>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F180" t="inlineStr"/>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr"/>
+      <c r="I180" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J180" t="inlineStr"/>
+      <c r="K180" t="inlineStr"/>
+      <c r="L180" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/3ed37e51-40dc-4d17-8219-d3500af8892c</t>
+        </is>
+      </c>
+      <c r="M180" t="inlineStr"/>
+      <c r="N180" t="inlineStr"/>
+      <c r="O180" t="inlineStr"/>
+      <c r="P180" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q180" t="n">
+        <v>15</v>
+      </c>
+      <c r="R180" t="inlineStr">
+        <is>
+          <t>Ops/program management role; candidate is a technical measurement leader, not a marketing operations PM. This is about operating cadences, portfolio management, and prioritization systems for a marketing org — program/ops skillset, not analytics or measurement leadership, even though the team touches 'measurement and organizational learning' tangentially. Gaps: No program/ops management track record; Not a measurement or data science role despite the team name</t>
+        </is>
+      </c>
+      <c r="S180" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T180" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U180" t="inlineStr"/>
+      <c r="V180" t="inlineStr"/>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Secure Manufacturing &amp; Stealth Partner, Marketing</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr"/>
+      <c r="D181" t="inlineStr"/>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F181" t="inlineStr"/>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr"/>
+      <c r="I181" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J181" t="inlineStr"/>
+      <c r="K181" t="inlineStr"/>
+      <c r="L181" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/dbfc77d3-8b6f-4a82-bb14-53eeaa6c4124</t>
+        </is>
+      </c>
+      <c r="M181" t="inlineStr"/>
+      <c r="N181" t="inlineStr"/>
+      <c r="O181" t="inlineStr"/>
+      <c r="P181" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q181" t="n">
+        <v>3</v>
+      </c>
+      <c r="R181" t="inlineStr">
+        <is>
+          <t>Corporate security/counter-espionage role embedded in Marketing — unrelated track and domain. This is a security and information-control function (protecting launch secrecy, embedding OPSEC into marketing production), with zero overlap with measurement, causal inference, or marketing science. Gaps: No security/OPSEC background; Not an analytics or measurement role at all</t>
+        </is>
+      </c>
+      <c r="S181" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T181" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U181" t="inlineStr"/>
+      <c r="V181" t="inlineStr"/>
+    </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Senior Marketing Strategist, Paid &amp; New Demand Channels</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr"/>
+      <c r="D182" t="inlineStr"/>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F182" t="inlineStr"/>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/f269776d-f2e2-4e65-aafa-7b62cb381594</t>
+        </is>
+      </c>
+      <c r="M182" t="inlineStr"/>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
+      <c r="P182" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q182" t="n">
+        <v>28</v>
+      </c>
+      <c r="R182" t="inlineStr">
+        <is>
+          <t>Senior IC/strategist role in performance marketing — adjacent domain (media spend, channel ROI) but a demand-gen execution role, not measurement science leadership. There's real surface overlap — media spend, channel-level performance, ROI reconciliation are things the candidate has done (MMM vendor reconciliation at OMD) — but this role is about running and scaling paid/demand channels themselves, not building the measurement infrastructure behind them. It's closer to a media buyer/growth marketer function than a data science lead role. Gaps: No hands-on paid media buying/channel execution experience; Role is demand-gen ownership, not measurement/analytics leadership</t>
+        </is>
+      </c>
+      <c r="S182" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T182" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U182" t="inlineStr"/>
+      <c r="V182" t="inlineStr"/>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Software Engineer, Full-Stack - Core Experimentation</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr"/>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr"/>
+      <c r="I183" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J183" t="inlineStr"/>
+      <c r="K183" t="inlineStr"/>
+      <c r="L183" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/73e56947-5d8b-414d-a0ac-9dc9b04e2406</t>
+        </is>
+      </c>
+      <c r="M183" t="inlineStr"/>
+      <c r="N183" t="inlineStr"/>
+      <c r="O183" t="inlineStr"/>
+      <c r="P183" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q183" t="n">
+        <v>12</v>
+      </c>
+      <c r="R183" t="inlineStr">
+        <is>
+          <t>Software engineering IC role; candidate is not a software engineer and has no full-stack engineering background. Despite the appealing keyword ('Core Experimentation', 'experimentation platform'), this is a hands-on full-stack SWE role building the Statsig platform itself. The candidate consumes and designs experiments, he doesn't build experimentation infrastructure in code. Gaps: No software engineering track record; Resume shows no production systems engineering, only modeling/analytics</t>
+        </is>
+      </c>
+      <c r="S183" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T183" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U183" t="inlineStr"/>
+      <c r="V183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Software Engineer, Infrastructure - Core Experimentation</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr"/>
+      <c r="D184" t="inlineStr"/>
+      <c r="E184" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr"/>
+      <c r="I184" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J184" t="inlineStr"/>
+      <c r="K184" t="inlineStr"/>
+      <c r="L184" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/823a05bf-33fb-4d94-9dd8-571723d27b1a</t>
+        </is>
+      </c>
+      <c r="M184" t="inlineStr"/>
+      <c r="N184" t="inlineStr"/>
+      <c r="O184" t="inlineStr"/>
+      <c r="P184" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q184" t="n">
+        <v>10</v>
+      </c>
+      <c r="R184" t="inlineStr">
+        <is>
+          <t>Infrastructure engineering IC role; same mismatch as the full-stack variant, and infra engineering is even further from the candidate's stack. This needs distributed-systems/infrastructure engineering skill to build the experimentation platform's backend, not someone who designs or interprets experiments. The 'experimentation' keyword is the only overlap and it's superficial. Gaps: No infrastructure/backend engineering experience; Not a data science or measurement role despite adjacent team name</t>
+        </is>
+      </c>
+      <c r="S184" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T184" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U184" t="inlineStr"/>
+      <c r="V184" t="inlineStr"/>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Startup Content Marketing Manager</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr"/>
+      <c r="D185" t="inlineStr"/>
+      <c r="E185" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F185" t="inlineStr"/>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr"/>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J185" t="inlineStr"/>
+      <c r="K185" t="inlineStr"/>
+      <c r="L185" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/45d0ccb6-d26f-4b1f-b24d-fe67ec5b708a</t>
+        </is>
+      </c>
+      <c r="M185" t="inlineStr"/>
+      <c r="N185" t="inlineStr"/>
+      <c r="O185" t="inlineStr"/>
+      <c r="P185" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q185" t="n">
+        <v>6</v>
+      </c>
+      <c r="R185" t="inlineStr">
+        <is>
+          <t>Content marketing IC role, unrelated track. This is content creation and editorial strategy for the startup ecosystem audience — writing and content programs, not measurement or causal analysis. Gaps: No content marketing/editorial background; No measurement component to the role</t>
+        </is>
+      </c>
+      <c r="S185" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T185" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U185" t="inlineStr"/>
+      <c r="V185" t="inlineStr"/>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Strategic Finance, International &amp; Marketing</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr"/>
+      <c r="D186" t="inlineStr"/>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr"/>
+      <c r="I186" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J186" t="inlineStr"/>
+      <c r="K186" t="inlineStr"/>
+      <c r="L186" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/5b85c0cc-3f19-4b96-9bd3-3b7521e54f44</t>
+        </is>
+      </c>
+      <c r="M186" t="inlineStr"/>
+      <c r="N186" t="inlineStr"/>
+      <c r="O186" t="inlineStr"/>
+      <c r="P186" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q186" t="n">
+        <v>18</v>
+      </c>
+      <c r="R186" t="inlineStr">
+        <is>
+          <t>Senior strategic finance partner role — right seniority band conceptually, but wrong function (FP&amp;A, not measurement science). The role touches marketing effectiveness and uses data to guide investment decisions, which sounds adjacent, but it's a strategic finance/FP&amp;A seat advising regional GMs on operating models — not a measurement or causal inference role. The candidate has no finance/FP&amp;A background. Gaps: No strategic finance or FP&amp;A experience; No track record owning headcount/OpEx/revenue operating models</t>
+        </is>
+      </c>
+      <c r="S186" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T186" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U186" t="inlineStr"/>
+      <c r="V186" t="inlineStr"/>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Acceleration Partners</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Associate Director / Director, Data Strategy &amp; Measurement</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr"/>
+      <c r="D187" t="inlineStr"/>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F187" t="inlineStr"/>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr"/>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J187" t="inlineStr"/>
+      <c r="K187" t="inlineStr"/>
+      <c r="L187" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/director-data-strategy-measurement/11055963</t>
+        </is>
+      </c>
+      <c r="M187" t="inlineStr"/>
+      <c r="N187" t="inlineStr"/>
+      <c r="O187" t="inlineStr"/>
+      <c r="P187" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q187" t="n">
+        <v>74</v>
+      </c>
+      <c r="R187" t="inlineStr">
+        <is>
+          <t>Director-level people-manager role — matches current Senior Director level and track closely. This is a genuine match: attribution, incrementality, and MMM advisory work for enterprise clients, building measurement frameworks, and coaching talent — essentially the same function the candidate runs at OMD, just in an agency/consultancy client-advisory format rather than in-house. Level and track both line up cleanly. Gaps: No direct affiliate/partnership marketing channel experience (Acceleration Partners' core vertical); Role is fully remote/Sun Belt-based, not NY — relocation or remote-work fit needs confirming</t>
+        </is>
+      </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>apply</t>
+        </is>
+      </c>
+      <c r="T187" t="inlineStr">
+        <is>
+          <t>Marketing - Performance Marketing</t>
+        </is>
+      </c>
+      <c r="U187" t="inlineStr"/>
+      <c r="V187" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Advansys</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Measurement Engineer</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr"/>
+      <c r="D188" t="inlineStr"/>
+      <c r="E188" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr"/>
+      <c r="I188" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J188" t="inlineStr"/>
+      <c r="K188" t="inlineStr"/>
+      <c r="L188" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/measurement-engineer/11033734</t>
+        </is>
+      </c>
+      <c r="M188" t="inlineStr"/>
+      <c r="N188" t="inlineStr"/>
+      <c r="O188" t="inlineStr"/>
+      <c r="P188" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q188" t="n">
+        <v>15</v>
+      </c>
+      <c r="R188" t="inlineStr">
+        <is>
+          <t>IC engineering role, junior/mid-level title ('Engineer') — a level and domain mismatch for a Senior Director. This is industrial/operational measurement (Balanced Scorecard reporting, dashboards, root-cause analysis on operational data) at what reads as a manufacturing or operations context, not marketing measurement science. Title and scope are also well below the candidate's current level. Gaps: Wrong domain — operational/industrial measurement, not marketing/causal measurement; Title and scope are individual-contributor engineer level, a step down from Senior Director</t>
+        </is>
+      </c>
+      <c r="S188" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T188" t="inlineStr">
+        <is>
+          <t>Tech - Industrial Software</t>
+        </is>
+      </c>
+      <c r="U188" t="inlineStr"/>
+      <c r="V188" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Agentio</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Marketing Science Lead</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr"/>
+      <c r="D189" t="inlineStr"/>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F189" t="inlineStr"/>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr"/>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J189" t="inlineStr"/>
+      <c r="K189" t="inlineStr"/>
+      <c r="L189" t="inlineStr">
+        <is>
+          <t>https://builtin.com/job/marketing-science-lead/8328709</t>
+        </is>
+      </c>
+      <c r="M189" t="inlineStr"/>
+      <c r="N189" t="inlineStr"/>
+      <c r="O189" t="inlineStr"/>
+      <c r="P189" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q189" t="n">
+        <v>68</v>
+      </c>
+      <c r="R189" t="inlineStr">
+        <is>
+          <t>Title matches exactly ('Marketing Science Lead'), but likely a smaller-scope, more hands-on IC-heavy seat at a startup versus leading a 5-person team at a media holding company — probably a lateral move in title, modest step down in scope. Domain and title are a near-perfect match on paper — measurement frameworks, creator marketing, hands-on analysis is exactly the candidate's lane. The open question is whether this is a real leadership seat or a solo-IC 'lead' title at an early-stage company, and creator/influencer marketing measurement is a narrower niche than the candidate's broader cross-channel MMM/attribution background. Gaps: No direct creator/influencer marketing measurement experience; Company stage/team size unclear — may be a solo IC role despite the 'Lead' title</t>
+        </is>
+      </c>
+      <c r="S189" t="inlineStr">
+        <is>
+          <t>research</t>
+        </is>
+      </c>
+      <c r="T189" t="inlineStr">
+        <is>
+          <t>Tech - AI Recruitment</t>
+        </is>
+      </c>
+      <c r="U189" t="inlineStr"/>
+      <c r="V189" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after live-scan quota change
188 -> 200-capacity judging queue; tracker/db reflect the new mix.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -6389,7 +6389,11 @@
           <t>Applied AI Architect</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr"/>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr">
         <is>
@@ -6599,7 +6603,11 @@
           <t>Applied AI Architect, Digital Natives Business</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr"/>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after add_role no-scan fix; widen auto-close list
Includes the OpenAI TPM role added during verification, plus an existing broadening of rules.auto_close_titles to bare 'engineer'/'manager'.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V467"/>
+  <dimension ref="A1:V468"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -29809,7 +29809,7 @@
       <c r="F430" t="inlineStr"/>
       <c r="G430" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H430" t="inlineStr"/>
@@ -29879,7 +29879,7 @@
       <c r="F431" t="inlineStr"/>
       <c r="G431" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H431" t="inlineStr"/>
@@ -29945,7 +29945,7 @@
       <c r="F432" t="inlineStr"/>
       <c r="G432" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H432" t="inlineStr"/>
@@ -30011,7 +30011,7 @@
       <c r="F433" t="inlineStr"/>
       <c r="G433" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H433" t="inlineStr"/>
@@ -30081,7 +30081,7 @@
       <c r="F434" t="inlineStr"/>
       <c r="G434" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H434" t="inlineStr"/>
@@ -30147,7 +30147,7 @@
       <c r="F435" t="inlineStr"/>
       <c r="G435" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H435" t="inlineStr"/>
@@ -30217,7 +30217,7 @@
       <c r="F436" t="inlineStr"/>
       <c r="G436" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H436" t="inlineStr"/>
@@ -30287,7 +30287,7 @@
       <c r="F437" t="inlineStr"/>
       <c r="G437" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H437" t="inlineStr"/>
@@ -30357,7 +30357,7 @@
       <c r="F438" t="inlineStr"/>
       <c r="G438" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H438" t="inlineStr"/>
@@ -30427,7 +30427,7 @@
       <c r="F439" t="inlineStr"/>
       <c r="G439" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H439" t="inlineStr"/>
@@ -30493,7 +30493,7 @@
       <c r="F440" t="inlineStr"/>
       <c r="G440" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H440" t="inlineStr"/>
@@ -30559,7 +30559,7 @@
       <c r="F441" t="inlineStr"/>
       <c r="G441" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H441" t="inlineStr"/>
@@ -30629,7 +30629,7 @@
       <c r="F442" t="inlineStr"/>
       <c r="G442" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H442" t="inlineStr"/>
@@ -30699,7 +30699,7 @@
       <c r="F443" t="inlineStr"/>
       <c r="G443" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H443" t="inlineStr"/>
@@ -30769,7 +30769,7 @@
       <c r="F444" t="inlineStr"/>
       <c r="G444" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H444" t="inlineStr"/>
@@ -30839,7 +30839,7 @@
       <c r="F445" t="inlineStr"/>
       <c r="G445" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H445" t="inlineStr"/>
@@ -30905,7 +30905,7 @@
       <c r="F446" t="inlineStr"/>
       <c r="G446" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H446" t="inlineStr"/>
@@ -30975,7 +30975,7 @@
       <c r="F447" t="inlineStr"/>
       <c r="G447" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H447" t="inlineStr"/>
@@ -31045,7 +31045,7 @@
       <c r="F448" t="inlineStr"/>
       <c r="G448" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H448" t="inlineStr"/>
@@ -31115,7 +31115,7 @@
       <c r="F449" t="inlineStr"/>
       <c r="G449" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H449" t="inlineStr"/>
@@ -31185,7 +31185,7 @@
       <c r="F450" t="inlineStr"/>
       <c r="G450" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H450" t="inlineStr"/>
@@ -32416,6 +32416,80 @@
         </is>
       </c>
     </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Technical Program Manager, Compute Infrastructure</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr"/>
+      <c r="D468" t="inlineStr"/>
+      <c r="E468" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F468" t="inlineStr"/>
+      <c r="G468" t="inlineStr">
+        <is>
+          <t>01 Open</t>
+        </is>
+      </c>
+      <c r="H468" t="inlineStr"/>
+      <c r="I468" t="inlineStr">
+        <is>
+          <t>manual-add</t>
+        </is>
+      </c>
+      <c r="J468" t="inlineStr"/>
+      <c r="K468" t="inlineStr"/>
+      <c r="L468" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/openai/8fb1615c-34bf-47c4-a1d1-b7b2f836bbd3</t>
+        </is>
+      </c>
+      <c r="M468" t="inlineStr">
+        <is>
+          <t>$257,000 - $335,000 per year</t>
+        </is>
+      </c>
+      <c r="N468" t="inlineStr"/>
+      <c r="O468" t="inlineStr"/>
+      <c r="P468" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q468" t="n">
+        <v>4</v>
+      </c>
+      <c r="R468" t="inlineStr">
+        <is>
+          <t>Irrelevant axis — this isn't a measurement/data-science role at any level, it's a hardware/datacenter TPM role. This is a technical program management role for GPU cluster bring-up: hardware, networking, power, cooling, vendor/construction coordination. Nothing in the candidate's background — MMM, attribution, causal inference, marketing analytics leadership — maps to running compute infrastructure delivery. Gaps: No infrastructure/hyperscaler program management experience (capital projects, networking, power/cooling); No TPM track record; candidate is a data science/analytics people-manager, not an engineering program manager</t>
+        </is>
+      </c>
+      <c r="S468" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T468" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U468" t="inlineStr"/>
+      <c r="V468" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist (high)</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after link/notes/salary/category-accept changes
120 roles auto-accepted from cached suggestions; new Salary column populated where discoverable.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V468"/>
+  <dimension ref="A1:V470"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3507,7 +3507,11 @@
           <t>Senior Manager, Measurement - APAC</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr"/>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D42" t="n">
         <v>2</v>
       </c>
@@ -3572,11 +3576,7 @@
         </is>
       </c>
       <c r="U42" t="inlineStr"/>
-      <c r="V42" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3901,7 +3901,11 @@
           <t>Sr. Staff Data Scientist - Ads Measurement, Signals, Privacy</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr"/>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D47" t="n">
         <v>2</v>
       </c>
@@ -3966,11 +3970,7 @@
         </is>
       </c>
       <c r="U47" t="inlineStr"/>
-      <c r="V47" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -3983,7 +3983,11 @@
           <t>Staff Data Scientist - Ads Measurement, Signals, Privacy</t>
         </is>
       </c>
-      <c r="C48" t="inlineStr"/>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D48" t="n">
         <v>2</v>
       </c>
@@ -4048,11 +4052,7 @@
         </is>
       </c>
       <c r="U48" t="inlineStr"/>
-      <c r="V48" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4065,7 +4065,11 @@
           <t>Staff Data Scientist - Ads Measurement, Signals, Privacy</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr"/>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D49" t="n">
         <v>2</v>
       </c>
@@ -4130,11 +4134,7 @@
         </is>
       </c>
       <c r="U49" t="inlineStr"/>
-      <c r="V49" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4425,7 +4425,11 @@
           <t>Partner, Insights &amp; Analytics</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr"/>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>05 Practice Lead at Consultancy</t>
+        </is>
+      </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr">
         <is>
@@ -4482,11 +4486,7 @@
         </is>
       </c>
       <c r="U54" t="inlineStr"/>
-      <c r="V54" t="inlineStr">
-        <is>
-          <t>05 Practice Lead at Consultancy (medium)</t>
-        </is>
-      </c>
+      <c r="V54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4643,7 +4643,11 @@
           <t>Director of Applied AI/ML Science - Ads</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr"/>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr">
         <is>
@@ -4700,11 +4704,7 @@
         </is>
       </c>
       <c r="U57" t="inlineStr"/>
-      <c r="V57" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -6459,7 +6459,11 @@
           <t>Applied AI Architect, Beneficial Deployments (Life Sciences)</t>
         </is>
       </c>
-      <c r="C84" t="inlineStr"/>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr">
         <is>
@@ -6512,11 +6516,7 @@
         </is>
       </c>
       <c r="U84" t="inlineStr"/>
-      <c r="V84" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6529,7 +6529,11 @@
           <t>Applied AI Architect, Cyber</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr"/>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr">
         <is>
@@ -6582,11 +6586,7 @@
         </is>
       </c>
       <c r="U85" t="inlineStr"/>
-      <c r="V85" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -6669,7 +6669,11 @@
           <t>Applied AI Architect, Partnerships</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr"/>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D87" t="inlineStr"/>
       <c r="E87" t="inlineStr">
         <is>
@@ -6722,11 +6726,7 @@
         </is>
       </c>
       <c r="U87" t="inlineStr"/>
-      <c r="V87" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -6739,7 +6739,11 @@
           <t>Applied AI Architect, Public Sector (National Security)</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr"/>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D88" t="inlineStr"/>
       <c r="E88" t="inlineStr">
         <is>
@@ -6792,11 +6796,7 @@
         </is>
       </c>
       <c r="U88" t="inlineStr"/>
-      <c r="V88" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -6809,7 +6809,11 @@
           <t>Applied AI Architect, Startups</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr"/>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D89" t="inlineStr"/>
       <c r="E89" t="inlineStr">
         <is>
@@ -6862,11 +6866,7 @@
         </is>
       </c>
       <c r="U89" t="inlineStr"/>
-      <c r="V89" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -6879,7 +6879,11 @@
           <t>Applied AI Architect, Strategic Enterprise Tech</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr"/>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D90" t="inlineStr"/>
       <c r="E90" t="inlineStr">
         <is>
@@ -6932,11 +6936,7 @@
         </is>
       </c>
       <c r="U90" t="inlineStr"/>
-      <c r="V90" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7901,7 +7901,11 @@
           <t>Manager, Applied AI Architect, Enterprise Tech</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr"/>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D105" t="inlineStr"/>
       <c r="E105" t="inlineStr">
         <is>
@@ -7954,11 +7958,7 @@
         </is>
       </c>
       <c r="U105" t="inlineStr"/>
-      <c r="V105" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -7971,7 +7971,11 @@
           <t>Manager Applied AI Architecture, Financial Services</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr"/>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D106" t="inlineStr"/>
       <c r="E106" t="inlineStr">
         <is>
@@ -8024,11 +8028,7 @@
         </is>
       </c>
       <c r="U106" t="inlineStr"/>
-      <c r="V106" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8111,7 +8111,11 @@
           <t>Manager, Applied AI Engineering,  Beneficial Deployments (Life Sciences)</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr"/>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D108" t="inlineStr"/>
       <c r="E108" t="inlineStr">
         <is>
@@ -8164,11 +8168,7 @@
         </is>
       </c>
       <c r="U108" t="inlineStr"/>
-      <c r="V108" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8181,7 +8181,11 @@
           <t>Manager, Forward Deployed Engineering</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr"/>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D109" t="inlineStr"/>
       <c r="E109" t="inlineStr">
         <is>
@@ -8234,11 +8238,7 @@
         </is>
       </c>
       <c r="U109" t="inlineStr"/>
-      <c r="V109" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -8251,7 +8251,11 @@
           <t>Manager of Applied AI Architecture, Commercial</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr"/>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D110" t="inlineStr"/>
       <c r="E110" t="inlineStr">
         <is>
@@ -8304,11 +8308,7 @@
         </is>
       </c>
       <c r="U110" t="inlineStr"/>
-      <c r="V110" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -8321,7 +8321,11 @@
           <t>Pre-Sales Program Lead, Forward Deployed Engineering</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr"/>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D111" t="inlineStr"/>
       <c r="E111" t="inlineStr">
         <is>
@@ -8374,11 +8378,7 @@
         </is>
       </c>
       <c r="U111" t="inlineStr"/>
-      <c r="V111" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -8523,7 +8523,11 @@
           <t>Strategy &amp; Operations, Applied AI - AMER</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr"/>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D114" t="inlineStr"/>
       <c r="E114" t="inlineStr">
         <is>
@@ -8576,11 +8580,7 @@
         </is>
       </c>
       <c r="U114" t="inlineStr"/>
-      <c r="V114" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -13415,7 +13415,11 @@
           <t>Measurement Engineer</t>
         </is>
       </c>
-      <c r="C188" t="inlineStr"/>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D188" t="inlineStr"/>
       <c r="E188" t="inlineStr">
         <is>
@@ -13468,11 +13472,7 @@
         </is>
       </c>
       <c r="U188" t="inlineStr"/>
-      <c r="V188" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -13625,7 +13625,11 @@
           <t>Consultant (Manager), Marketing Science Analytics</t>
         </is>
       </c>
-      <c r="C191" t="inlineStr"/>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>05 Practice Lead at Consultancy</t>
+        </is>
+      </c>
       <c r="D191" t="inlineStr"/>
       <c r="E191" t="inlineStr">
         <is>
@@ -13678,11 +13682,7 @@
         </is>
       </c>
       <c r="U191" t="inlineStr"/>
-      <c r="V191" t="inlineStr">
-        <is>
-          <t>05 Practice Lead at Consultancy (high)</t>
-        </is>
-      </c>
+      <c r="V191" t="inlineStr"/>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -13695,7 +13695,11 @@
           <t>Consultant, Marketing Science Analytics</t>
         </is>
       </c>
-      <c r="C192" t="inlineStr"/>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>05 Practice Lead at Consultancy</t>
+        </is>
+      </c>
       <c r="D192" t="inlineStr"/>
       <c r="E192" t="inlineStr">
         <is>
@@ -13748,11 +13752,7 @@
         </is>
       </c>
       <c r="U192" t="inlineStr"/>
-      <c r="V192" t="inlineStr">
-        <is>
-          <t>05 Practice Lead at Consultancy (high)</t>
-        </is>
-      </c>
+      <c r="V192" t="inlineStr"/>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -13765,7 +13765,11 @@
           <t>Director of Marketing Science Analytics &amp; Commercial Intelligence (Customer Engagement Team)</t>
         </is>
       </c>
-      <c r="C193" t="inlineStr"/>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>05 Practice Lead at Consultancy</t>
+        </is>
+      </c>
       <c r="D193" t="inlineStr"/>
       <c r="E193" t="inlineStr">
         <is>
@@ -13818,11 +13822,7 @@
         </is>
       </c>
       <c r="U193" t="inlineStr"/>
-      <c r="V193" t="inlineStr">
-        <is>
-          <t>05 Practice Lead at Consultancy (high)</t>
-        </is>
-      </c>
+      <c r="V193" t="inlineStr"/>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -14367,7 +14367,11 @@
           <t>Lead of Digital Marketing Measurement and Data Science</t>
         </is>
       </c>
-      <c r="C202" t="inlineStr"/>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D202" t="inlineStr"/>
       <c r="E202" t="inlineStr">
         <is>
@@ -14420,11 +14424,7 @@
         </is>
       </c>
       <c r="U202" t="inlineStr"/>
-      <c r="V202" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -14771,7 +14771,11 @@
           <t>Senior Lead Software Engineer, Marketing and Messaging Experimentation</t>
         </is>
       </c>
-      <c r="C208" t="inlineStr"/>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D208" t="inlineStr"/>
       <c r="E208" t="inlineStr">
         <is>
@@ -14824,11 +14828,7 @@
         </is>
       </c>
       <c r="U208" t="inlineStr"/>
-      <c r="V208" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -15241,7 +15241,11 @@
           <t>Manager,  Marketing Science &amp; Analytics</t>
         </is>
       </c>
-      <c r="C215" t="inlineStr"/>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D215" t="inlineStr"/>
       <c r="E215" t="inlineStr">
         <is>
@@ -15294,11 +15298,7 @@
         </is>
       </c>
       <c r="U215" t="inlineStr"/>
-      <c r="V215" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V215" t="inlineStr"/>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -15579,7 +15579,11 @@
           <t>Marketing Data Science Analytics Lead</t>
         </is>
       </c>
-      <c r="C220" t="inlineStr"/>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D220" t="inlineStr"/>
       <c r="E220" t="inlineStr">
         <is>
@@ -15632,11 +15636,7 @@
         </is>
       </c>
       <c r="U220" t="inlineStr"/>
-      <c r="V220" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -15785,7 +15785,11 @@
           <t>Senior Data Scientist, Marketing Science</t>
         </is>
       </c>
-      <c r="C223" t="inlineStr"/>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D223" t="inlineStr"/>
       <c r="E223" t="inlineStr">
         <is>
@@ -15838,11 +15842,7 @@
         </is>
       </c>
       <c r="U223" t="inlineStr"/>
-      <c r="V223" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -15855,7 +15855,11 @@
           <t>Marketing Science Lead - Austin, TX</t>
         </is>
       </c>
-      <c r="C224" t="inlineStr"/>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D224" t="inlineStr"/>
       <c r="E224" t="inlineStr">
         <is>
@@ -15908,11 +15912,7 @@
         </is>
       </c>
       <c r="U224" t="inlineStr"/>
-      <c r="V224" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V224" t="inlineStr"/>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -16457,7 +16457,11 @@
           <t>Data Science Manager, Marketing Analytics</t>
         </is>
       </c>
-      <c r="C233" t="inlineStr"/>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D233" t="inlineStr"/>
       <c r="E233" t="inlineStr">
         <is>
@@ -16510,11 +16514,7 @@
         </is>
       </c>
       <c r="U233" t="inlineStr"/>
-      <c r="V233" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V233" t="inlineStr"/>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -16989,7 +16989,11 @@
           <t>Vice President-Marketing Strategy Lead, Shopping Innovation &amp; AI Strategy</t>
         </is>
       </c>
-      <c r="C241" t="inlineStr"/>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>02 Field CTO / Head AI Solutions at Vendor</t>
+        </is>
+      </c>
       <c r="D241" t="inlineStr"/>
       <c r="E241" t="inlineStr">
         <is>
@@ -17042,11 +17046,7 @@
         </is>
       </c>
       <c r="U241" t="inlineStr"/>
-      <c r="V241" t="inlineStr">
-        <is>
-          <t>02 Field CTO / Head AI Solutions at Vendor (high)</t>
-        </is>
-      </c>
+      <c r="V241" t="inlineStr"/>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
@@ -17129,7 +17129,11 @@
           <t>Marketing Analytics &amp; Data Science Senior Lead</t>
         </is>
       </c>
-      <c r="C243" t="inlineStr"/>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D243" t="inlineStr"/>
       <c r="E243" t="inlineStr">
         <is>
@@ -17182,11 +17186,7 @@
         </is>
       </c>
       <c r="U243" t="inlineStr"/>
-      <c r="V243" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V243" t="inlineStr"/>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
@@ -17463,7 +17463,11 @@
           <t>Sr Director, Technology- Media/Customer Analytics, Measurement and Data Science</t>
         </is>
       </c>
-      <c r="C248" t="inlineStr"/>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D248" t="inlineStr"/>
       <c r="E248" t="inlineStr">
         <is>
@@ -17516,11 +17520,7 @@
         </is>
       </c>
       <c r="U248" t="inlineStr"/>
-      <c r="V248" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V248" t="inlineStr"/>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
@@ -17603,7 +17603,11 @@
           <t>Growth Science &amp; Marketing Capabilities Lead</t>
         </is>
       </c>
-      <c r="C250" t="inlineStr"/>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D250" t="inlineStr"/>
       <c r="E250" t="inlineStr">
         <is>
@@ -17656,11 +17660,7 @@
         </is>
       </c>
       <c r="U250" t="inlineStr"/>
-      <c r="V250" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V250" t="inlineStr"/>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
@@ -18201,7 +18201,11 @@
           <t>(Senior) Software Engineer, Experimentation Platform - CoreAI</t>
         </is>
       </c>
-      <c r="C259" t="inlineStr"/>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D259" t="inlineStr"/>
       <c r="E259" t="inlineStr">
         <is>
@@ -18254,11 +18258,7 @@
         </is>
       </c>
       <c r="U259" t="inlineStr"/>
-      <c r="V259" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V259" t="inlineStr"/>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
@@ -18403,7 +18403,11 @@
           <t>Vice President, Marketing</t>
         </is>
       </c>
-      <c r="C262" t="inlineStr"/>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>05 Practice Lead at Consultancy</t>
+        </is>
+      </c>
       <c r="D262" t="inlineStr"/>
       <c r="E262" t="inlineStr">
         <is>
@@ -18456,11 +18460,7 @@
         </is>
       </c>
       <c r="U262" t="inlineStr"/>
-      <c r="V262" t="inlineStr">
-        <is>
-          <t>05 Practice Lead at Consultancy (high)</t>
-        </is>
-      </c>
+      <c r="V262" t="inlineStr"/>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
@@ -18543,7 +18543,11 @@
           <t>Marketing Science &amp; Engineering Senior Manager</t>
         </is>
       </c>
-      <c r="C264" t="inlineStr"/>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D264" t="inlineStr"/>
       <c r="E264" t="inlineStr">
         <is>
@@ -18596,11 +18600,7 @@
         </is>
       </c>
       <c r="U264" t="inlineStr"/>
-      <c r="V264" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V264" t="inlineStr"/>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
@@ -18613,7 +18613,11 @@
           <t>Data Engineer (L6) - Ads (Signals and Measurement)</t>
         </is>
       </c>
-      <c r="C265" t="inlineStr"/>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D265" t="inlineStr"/>
       <c r="E265" t="inlineStr">
         <is>
@@ -18666,11 +18670,7 @@
         </is>
       </c>
       <c r="U265" t="inlineStr"/>
-      <c r="V265" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V265" t="inlineStr"/>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
@@ -19215,7 +19215,11 @@
           <t>Senior Strategist, Marketing Science</t>
         </is>
       </c>
-      <c r="C274" t="inlineStr"/>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D274" t="inlineStr"/>
       <c r="E274" t="inlineStr">
         <is>
@@ -19268,11 +19272,7 @@
         </is>
       </c>
       <c r="U274" t="inlineStr"/>
-      <c r="V274" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V274" t="inlineStr"/>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
@@ -19487,7 +19487,11 @@
           <t>Measurement Strategy Manager</t>
         </is>
       </c>
-      <c r="C278" t="inlineStr"/>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D278" t="inlineStr"/>
       <c r="E278" t="inlineStr">
         <is>
@@ -19540,11 +19544,7 @@
         </is>
       </c>
       <c r="U278" t="inlineStr"/>
-      <c r="V278" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V278" t="inlineStr"/>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
@@ -19623,7 +19623,11 @@
           <t>Director, Insights and Measurement</t>
         </is>
       </c>
-      <c r="C280" t="inlineStr"/>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D280" t="inlineStr"/>
       <c r="E280" t="inlineStr">
         <is>
@@ -19676,11 +19680,7 @@
         </is>
       </c>
       <c r="U280" t="inlineStr"/>
-      <c r="V280" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V280" t="inlineStr"/>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
@@ -20159,7 +20159,11 @@
           <t>Staff / VP, Data Science - Marketing &amp; Sales Focus</t>
         </is>
       </c>
-      <c r="C288" t="inlineStr"/>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D288" t="inlineStr"/>
       <c r="E288" t="inlineStr">
         <is>
@@ -20212,11 +20216,7 @@
         </is>
       </c>
       <c r="U288" t="inlineStr"/>
-      <c r="V288" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V288" t="inlineStr"/>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
@@ -20497,7 +20497,11 @@
           <t>(USA) Principal, Software Engineer-Experimentation Platform</t>
         </is>
       </c>
-      <c r="C293" t="inlineStr"/>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D293" t="inlineStr"/>
       <c r="E293" t="inlineStr">
         <is>
@@ -20550,11 +20554,7 @@
         </is>
       </c>
       <c r="U293" t="inlineStr"/>
-      <c r="V293" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V293" t="inlineStr"/>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
@@ -20567,7 +20567,11 @@
           <t>AEO Measurement &amp; Insights Lead</t>
         </is>
       </c>
-      <c r="C294" t="inlineStr"/>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D294" t="inlineStr"/>
       <c r="E294" t="inlineStr">
         <is>
@@ -20620,11 +20624,7 @@
         </is>
       </c>
       <c r="U294" t="inlineStr"/>
-      <c r="V294" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V294" t="inlineStr"/>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
@@ -20975,7 +20975,11 @@
           <t>Sr.Director, Data Science &amp; Data Engineering</t>
         </is>
       </c>
-      <c r="C300" t="inlineStr"/>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D300" t="inlineStr"/>
       <c r="E300" t="inlineStr">
         <is>
@@ -21028,11 +21032,7 @@
         </is>
       </c>
       <c r="U300" t="inlineStr"/>
-      <c r="V300" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V300" t="inlineStr"/>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
@@ -21181,7 +21181,11 @@
           <t>Staff Applied AI/ML Scientist</t>
         </is>
       </c>
-      <c r="C303" t="inlineStr"/>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D303" t="inlineStr"/>
       <c r="E303" t="inlineStr">
         <is>
@@ -21234,11 +21238,7 @@
         </is>
       </c>
       <c r="U303" t="inlineStr"/>
-      <c r="V303" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V303" t="inlineStr"/>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
@@ -21317,7 +21317,11 @@
           <t>Data Science Manager II, Digital Partnerships</t>
         </is>
       </c>
-      <c r="C305" t="inlineStr"/>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D305" t="inlineStr"/>
       <c r="E305" t="inlineStr">
         <is>
@@ -21370,11 +21374,7 @@
         </is>
       </c>
       <c r="U305" t="inlineStr"/>
-      <c r="V305" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21791,7 +21791,11 @@
           <t>Applied AI Architect, Digital Natives</t>
         </is>
       </c>
-      <c r="C312" t="inlineStr"/>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D312" t="inlineStr"/>
       <c r="E312" t="inlineStr">
         <is>
@@ -21844,11 +21848,7 @@
         </is>
       </c>
       <c r="U312" t="inlineStr"/>
-      <c r="V312" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V312" t="inlineStr"/>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
@@ -21931,7 +21931,11 @@
           <t>Applied AI Architect - EDU</t>
         </is>
       </c>
-      <c r="C314" t="inlineStr"/>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D314" t="inlineStr"/>
       <c r="E314" t="inlineStr">
         <is>
@@ -21984,11 +21988,7 @@
         </is>
       </c>
       <c r="U314" t="inlineStr"/>
-      <c r="V314" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V314" t="inlineStr"/>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
@@ -22067,7 +22067,11 @@
           <t>Applied AI Architect, Enterprise</t>
         </is>
       </c>
-      <c r="C316" t="inlineStr"/>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D316" t="inlineStr"/>
       <c r="E316" t="inlineStr">
         <is>
@@ -22120,11 +22124,7 @@
         </is>
       </c>
       <c r="U316" t="inlineStr"/>
-      <c r="V316" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V316" t="inlineStr"/>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
@@ -22137,7 +22137,11 @@
           <t>Applied AI Architect, Government</t>
         </is>
       </c>
-      <c r="C317" t="inlineStr"/>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D317" t="inlineStr"/>
       <c r="E317" t="inlineStr">
         <is>
@@ -22190,11 +22194,7 @@
         </is>
       </c>
       <c r="U317" t="inlineStr"/>
-      <c r="V317" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V317" t="inlineStr"/>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
@@ -22207,7 +22207,11 @@
           <t>Applied AI Architect, Large Enterprise</t>
         </is>
       </c>
-      <c r="C318" t="inlineStr"/>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D318" t="inlineStr"/>
       <c r="E318" t="inlineStr">
         <is>
@@ -22260,11 +22264,7 @@
         </is>
       </c>
       <c r="U318" t="inlineStr"/>
-      <c r="V318" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V318" t="inlineStr"/>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
@@ -22277,7 +22277,11 @@
           <t>Applied AI Architect - Tokyo</t>
         </is>
       </c>
-      <c r="C319" t="inlineStr"/>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D319" t="inlineStr"/>
       <c r="E319" t="inlineStr">
         <is>
@@ -22330,11 +22334,7 @@
         </is>
       </c>
       <c r="U319" t="inlineStr"/>
-      <c r="V319" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V319" t="inlineStr"/>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
@@ -22347,7 +22347,11 @@
           <t>Applied AI Engineer</t>
         </is>
       </c>
-      <c r="C320" t="inlineStr"/>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D320" t="inlineStr"/>
       <c r="E320" t="inlineStr">
         <is>
@@ -22400,11 +22404,7 @@
         </is>
       </c>
       <c r="U320" t="inlineStr"/>
-      <c r="V320" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V320" t="inlineStr"/>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
@@ -22417,7 +22417,11 @@
           <t>Applied AI Engineer, Agent Enablement</t>
         </is>
       </c>
-      <c r="C321" t="inlineStr"/>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D321" t="inlineStr"/>
       <c r="E321" t="inlineStr">
         <is>
@@ -22470,11 +22474,7 @@
         </is>
       </c>
       <c r="U321" t="inlineStr"/>
-      <c r="V321" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V321" t="inlineStr"/>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
@@ -22487,7 +22487,11 @@
           <t>Applied AI Engineer, Codex</t>
         </is>
       </c>
-      <c r="C322" t="inlineStr"/>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D322" t="inlineStr"/>
       <c r="E322" t="inlineStr">
         <is>
@@ -22540,11 +22544,7 @@
         </is>
       </c>
       <c r="U322" t="inlineStr"/>
-      <c r="V322" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V322" t="inlineStr"/>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
@@ -22557,7 +22557,11 @@
           <t>Applied AI Engineer, Codex Core Agent</t>
         </is>
       </c>
-      <c r="C323" t="inlineStr"/>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D323" t="inlineStr"/>
       <c r="E323" t="inlineStr">
         <is>
@@ -22610,11 +22614,7 @@
         </is>
       </c>
       <c r="U323" t="inlineStr"/>
-      <c r="V323" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V323" t="inlineStr"/>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
@@ -22627,7 +22627,11 @@
           <t>Applied AI Engineer, Codex | Tokyo</t>
         </is>
       </c>
-      <c r="C324" t="inlineStr"/>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D324" t="inlineStr"/>
       <c r="E324" t="inlineStr">
         <is>
@@ -22680,11 +22684,7 @@
         </is>
       </c>
       <c r="U324" t="inlineStr"/>
-      <c r="V324" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V324" t="inlineStr"/>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
@@ -22697,7 +22697,11 @@
           <t>Applied AI Engineer, Cyber</t>
         </is>
       </c>
-      <c r="C325" t="inlineStr"/>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D325" t="inlineStr"/>
       <c r="E325" t="inlineStr">
         <is>
@@ -22750,11 +22754,7 @@
         </is>
       </c>
       <c r="U325" t="inlineStr"/>
-      <c r="V325" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V325" t="inlineStr"/>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
@@ -22767,7 +22767,11 @@
           <t>Applied AI Engineer, Cyber, Government</t>
         </is>
       </c>
-      <c r="C326" t="inlineStr"/>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D326" t="inlineStr"/>
       <c r="E326" t="inlineStr">
         <is>
@@ -22820,11 +22824,7 @@
         </is>
       </c>
       <c r="U326" t="inlineStr"/>
-      <c r="V326" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V326" t="inlineStr"/>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
@@ -22837,7 +22837,11 @@
           <t>Applied AI Engineer, Cyber | Tokyo</t>
         </is>
       </c>
-      <c r="C327" t="inlineStr"/>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D327" t="inlineStr"/>
       <c r="E327" t="inlineStr">
         <is>
@@ -22890,11 +22894,7 @@
         </is>
       </c>
       <c r="U327" t="inlineStr"/>
-      <c r="V327" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V327" t="inlineStr"/>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
@@ -22977,7 +22977,11 @@
           <t>Applied AI Engineer, Enterprise</t>
         </is>
       </c>
-      <c r="C329" t="inlineStr"/>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D329" t="inlineStr"/>
       <c r="E329" t="inlineStr">
         <is>
@@ -23030,11 +23034,7 @@
         </is>
       </c>
       <c r="U329" t="inlineStr"/>
-      <c r="V329" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V329" t="inlineStr"/>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
@@ -23047,7 +23047,11 @@
           <t>Applied AI Engineer, Government</t>
         </is>
       </c>
-      <c r="C330" t="inlineStr"/>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D330" t="inlineStr"/>
       <c r="E330" t="inlineStr">
         <is>
@@ -23100,11 +23104,7 @@
         </is>
       </c>
       <c r="U330" t="inlineStr"/>
-      <c r="V330" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V330" t="inlineStr"/>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
@@ -23117,7 +23117,11 @@
           <t>Applied AI Engineer, Plugins</t>
         </is>
       </c>
-      <c r="C331" t="inlineStr"/>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D331" t="inlineStr"/>
       <c r="E331" t="inlineStr">
         <is>
@@ -23170,11 +23174,7 @@
         </is>
       </c>
       <c r="U331" t="inlineStr"/>
-      <c r="V331" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V331" t="inlineStr"/>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
@@ -23187,7 +23187,11 @@
           <t>Applied AI Engineer, Startups</t>
         </is>
       </c>
-      <c r="C332" t="inlineStr"/>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D332" t="inlineStr"/>
       <c r="E332" t="inlineStr">
         <is>
@@ -23240,11 +23244,7 @@
         </is>
       </c>
       <c r="U332" t="inlineStr"/>
-      <c r="V332" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V332" t="inlineStr"/>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
@@ -23257,7 +23257,11 @@
           <t>Applied AI Engineer - Tokyo</t>
         </is>
       </c>
-      <c r="C333" t="inlineStr"/>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D333" t="inlineStr"/>
       <c r="E333" t="inlineStr">
         <is>
@@ -23310,11 +23314,7 @@
         </is>
       </c>
       <c r="U333" t="inlineStr"/>
-      <c r="V333" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V333" t="inlineStr"/>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
@@ -23327,7 +23327,11 @@
           <t>Applied AI Software Engineer, GTM Growth Engineering</t>
         </is>
       </c>
-      <c r="C334" t="inlineStr"/>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D334" t="inlineStr"/>
       <c r="E334" t="inlineStr">
         <is>
@@ -23380,11 +23384,7 @@
         </is>
       </c>
       <c r="U334" t="inlineStr"/>
-      <c r="V334" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V334" t="inlineStr"/>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
@@ -23397,7 +23397,11 @@
           <t>Applied Data Science &amp; Insights Leader - GTM Intelligence Solutions and Technical Success</t>
         </is>
       </c>
-      <c r="C335" t="inlineStr"/>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D335" t="inlineStr"/>
       <c r="E335" t="inlineStr">
         <is>
@@ -23450,11 +23454,7 @@
         </is>
       </c>
       <c r="U335" t="inlineStr"/>
-      <c r="V335" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V335" t="inlineStr"/>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
@@ -24193,7 +24193,11 @@
           <t>Forward Deployed Engineer (FDE), Healthcare - NYC</t>
         </is>
       </c>
-      <c r="C347" t="inlineStr"/>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D347" t="inlineStr"/>
       <c r="E347" t="inlineStr">
         <is>
@@ -24246,11 +24250,7 @@
         </is>
       </c>
       <c r="U347" t="inlineStr"/>
-      <c r="V347" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V347" t="inlineStr"/>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
@@ -24263,7 +24263,11 @@
           <t>Forward Deployed Engineer (FDE), Healthcare - Seattle</t>
         </is>
       </c>
-      <c r="C348" t="inlineStr"/>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D348" t="inlineStr"/>
       <c r="E348" t="inlineStr">
         <is>
@@ -24316,11 +24320,7 @@
         </is>
       </c>
       <c r="U348" t="inlineStr"/>
-      <c r="V348" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V348" t="inlineStr"/>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
@@ -24333,7 +24333,11 @@
           <t>Forward Deployed Engineer (FDE), Healthcare - SF</t>
         </is>
       </c>
-      <c r="C349" t="inlineStr"/>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D349" t="inlineStr"/>
       <c r="E349" t="inlineStr">
         <is>
@@ -24386,11 +24390,7 @@
         </is>
       </c>
       <c r="U349" t="inlineStr"/>
-      <c r="V349" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V349" t="inlineStr"/>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
@@ -24403,7 +24403,11 @@
           <t>Forward Deployed Engineer (FDE), Legal-NYC</t>
         </is>
       </c>
-      <c r="C350" t="inlineStr"/>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D350" t="inlineStr"/>
       <c r="E350" t="inlineStr">
         <is>
@@ -24456,11 +24460,7 @@
         </is>
       </c>
       <c r="U350" t="inlineStr"/>
-      <c r="V350" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V350" t="inlineStr"/>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
@@ -24473,7 +24473,11 @@
           <t>Forward Deployed Engineer (FDE), Legal-SF</t>
         </is>
       </c>
-      <c r="C351" t="inlineStr"/>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D351" t="inlineStr"/>
       <c r="E351" t="inlineStr">
         <is>
@@ -24526,11 +24530,7 @@
         </is>
       </c>
       <c r="U351" t="inlineStr"/>
-      <c r="V351" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V351" t="inlineStr"/>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
@@ -24613,7 +24613,11 @@
           <t>Forward Deployed Engineer (FDE) - Seattle</t>
         </is>
       </c>
-      <c r="C353" t="inlineStr"/>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D353" t="inlineStr"/>
       <c r="E353" t="inlineStr">
         <is>
@@ -24666,11 +24670,7 @@
         </is>
       </c>
       <c r="U353" t="inlineStr"/>
-      <c r="V353" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V353" t="inlineStr"/>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
@@ -24683,7 +24683,11 @@
           <t>Forward Deployed Engineer (FDE) - SF</t>
         </is>
       </c>
-      <c r="C354" t="inlineStr"/>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D354" t="inlineStr"/>
       <c r="E354" t="inlineStr">
         <is>
@@ -24736,11 +24740,7 @@
         </is>
       </c>
       <c r="U354" t="inlineStr"/>
-      <c r="V354" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V354" t="inlineStr"/>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
@@ -24823,7 +24823,11 @@
           <t>Forward Deployed Engineer - London (Spanish-speaking)</t>
         </is>
       </c>
-      <c r="C356" t="inlineStr"/>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D356" t="inlineStr"/>
       <c r="E356" t="inlineStr">
         <is>
@@ -24876,11 +24880,7 @@
         </is>
       </c>
       <c r="U356" t="inlineStr"/>
-      <c r="V356" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V356" t="inlineStr"/>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
@@ -24893,7 +24893,11 @@
           <t>Forward Deployed Engineer - Madrid (Spanish-speaking)</t>
         </is>
       </c>
-      <c r="C357" t="inlineStr"/>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D357" t="inlineStr"/>
       <c r="E357" t="inlineStr">
         <is>
@@ -24946,11 +24950,7 @@
         </is>
       </c>
       <c r="U357" t="inlineStr"/>
-      <c r="V357" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V357" t="inlineStr"/>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -24963,7 +24963,11 @@
           <t>Forward Deployed Engineer - Seoul</t>
         </is>
       </c>
-      <c r="C358" t="inlineStr"/>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D358" t="inlineStr"/>
       <c r="E358" t="inlineStr">
         <is>
@@ -25016,11 +25020,7 @@
         </is>
       </c>
       <c r="U358" t="inlineStr"/>
-      <c r="V358" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V358" t="inlineStr"/>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
@@ -25033,7 +25033,11 @@
           <t>Forward Deployed Engineer - Singapore</t>
         </is>
       </c>
-      <c r="C359" t="inlineStr"/>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D359" t="inlineStr"/>
       <c r="E359" t="inlineStr">
         <is>
@@ -25086,11 +25090,7 @@
         </is>
       </c>
       <c r="U359" t="inlineStr"/>
-      <c r="V359" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V359" t="inlineStr"/>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
@@ -25103,7 +25103,11 @@
           <t>Forward Deployed Engineer - Sydney</t>
         </is>
       </c>
-      <c r="C360" t="inlineStr"/>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D360" t="inlineStr"/>
       <c r="E360" t="inlineStr">
         <is>
@@ -25156,11 +25160,7 @@
         </is>
       </c>
       <c r="U360" t="inlineStr"/>
-      <c r="V360" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V360" t="inlineStr"/>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
@@ -25173,7 +25173,11 @@
           <t>Forward Deployed Engineer - Tokyo</t>
         </is>
       </c>
-      <c r="C361" t="inlineStr"/>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D361" t="inlineStr"/>
       <c r="E361" t="inlineStr">
         <is>
@@ -25226,11 +25230,7 @@
         </is>
       </c>
       <c r="U361" t="inlineStr"/>
-      <c r="V361" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V361" t="inlineStr"/>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
@@ -26075,7 +26075,11 @@
           <t>Manager, Forward Deployed Engineer - Tokyo</t>
         </is>
       </c>
-      <c r="C374" t="inlineStr"/>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D374" t="inlineStr"/>
       <c r="E374" t="inlineStr">
         <is>
@@ -26128,11 +26132,7 @@
         </is>
       </c>
       <c r="U374" t="inlineStr"/>
-      <c r="V374" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V374" t="inlineStr"/>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
@@ -26145,7 +26145,11 @@
           <t>Partner Applied AI Engineer</t>
         </is>
       </c>
-      <c r="C375" t="inlineStr"/>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D375" t="inlineStr"/>
       <c r="E375" t="inlineStr">
         <is>
@@ -26198,11 +26202,7 @@
         </is>
       </c>
       <c r="U375" t="inlineStr"/>
-      <c r="V375" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V375" t="inlineStr"/>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
@@ -26281,7 +26281,11 @@
           <t>Physical Design Engineer, Forward Deployed Engineering</t>
         </is>
       </c>
-      <c r="C377" t="inlineStr"/>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D377" t="inlineStr"/>
       <c r="E377" t="inlineStr">
         <is>
@@ -26334,11 +26338,7 @@
         </is>
       </c>
       <c r="U377" t="inlineStr"/>
-      <c r="V377" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V377" t="inlineStr"/>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
@@ -26351,7 +26351,11 @@
           <t>Software Engineer, Infrastructure - Analytics Platform</t>
         </is>
       </c>
-      <c r="C378" t="inlineStr"/>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D378" t="inlineStr"/>
       <c r="E378" t="inlineStr">
         <is>
@@ -26404,11 +26408,7 @@
         </is>
       </c>
       <c r="U378" t="inlineStr"/>
-      <c r="V378" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V378" t="inlineStr"/>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
@@ -26421,7 +26421,11 @@
           <t>Staff Applied Scientist - Agentic Interfaces</t>
         </is>
       </c>
-      <c r="C379" t="inlineStr"/>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D379" t="inlineStr"/>
       <c r="E379" t="inlineStr">
         <is>
@@ -26474,11 +26478,7 @@
         </is>
       </c>
       <c r="U379" t="inlineStr"/>
-      <c r="V379" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V379" t="inlineStr"/>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
@@ -29799,7 +29799,11 @@
           <t>Manager II, Machine Learning – Conversion Visibility</t>
         </is>
       </c>
-      <c r="C430" t="inlineStr"/>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D430" t="inlineStr"/>
       <c r="E430" t="inlineStr">
         <is>
@@ -29852,11 +29856,7 @@
         </is>
       </c>
       <c r="U430" t="inlineStr"/>
-      <c r="V430" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V430" t="inlineStr"/>
     </row>
     <row r="431">
       <c r="A431" t="inlineStr">
@@ -30001,7 +30001,11 @@
           <t>Sr. Manager, Machine Learning Engineering-Applied Research</t>
         </is>
       </c>
-      <c r="C433" t="inlineStr"/>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D433" t="inlineStr"/>
       <c r="E433" t="inlineStr">
         <is>
@@ -30054,11 +30058,7 @@
         </is>
       </c>
       <c r="U433" t="inlineStr"/>
-      <c r="V433" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V433" t="inlineStr"/>
     </row>
     <row r="434">
       <c r="A434" t="inlineStr">
@@ -30137,7 +30137,11 @@
           <t>Ads Conversion Modeling, Machine Learning Engineering Manager</t>
         </is>
       </c>
-      <c r="C435" t="inlineStr"/>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D435" t="inlineStr"/>
       <c r="E435" t="inlineStr">
         <is>
@@ -30190,11 +30194,7 @@
         </is>
       </c>
       <c r="U435" t="inlineStr"/>
-      <c r="V435" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V435" t="inlineStr"/>
     </row>
     <row r="436">
       <c r="A436" t="inlineStr">
@@ -30207,7 +30207,11 @@
           <t>Machine Learning Engineering Manager - Ads Engagement Modeling</t>
         </is>
       </c>
-      <c r="C436" t="inlineStr"/>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D436" t="inlineStr"/>
       <c r="E436" t="inlineStr">
         <is>
@@ -30260,11 +30264,7 @@
         </is>
       </c>
       <c r="U436" t="inlineStr"/>
-      <c r="V436" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V436" t="inlineStr"/>
     </row>
     <row r="437">
       <c r="A437" t="inlineStr">
@@ -30277,7 +30277,11 @@
           <t>Machine Learning Manager, Feed Ecosystems</t>
         </is>
       </c>
-      <c r="C437" t="inlineStr"/>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D437" t="inlineStr"/>
       <c r="E437" t="inlineStr">
         <is>
@@ -30330,11 +30334,7 @@
         </is>
       </c>
       <c r="U437" t="inlineStr"/>
-      <c r="V437" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V437" t="inlineStr"/>
     </row>
     <row r="438">
       <c r="A438" t="inlineStr">
@@ -30347,7 +30347,11 @@
           <t>Machine Learning Manager, Feed Relevance (Retrieval)</t>
         </is>
       </c>
-      <c r="C438" t="inlineStr"/>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D438" t="inlineStr"/>
       <c r="E438" t="inlineStr">
         <is>
@@ -30400,11 +30404,7 @@
         </is>
       </c>
       <c r="U438" t="inlineStr"/>
-      <c r="V438" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V438" t="inlineStr"/>
     </row>
     <row r="439">
       <c r="A439" t="inlineStr">
@@ -30549,7 +30549,11 @@
           <t>Senior Machine Learning Infrastructure Engineer, Embedding Platform</t>
         </is>
       </c>
-      <c r="C441" t="inlineStr"/>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D441" t="inlineStr"/>
       <c r="E441" t="inlineStr">
         <is>
@@ -30602,11 +30606,7 @@
         </is>
       </c>
       <c r="U441" t="inlineStr"/>
-      <c r="V441" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V441" t="inlineStr"/>
     </row>
     <row r="442">
       <c r="A442" t="inlineStr">
@@ -30619,7 +30619,11 @@
           <t>Senior Machine Learning Manager, Video Ranking</t>
         </is>
       </c>
-      <c r="C442" t="inlineStr"/>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>01 Meas/Mkt Science Lead AI Ads or Platform</t>
+        </is>
+      </c>
       <c r="D442" t="inlineStr"/>
       <c r="E442" t="inlineStr">
         <is>
@@ -30672,11 +30676,7 @@
         </is>
       </c>
       <c r="U442" t="inlineStr"/>
-      <c r="V442" t="inlineStr">
-        <is>
-          <t>01 Meas/Mkt Science Lead AI Ads or Platform (high)</t>
-        </is>
-      </c>
+      <c r="V442" t="inlineStr"/>
     </row>
     <row r="443">
       <c r="A443" t="inlineStr">
@@ -30689,7 +30689,11 @@
           <t>Senior Machine Learning Systems Engineer</t>
         </is>
       </c>
-      <c r="C443" t="inlineStr"/>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D443" t="inlineStr"/>
       <c r="E443" t="inlineStr">
         <is>
@@ -30742,11 +30746,7 @@
         </is>
       </c>
       <c r="U443" t="inlineStr"/>
-      <c r="V443" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -30759,7 +30759,11 @@
           <t>Senior Machine Learning Systems Engineer, Ads ML Experience Platform</t>
         </is>
       </c>
-      <c r="C444" t="inlineStr"/>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D444" t="inlineStr"/>
       <c r="E444" t="inlineStr">
         <is>
@@ -30812,11 +30816,7 @@
         </is>
       </c>
       <c r="U444" t="inlineStr"/>
-      <c r="V444" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -30895,7 +30895,11 @@
           <t>Senior Staff Machine Learning Systems Engineer, Ads ML Platform</t>
         </is>
       </c>
-      <c r="C446" t="inlineStr"/>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D446" t="inlineStr"/>
       <c r="E446" t="inlineStr">
         <is>
@@ -30948,11 +30952,7 @@
         </is>
       </c>
       <c r="U446" t="inlineStr"/>
-      <c r="V446" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V446" t="inlineStr"/>
     </row>
     <row r="447">
       <c r="A447" t="inlineStr">
@@ -30965,7 +30965,11 @@
           <t>Senior Staff ML Engineer, Search &amp; Recommendation</t>
         </is>
       </c>
-      <c r="C447" t="inlineStr"/>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D447" t="inlineStr"/>
       <c r="E447" t="inlineStr">
         <is>
@@ -31018,11 +31022,7 @@
         </is>
       </c>
       <c r="U447" t="inlineStr"/>
-      <c r="V447" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V447" t="inlineStr"/>
     </row>
     <row r="448">
       <c r="A448" t="inlineStr">
@@ -31035,7 +31035,11 @@
           <t>Staff Machine Learning Infrastructure Engineer, Embedding Platform</t>
         </is>
       </c>
-      <c r="C448" t="inlineStr"/>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D448" t="inlineStr"/>
       <c r="E448" t="inlineStr">
         <is>
@@ -31088,11 +31092,7 @@
         </is>
       </c>
       <c r="U448" t="inlineStr"/>
-      <c r="V448" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V448" t="inlineStr"/>
     </row>
     <row r="449">
       <c r="A449" t="inlineStr">
@@ -31105,7 +31105,11 @@
           <t>Staff Machine Learning Systems Engineer</t>
         </is>
       </c>
-      <c r="C449" t="inlineStr"/>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D449" t="inlineStr"/>
       <c r="E449" t="inlineStr">
         <is>
@@ -31158,11 +31162,7 @@
         </is>
       </c>
       <c r="U449" t="inlineStr"/>
-      <c r="V449" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V449" t="inlineStr"/>
     </row>
     <row r="450">
       <c r="A450" t="inlineStr">
@@ -31241,7 +31241,11 @@
           <t>Machine Learning Engineer, Monetization Engineering</t>
         </is>
       </c>
-      <c r="C451" t="inlineStr"/>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D451" t="inlineStr"/>
       <c r="E451" t="inlineStr">
         <is>
@@ -31294,11 +31298,7 @@
         </is>
       </c>
       <c r="U451" t="inlineStr"/>
-      <c r="V451" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V451" t="inlineStr"/>
     </row>
     <row r="452">
       <c r="A452" t="inlineStr">
@@ -31311,7 +31311,11 @@
           <t>Principal Machine Learning Engineer, Ads Delivery</t>
         </is>
       </c>
-      <c r="C452" t="inlineStr"/>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D452" t="inlineStr"/>
       <c r="E452" t="inlineStr">
         <is>
@@ -31364,11 +31368,7 @@
         </is>
       </c>
       <c r="U452" t="inlineStr"/>
-      <c r="V452" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V452" t="inlineStr"/>
     </row>
     <row r="453">
       <c r="A453" t="inlineStr">
@@ -31381,7 +31381,11 @@
           <t>Sr. Machine Learning Engineer, Applied Science</t>
         </is>
       </c>
-      <c r="C453" t="inlineStr"/>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D453" t="inlineStr"/>
       <c r="E453" t="inlineStr">
         <is>
@@ -31434,11 +31438,7 @@
         </is>
       </c>
       <c r="U453" t="inlineStr"/>
-      <c r="V453" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V453" t="inlineStr"/>
     </row>
     <row r="454">
       <c r="A454" t="inlineStr">
@@ -31451,7 +31451,11 @@
           <t>Sr. Machine Learning Engineer, Core Engineering</t>
         </is>
       </c>
-      <c r="C454" t="inlineStr"/>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D454" t="inlineStr"/>
       <c r="E454" t="inlineStr">
         <is>
@@ -31504,11 +31508,7 @@
         </is>
       </c>
       <c r="U454" t="inlineStr"/>
-      <c r="V454" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V454" t="inlineStr"/>
     </row>
     <row r="455">
       <c r="A455" t="inlineStr">
@@ -31521,7 +31521,11 @@
           <t>Sr. Machine Learning Engineer, Monetization Engineering</t>
         </is>
       </c>
-      <c r="C455" t="inlineStr"/>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D455" t="inlineStr"/>
       <c r="E455" t="inlineStr">
         <is>
@@ -31574,11 +31578,7 @@
         </is>
       </c>
       <c r="U455" t="inlineStr"/>
-      <c r="V455" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V455" t="inlineStr"/>
     </row>
     <row r="456">
       <c r="A456" t="inlineStr">
@@ -31591,7 +31591,11 @@
           <t>Sr. Staff Machine Learning Engineer, Content Quality</t>
         </is>
       </c>
-      <c r="C456" t="inlineStr"/>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D456" t="inlineStr"/>
       <c r="E456" t="inlineStr">
         <is>
@@ -31644,11 +31648,7 @@
         </is>
       </c>
       <c r="U456" t="inlineStr"/>
-      <c r="V456" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V456" t="inlineStr"/>
     </row>
     <row r="457">
       <c r="A457" t="inlineStr">
@@ -31661,7 +31661,11 @@
           <t>Sr. Staff Machine Learning Engineer, Monetization Engineering</t>
         </is>
       </c>
-      <c r="C457" t="inlineStr"/>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D457" t="inlineStr"/>
       <c r="E457" t="inlineStr">
         <is>
@@ -31714,11 +31718,7 @@
         </is>
       </c>
       <c r="U457" t="inlineStr"/>
-      <c r="V457" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V457" t="inlineStr"/>
     </row>
     <row r="458">
       <c r="A458" t="inlineStr">
@@ -31731,7 +31731,11 @@
           <t>Staff Machine Learning Engineer, Ads Conversion Core Modeling</t>
         </is>
       </c>
-      <c r="C458" t="inlineStr"/>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D458" t="inlineStr"/>
       <c r="E458" t="inlineStr">
         <is>
@@ -31784,11 +31788,7 @@
         </is>
       </c>
       <c r="U458" t="inlineStr"/>
-      <c r="V458" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V458" t="inlineStr"/>
     </row>
     <row r="459">
       <c r="A459" t="inlineStr">
@@ -31801,7 +31801,11 @@
           <t>Staff Machine Learning Engineer, Visual AI</t>
         </is>
       </c>
-      <c r="C459" t="inlineStr"/>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D459" t="inlineStr"/>
       <c r="E459" t="inlineStr">
         <is>
@@ -31854,11 +31858,7 @@
         </is>
       </c>
       <c r="U459" t="inlineStr"/>
-      <c r="V459" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V459" t="inlineStr"/>
     </row>
     <row r="460">
       <c r="A460" t="inlineStr">
@@ -31937,7 +31937,11 @@
           <t>Senior Machine Learning Engineer</t>
         </is>
       </c>
-      <c r="C461" t="inlineStr"/>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D461" t="inlineStr"/>
       <c r="E461" t="inlineStr">
         <is>
@@ -31990,11 +31994,7 @@
         </is>
       </c>
       <c r="U461" t="inlineStr"/>
-      <c r="V461" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V461" t="inlineStr"/>
     </row>
     <row r="462">
       <c r="A462" t="inlineStr">
@@ -32007,7 +32007,11 @@
           <t>Senior Machine Learning Engineer, Ads Optimization</t>
         </is>
       </c>
-      <c r="C462" t="inlineStr"/>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D462" t="inlineStr"/>
       <c r="E462" t="inlineStr">
         <is>
@@ -32060,11 +32064,7 @@
         </is>
       </c>
       <c r="U462" t="inlineStr"/>
-      <c r="V462" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V462" t="inlineStr"/>
     </row>
     <row r="463">
       <c r="A463" t="inlineStr">
@@ -32077,7 +32077,11 @@
           <t>Senior Staff Machine Learning Engineer, Feed Relevance</t>
         </is>
       </c>
-      <c r="C463" t="inlineStr"/>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D463" t="inlineStr"/>
       <c r="E463" t="inlineStr">
         <is>
@@ -32130,11 +32134,7 @@
         </is>
       </c>
       <c r="U463" t="inlineStr"/>
-      <c r="V463" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V463" t="inlineStr"/>
     </row>
     <row r="464">
       <c r="A464" t="inlineStr">
@@ -32147,7 +32147,11 @@
           <t>Senior Staff Machine Learning Engineer, GenAI Platform</t>
         </is>
       </c>
-      <c r="C464" t="inlineStr"/>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D464" t="inlineStr"/>
       <c r="E464" t="inlineStr">
         <is>
@@ -32200,11 +32204,7 @@
         </is>
       </c>
       <c r="U464" t="inlineStr"/>
-      <c r="V464" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V464" t="inlineStr"/>
     </row>
     <row r="465">
       <c r="A465" t="inlineStr">
@@ -32217,7 +32217,11 @@
           <t>Senior Staff Machine Learning Engineer, Notifications</t>
         </is>
       </c>
-      <c r="C465" t="inlineStr"/>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D465" t="inlineStr"/>
       <c r="E465" t="inlineStr">
         <is>
@@ -32270,11 +32274,7 @@
         </is>
       </c>
       <c r="U465" t="inlineStr"/>
-      <c r="V465" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V465" t="inlineStr"/>
     </row>
     <row r="466">
       <c r="A466" t="inlineStr">
@@ -32287,7 +32287,11 @@
           <t>Staff Machine Learning Engineer, Ads Foundational Representations</t>
         </is>
       </c>
-      <c r="C466" t="inlineStr"/>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D466" t="inlineStr"/>
       <c r="E466" t="inlineStr">
         <is>
@@ -32340,11 +32344,7 @@
         </is>
       </c>
       <c r="U466" t="inlineStr"/>
-      <c r="V466" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V466" t="inlineStr"/>
     </row>
     <row r="467">
       <c r="A467" t="inlineStr">
@@ -32357,7 +32357,11 @@
           <t>Staff Machine Learning Engineer, Consumer</t>
         </is>
       </c>
-      <c r="C467" t="inlineStr"/>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
       <c r="D467" t="inlineStr"/>
       <c r="E467" t="inlineStr">
         <is>
@@ -32410,11 +32414,7 @@
         </is>
       </c>
       <c r="U467" t="inlineStr"/>
-      <c r="V467" t="inlineStr">
-        <is>
-          <t>03 Applied AI Architect (high)</t>
-        </is>
-      </c>
+      <c r="V467" t="inlineStr"/>
     </row>
     <row r="468">
       <c r="A468" t="inlineStr">
@@ -32427,7 +32427,11 @@
           <t>Technical Program Manager, Compute Infrastructure</t>
         </is>
       </c>
-      <c r="C468" t="inlineStr"/>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>04 Technical Deployment Lead / Strategist</t>
+        </is>
+      </c>
       <c r="D468" t="inlineStr"/>
       <c r="E468" t="inlineStr">
         <is>
@@ -32484,11 +32488,143 @@
         </is>
       </c>
       <c r="U468" t="inlineStr"/>
-      <c r="V468" t="inlineStr">
-        <is>
-          <t>04 Technical Deployment Lead / Strategist (high)</t>
-        </is>
-      </c>
+      <c r="V468" t="inlineStr"/>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>ambral</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Head of Research</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr"/>
+      <c r="D469" t="inlineStr"/>
+      <c r="E469" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F469" t="inlineStr"/>
+      <c r="G469" t="inlineStr">
+        <is>
+          <t>04 Closed</t>
+        </is>
+      </c>
+      <c r="H469" t="inlineStr"/>
+      <c r="I469" t="inlineStr">
+        <is>
+          <t>manual-add</t>
+        </is>
+      </c>
+      <c r="J469" t="inlineStr"/>
+      <c r="K469" t="inlineStr"/>
+      <c r="L469" t="inlineStr">
+        <is>
+          <t>https://jobs.ashbyhq.com/Ambral/9a7d8a93-3c90-4a77-a022-f19c158a1fb3</t>
+        </is>
+      </c>
+      <c r="M469" t="inlineStr">
+        <is>
+          <t>$250,000 - $400,000 per year</t>
+        </is>
+      </c>
+      <c r="N469" t="inlineStr"/>
+      <c r="O469" t="inlineStr"/>
+      <c r="P469" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q469" t="n">
+        <v>5</v>
+      </c>
+      <c r="R469" t="inlineStr">
+        <is>
+          <t>Level is plausible (senior leadership) but track is completely wrong — this is a hands-on ML research role, not measurement/marketing science leadership. This is a PhD-level RL/LLM post-training research role building agent training environments and reward graders for foundation models — nothing in the candidate's background (MMM, attribution, propensity modeling, marketing measurement) touches reinforcement learning, LLM post-training, or agent evals. The domain overlap is zero; only the word 'model' connects them. Gaps: No PhD or research-scientist track record in ML/RL; No experience with LLM post-training, agent environments, or eval/grader design; Entire career is applied marketing/commercial data science, not foundation-model research</t>
+        </is>
+      </c>
+      <c r="S469" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T469" t="inlineStr">
+        <is>
+          <t>Unknown - Unknown</t>
+        </is>
+      </c>
+      <c r="U469" t="inlineStr"/>
+      <c r="V469" t="inlineStr"/>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>sentra</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Job opportunity: GTM Engineer at Sentra</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr"/>
+      <c r="D470" t="inlineStr"/>
+      <c r="E470" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F470" t="inlineStr"/>
+      <c r="G470" t="inlineStr">
+        <is>
+          <t>01 Open</t>
+        </is>
+      </c>
+      <c r="H470" t="inlineStr"/>
+      <c r="I470" t="inlineStr">
+        <is>
+          <t>manual-add</t>
+        </is>
+      </c>
+      <c r="J470" t="inlineStr"/>
+      <c r="K470" t="inlineStr"/>
+      <c r="L470" t="inlineStr">
+        <is>
+          <t>https://www.comeet.com/jobs/sentra/87.00B/gtm-engineer/00.17E</t>
+        </is>
+      </c>
+      <c r="M470" t="inlineStr"/>
+      <c r="N470" t="inlineStr"/>
+      <c r="O470" t="inlineStr"/>
+      <c r="P470" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q470" t="n">
+        <v>5</v>
+      </c>
+      <c r="R470" t="inlineStr">
+        <is>
+          <t>Cannot assess — no real job content, and title (GTM Engineer) is a different function from measurement/marketing science leadership. The scraped JD is a dead careers-page error template ("no open positions" / Lever boilerplate), not an actual job description. Separately, 'GTM Engineer' is typically a sales-engineering/technical-GTM IC role at a security company (Sentra does data security posture management), unrelated to measurement science, MMM, or causal inference. Gaps: No actual JD content to evaluate against; Role title suggests sales/solutions engineering, not measurement or data science</t>
+        </is>
+      </c>
+      <c r="S470" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T470" t="inlineStr">
+        <is>
+          <t>Unknown - Unknown</t>
+        </is>
+      </c>
+      <c r="U470" t="inlineStr"/>
+      <c r="V470" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after salary format and ghost-role fix
0 of 470 roles missing store_id, down from 3.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V470"/>
+  <dimension ref="A1:V471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4731,7 +4731,7 @@
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>03 Applied</t>
         </is>
       </c>
       <c r="H58" t="inlineStr"/>
@@ -4871,7 +4871,7 @@
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>03 Applied</t>
         </is>
       </c>
       <c r="H60" t="inlineStr"/>
@@ -14987,7 +14987,7 @@
       <c r="F211" t="inlineStr"/>
       <c r="G211" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H211" t="inlineStr"/>
@@ -15325,7 +15325,7 @@
       <c r="F216" t="inlineStr"/>
       <c r="G216" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H216" t="inlineStr"/>
@@ -19159,7 +19159,7 @@
       <c r="F273" t="inlineStr"/>
       <c r="G273" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>03 Applied</t>
         </is>
       </c>
       <c r="H273" t="inlineStr"/>
@@ -20173,7 +20173,7 @@
       <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>03 Applied</t>
         </is>
       </c>
       <c r="H288" t="inlineStr"/>
@@ -32441,7 +32441,7 @@
       <c r="F468" t="inlineStr"/>
       <c r="G468" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H468" t="inlineStr"/>
@@ -32581,7 +32581,7 @@
       <c r="F470" t="inlineStr"/>
       <c r="G470" t="inlineStr">
         <is>
-          <t>01 Open</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H470" t="inlineStr"/>
@@ -32626,6 +32626,76 @@
       <c r="U470" t="inlineStr"/>
       <c r="V470" t="inlineStr"/>
     </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Applied AI Architect, Industries</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>03 Applied AI Architect</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr"/>
+      <c r="E471" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="F471" t="inlineStr"/>
+      <c r="G471" t="inlineStr">
+        <is>
+          <t>00 New find</t>
+        </is>
+      </c>
+      <c r="H471" t="inlineStr"/>
+      <c r="I471" t="inlineStr">
+        <is>
+          <t>live</t>
+        </is>
+      </c>
+      <c r="J471" t="inlineStr"/>
+      <c r="K471" t="inlineStr"/>
+      <c r="L471" t="inlineStr">
+        <is>
+          <t>https://job-boards.greenhouse.io/anthropic/jobs/5390765008</t>
+        </is>
+      </c>
+      <c r="M471" t="inlineStr"/>
+      <c r="N471" t="inlineStr"/>
+      <c r="O471" t="inlineStr"/>
+      <c r="P471" t="inlineStr">
+        <is>
+          <t>2026-09-12</t>
+        </is>
+      </c>
+      <c r="Q471" t="n">
+        <v>15</v>
+      </c>
+      <c r="R471" t="inlineStr">
+        <is>
+          <t>Level is roughly comparable (Senior Director/Principal vs Architect), but track is wrong: this is a hands-on, customer-facing solutions-engineering/architecture role, not a measurement-science leadership role. The candidate's entire career is marketing/measurement science - MMM, attribution, propensity and segmentation models built on classical ML and analytics stacks (scikit-learn, statsmodels, Snowflake, Databricks). Anthropic's Applied AI Architect role is about designing and building generative-AI/LLM solutions with enterprise customers across industries, which is a different technical domain (LLM application architecture, prompt/agent design, API integration) that the resume only gestures at with one vague Arjentic bullet ('custom agentic solutions'). Gaps: No demonstrated hands-on experience building with LLMs/foundation models, prompt engineering, or agentic frameworks - only a single unelaborated resume bullet; Role is customer-facing solutions architecture/engineering, not measurement or causal inference - core resume skills don't transfer directly; Based in New York; role is London-based with no relocation signal</t>
+        </is>
+      </c>
+      <c r="S471" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T471" t="inlineStr">
+        <is>
+          <t>Tech - AI Lab</t>
+        </is>
+      </c>
+      <c r="U471" t="inlineStr"/>
+      <c r="V471" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(artifacts): daily run 2026-09-13
0 new live roles judged (all cached); user closed 11 more roles via dashboard since yesterday.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -7647,7 +7647,7 @@
       <c r="F101" t="inlineStr"/>
       <c r="G101" t="inlineStr">
         <is>
-          <t>02 Researching</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H101" t="inlineStr"/>
@@ -19637,7 +19637,7 @@
       <c r="F280" t="inlineStr"/>
       <c r="G280" t="inlineStr">
         <is>
-          <t>02 Researching</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H280" t="inlineStr"/>
@@ -32651,7 +32651,7 @@
       <c r="F471" t="inlineStr"/>
       <c r="G471" t="inlineStr">
         <is>
-          <t>00 New find</t>
+          <t>04 Closed</t>
         </is>
       </c>
       <c r="H471" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after content-radar 6-pick change
Radar re-run this session picked up 6 stories, up from 3; tracker/db reflect the user's own dashboard salary edits.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -4247,7 +4247,7 @@
       </c>
       <c r="M51" t="inlineStr">
         <is>
-          <t>$255,000—$375,000</t>
+          <t>255-375</t>
         </is>
       </c>
       <c r="N51" t="inlineStr"/>
@@ -4383,7 +4383,7 @@
       </c>
       <c r="M53" t="inlineStr">
         <is>
-          <t>$129,840.00 - $194,760.00</t>
+          <t>130-195</t>
         </is>
       </c>
       <c r="N53" t="inlineStr"/>
@@ -4601,7 +4601,7 @@
       </c>
       <c r="M56" t="inlineStr">
         <is>
-          <t>$150,000 - $200,000,</t>
+          <t>150-200</t>
         </is>
       </c>
       <c r="N56" t="inlineStr"/>
@@ -4675,7 +4675,7 @@
       </c>
       <c r="M57" t="inlineStr">
         <is>
-          <t>$276,000 to $379,500</t>
+          <t>276-379</t>
         </is>
       </c>
       <c r="N57" t="inlineStr"/>
@@ -4749,7 +4749,7 @@
       </c>
       <c r="M58" t="inlineStr">
         <is>
-          <t>$320,000 - $380,000</t>
+          <t>320-380</t>
         </is>
       </c>
       <c r="N58" t="inlineStr"/>
@@ -4819,7 +4819,7 @@
       </c>
       <c r="M59" t="inlineStr">
         <is>
-          <t>$250K - $325K</t>
+          <t>250-325</t>
         </is>
       </c>
       <c r="N59" t="inlineStr"/>
@@ -4889,9 +4889,7 @@
       </c>
       <c r="M60" t="inlineStr">
         <is>
-          <t>$253,000.00
--
-$314,000.00</t>
+          <t>253-314</t>
         </is>
       </c>
       <c r="N60" t="inlineStr"/>
@@ -26985,7 +26983,7 @@
       </c>
       <c r="M387" t="inlineStr">
         <is>
-          <t>$163,600.00 - $245,400.00</t>
+          <t>163-245</t>
         </is>
       </c>
       <c r="N387" t="inlineStr"/>
@@ -32459,7 +32457,7 @@
       </c>
       <c r="M468" t="inlineStr">
         <is>
-          <t>$257,000 - $335,000 per year</t>
+          <t>257-335</t>
         </is>
       </c>
       <c r="N468" t="inlineStr"/>
@@ -32529,7 +32527,7 @@
       </c>
       <c r="M469" t="inlineStr">
         <is>
-          <t>$250,000 - $400,000 per year</t>
+          <t>250-400</t>
         </is>
       </c>
       <c r="N469" t="inlineStr"/>

</xml_diff>

<commit_message>
chore(artifacts): complete the Vouri record (category, sector) and daily verdicts
Completeness scan found one role (Vouri, added via VentureLoop URL) missing sector and category evaluation; a normal jobs run resolved both.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V471"/>
+  <dimension ref="A1:V472"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4258,16 +4258,16 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>35</v>
+        <v>55</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Director-to-Director on title, but this is in-house product/growth analytics leadership at a marketplace, not marketing measurement — a domain change dressed up as a level match. The candidate's entire track record is agency/brand-side marketing science — MMM, MTA, audience segmentation, media budget allocation. This role wants a Director running product experimentation and growth analytics for a consumer marketplace vertical (Grocery/Alcohol/Retail delivery), reporting to a Senior Director in a large in-house Analytics org. 'Causal inference and experimentation' overlaps on paper, but the actual job is product decision-making (what to build, which growth lever to pull), not marketing/media measurement — a different function wearing similar words. Gaps: No in-house consumer marketplace or product analytics experience — career is entirely agency/brand-side marketing measurement; No evidence of running product experimentation at DoorDash's scale (0→1 launches plus high-traffic Cx surfaces) vs. media/campaign-level experiments; Team scope here likely exceeds candidate's largest team led (5 people) given 'lead and grow a team of DS leaders and practitioners across a portfolio'</t>
+          <t>Director + people-manager track matches current level exactly, but this is product/growth analytics, not marketing measurement. Deep causal inference and experimentation chops transfer directly, and leading a DS team is exactly what this candidate does now. But the domain is product analytics for a marketplace vertical (grocery/alcohol/retail ops), not marketing science — no MMM, attribution, or media measurement in scope at all. Gaps: No consumer marketplace/product-analytics background (vs. media/marketing measurement); JD wants 0→1 product experimentation, not brand/channel measurement</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>research</t>
         </is>
       </c>
       <c r="T51" t="inlineStr">
@@ -4394,11 +4394,11 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>Banking 'VP' is typically a mid-level individual grade, not equivalent to Director/Senior Director — this reads as a step down despite the title. Marketing data science domain overlaps, but the posted comp ($130-195k) sits well below what the candidate should command at Senior Director level, and financial services is an unfamiliar regulated domain with no prior exposure. Gaps: Comp band implies a lower organizational level than current role; No financial-services/regulated-industry experience</t>
+          <t>VP at a bank is a mid-level IC/manager title, roughly a step below the candidate's current Senior Director seat — comp range (130-195k) confirms it. Marketing data science is the right domain, but the level and comp band both signal this sits below where the candidate is already operating. Taking this would be a step down in scope and title, not a lateral move. Gaps: Title/level is below current Senior Director seniority; Comp ceiling (195k) is below likely current comp</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -4612,11 +4612,11 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Exact title match (Senior Director, Marketing Science) at comparable scope — right level, right track. Direct title and domain match to the current OMD role, with the MMM reconciliation, forecasting, and cross-channel measurement experience translating well to sponsorship/media ROI questions a league would face. Comp is lower than agency-holdco norms but plausible for sports. Gaps: No demonstrated sports/sponsorship or ticketing-revenue measurement experience specifically; Would need to translate ad-agency MMM framing to league sponsorship and fan-engagement metrics</t>
+          <t>Title-for-title match: Senior Director, Marketing Science is the candidate's current exact title and level. This is squarely in-lane — marketing science leadership at the Senior Director level, same as the current OMD role. Comp (150-200k) is lower than current band, likely reflecting sports/entertainment budgets rather than agency holding-co scale, but the role itself is a real match. Gaps: Comp likely below current level; Sports/entertainment measurement maturity may be less developed than agency-side MMM work — could mean more building-from-scratch</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -4686,11 +4686,11 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Director title fits, but this is an applied AI/ML science track for an ads product (ranking, auction, budget optimization) — a function drift from marketing measurement science into ML/ads-engineering research. The comp band signals a bar for deep applied ML/research talent building the ads product itself, not a measurement leader evaluating campaign performance from the outside. Candidate's causal inference and MMM background doesn't map to ads-ranking ML systems. Gaps: No ad-ranking, auction, or ML-infra engineering background; Role likely wants research-caliber ML depth, not agency measurement science</t>
+          <t>Director level matches, but track is applied ML/ads science (ranking, ad systems), not measurement/causal inference leadership. This is an ads ML science role — building ranking and ad-serving models — not marketing measurement. The candidate has no applied ML/ads infrastructure background; the overlap is keyword-level ("ads", "director") not substantive. Gaps: No ad-ranking/ad-serving ML systems experience; Function is applied ML engineering leadership, not causal measurement</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -4760,16 +4760,16 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>66</v>
+        <v>40</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>"Leader" title and comp band ($320-380K) match Director+ level; track is right (management), but "Applied Science" naming suggests more ML-research emphasis than pure measurement science. Attentive is an SMS/email marketing platform — directly adjacent to the candidate's Samsung work deploying propensity/recommendation models across Email/SMS/Push. The gap is whether this role wants deep applied-ML/research chops (model architecture, experimentation at the algorithm level) versus measurement/causal leadership. Gaps: No causal inference / MMM / attribution language in the title — may skew toward core ML/personalization rather than measurement science; "Applied Science" framing could mean IC-adjacent technical depth beyond the candidate's stats/causal toolkit</t>
+          <t>Title is vague ("Applied Science / Data Science Leader") and skews toward a research/ML IC-adjacent track rather than a clear people-management measurement seat. Attentive is a marketing/messaging platform, so there's plausible domain adjacency, but "Applied Science" framing plus the high comp band suggests they want deep ML/research depth (likely for their own product's ML models) rather than a marketing measurement strategist. Gaps: Unclear if role is measurement-facing or product-ML-facing; "Applied Science" track typically wants hands-on modeling depth beyond marketing science scope</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>skip</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Head-level title is level-appropriate, but the domain is a hard swap: clinical documentation AI, not marketing measurement. Abridge builds AI for clinical note-taking — none of the candidate's causal inference, MMM, or attribution work transfers to healthcare NLP/clinical data science. This is a domain mismatch dressed up as a title match. Gaps: Zero healthcare/clinical data experience; No evidence of NLP/LLM-adjacent applied science work at the modeling level this role likely requires</t>
+          <t>Head of DS level is right, but domain is healthcare AI/clinical documentation — total function drift from marketing science. Abridge builds clinical documentation AI. There is no marketing, measurement, or causal-inference-for-commercial-decisions angle here; this would require an entirely different domain expertise (healthcare NLP/ML). Gaps: Zero healthcare/clinical domain experience; No NLP/LLM applied research background</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -4900,11 +4900,11 @@
         </is>
       </c>
       <c r="Q60" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Exact title match (Senior Director) — same level as current role, so this is a lateral move, not a promotion. Paramount is a media company where subscriber/marketing measurement work plausibly overlaps with the candidate's MMM and attribution background, but "Data Science" here could just as easily mean content/streaming recommendation or subscriber churn modeling with no marketing-measurement mandate. No JD excerpt to confirm. Gaps: Unclear if scope is marketing measurement vs. product/content data science; No detail on team size or whether this is a build vs. maintain mandate</t>
+          <t>Level matches exactly (Senior Director), but the generic "Data Science" title leaves the actual scope (subscriber/content analytics vs. marketing measurement) unclear. Media/entertainment is a plausible adjacent industry and the level is right, but without JD detail on whether this is marketing measurement, streaming subscriber analytics, or content ML, it's a bet on title alone. Worth researching before committing. Gaps: JD doesn't confirm marketing/measurement scope vs. broader subscriber or content data science; No streaming/media subscription analytics track record</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -26994,11 +26994,11 @@
         </is>
       </c>
       <c r="Q387" t="n">
-        <v>74</v>
+        <v>90</v>
       </c>
       <c r="R387" t="inlineStr">
         <is>
-          <t>SVP at a bank maps roughly to Senior Director/Director in agency terms — a lateral move, not a stretch or a demotion. This is a genuine measurement-science leadership role built around attribution, MMM, and incrementality testing — the candidate's actual core. Directly analogous to his OMD work reconciling two vendor MMMs into one cross-channel investment view, and to leading a measurement team; vendor management (MMM vendors at OMD, MTA vendors at Merkle) also lines up well. Gaps: No financial services or highly regulated-industry experience; JD explicitly calls for work with legal/compliance/procurement in a regulated environment; Career-goals notes flag clean rooms as a gap, and this JD implies adtech/identity-solution fluency (DSP/SSP, ADH-style environments) the resume doesn't evidence</t>
+          <t>SVP at a bank is a senior leadership title (roughly Director/Senior Director equivalent in tech) and matches current level and trajectory exactly. This is close to a direct restatement of the candidate's resume: attribution, MMM, incrementality testing, vendor management, cross-channel measurement narrative for senior stakeholders. Rare case where domain, level, and function all line up. Gaps: No banking/regulated-industry experience (compliance, legal, procurement rigor called out in JD); Clean rooms/adtech tool depth (DSP/SSP, identity solutions) is a stated gap vs. the candidate's agency-side background</t>
         </is>
       </c>
       <c r="S387" t="inlineStr">
@@ -32468,11 +32468,11 @@
         </is>
       </c>
       <c r="Q468" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="R468" t="inlineStr">
         <is>
-          <t>Irrelevant axis — this isn't a measurement/data-science role at any level, it's a hardware/datacenter TPM role. This is a technical program management role for GPU cluster bring-up: hardware, networking, power, cooling, vendor/construction coordination. Nothing in the candidate's background — MMM, attribution, causal inference, marketing analytics leadership — maps to running compute infrastructure delivery. Gaps: No infrastructure/hyperscaler program management experience (capital projects, networking, power/cooling); No TPM track record; candidate is a data science/analytics people-manager, not an engineering program manager</t>
+          <t>Completely different function — hardware/GPU infrastructure program management, not data science or measurement at any level. No overlap whatsoever: this role is about physical GPU cluster bring-up, networking, power, and cooling logistics. Nothing in the candidate's background — marketing science, causal inference, team leadership in analytics — applies here. Gaps: No infrastructure/hardware program management experience; No compute/datacenter operations background</t>
         </is>
       </c>
       <c r="S468" t="inlineStr">
@@ -32538,11 +32538,11 @@
         </is>
       </c>
       <c r="Q469" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="R469" t="inlineStr">
         <is>
-          <t>Level is plausible (senior leadership) but track is completely wrong — this is a hands-on ML research role, not measurement/marketing science leadership. This is a PhD-level RL/LLM post-training research role building agent training environments and reward graders for foundation models — nothing in the candidate's background (MMM, attribution, propensity modeling, marketing measurement) touches reinforcement learning, LLM post-training, or agent evals. The domain overlap is zero; only the word 'model' connects them. Gaps: No PhD or research-scientist track record in ML/RL; No experience with LLM post-training, agent environments, or eval/grader design; Entire career is applied marketing/commercial data science, not foundation-model research</t>
+          <t>Title-senior but a deep ML/RL research IC-track role requiring a PhD — different track entirely from marketing science leadership. This wants a hands-on RL/LLM post-training researcher building environment-and-reward systems for agent training. The candidate's causal inference and marketing measurement background doesn't translate to this research agenda. Gaps: No PhD or RL/LLM post-training research background; No agent environment/eval engineering experience</t>
         </is>
       </c>
       <c r="S469" t="inlineStr">
@@ -32694,6 +32694,72 @@
       <c r="U471" t="inlineStr"/>
       <c r="V471" t="inlineStr"/>
     </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Vouri</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Sr. Director, Data Science &amp; AI</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr"/>
+      <c r="D472" t="inlineStr"/>
+      <c r="E472" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="F472" t="inlineStr"/>
+      <c r="G472" t="inlineStr">
+        <is>
+          <t>01 Open</t>
+        </is>
+      </c>
+      <c r="H472" t="inlineStr"/>
+      <c r="I472" t="inlineStr">
+        <is>
+          <t>manual-add</t>
+        </is>
+      </c>
+      <c r="J472" t="inlineStr"/>
+      <c r="K472" t="inlineStr"/>
+      <c r="L472" t="inlineStr">
+        <is>
+          <t>https://www.ventureloop.com/ventureloop/jobdetail.php?jobid=2983149&amp;hc=vuori&amp;jt=sr-director-data-science-andamp-ai</t>
+        </is>
+      </c>
+      <c r="M472" t="inlineStr"/>
+      <c r="N472" t="inlineStr"/>
+      <c r="O472" t="inlineStr"/>
+      <c r="P472" t="inlineStr">
+        <is>
+          <t>2026-09-13</t>
+        </is>
+      </c>
+      <c r="Q472" t="n">
+        <v>48</v>
+      </c>
+      <c r="R472" t="inlineStr">
+        <is>
+          <t>Level (Sr. Director) matches, but the JD excerpt is too thin to confirm this is a marketing-measurement seat rather than broader DTC data science (demand planning, ops, personalization). Level and industry (DTC retail) are plausible fits, and the candidate has relevant segmentation/personalization experience from Samsung and L'Oréal, but without more JD detail this reads as a generic "Data Science &amp; AI" mandate that may extend well beyond marketing measurement. Gaps: Insufficient JD detail to confirm measurement/marketing scope; No DTC apparel/retail-specific experience</t>
+        </is>
+      </c>
+      <c r="S472" t="inlineStr">
+        <is>
+          <t>skip</t>
+        </is>
+      </c>
+      <c r="T472" t="inlineStr">
+        <is>
+          <t>Unknown - Unknown</t>
+        </is>
+      </c>
+      <c r="U472" t="inlineStr"/>
+      <c r="V472" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(artifacts): rebuild after fit-fingerprint fix (one-time 58-role re-judge)
Migration to the new fingerprint scheme judged 58 roles once; verified a second run reuses all 471 at $0.
</commit_message>
<xml_diff>
--- a/artifacts/jobs/org-roles-tracker.xlsx
+++ b/artifacts/jobs/org-roles-tracker.xlsx
@@ -1790,11 +1790,11 @@
         </is>
       </c>
       <c r="Q18" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>Director title matches level, but this reads as general retail/e-commerce DS, not a measurement-science mandate. Chewy's Director DS seat is almost certainly broad consumer DS (personalization, supply/demand forecasting, growth) rather than causal marketing measurement, so the candidate's differentiated MMM/attribution/clean-room specialization isn't the ask. WA location adds friction for an NY-based candidate. Gaps: Not a measurement/marketing-science mandate - general retail DS; WA location vs NY-based candidate</t>
+          <t>Director title matches, but you've already flagged this as a location/gap close — don't fight your own read. Chewy DS is retail e-commerce merchandising/ops focus, not marketing measurement or causal inference — this is domain drift dressed up as a title match. WA location is also a hard relocation ask you're not positioned for. Gaps: No retail/e-commerce ops DS background; WA location mismatch</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -1870,11 +1870,11 @@
         </is>
       </c>
       <c r="Q19" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>'Lead Decision Scientist' is a senior-IC title, a track change and likely a step down from candidate's people-manager Director track. Healthcare product/decision analytics for Aetna shares causal-inference DNA but none of the MMM/attribution/clean-room specialization the candidate is built around. It surfaced via a forward, not a targeted search, and the IC track cuts against a decade of managing teams. Gaps: Healthcare product analytics domain, not marketing measurement; IC 'Lead' title vs candidate's people-manager Director track</t>
+          <t>"Lead" is ambiguous IC/manager, likely a step down from your current Director scope either way. Product Analytics for a health plan is decision science applied to product/member experience, not marketing measurement or MMM — the causal-inference skill transfers in the abstract but the domain (healthcare product) and function (product analytics, not marketing science) are both off your core lane. Being forwarded doesn't change that the JD reads as product, not GTM. Gaps: No healthcare/health-insurance domain experience; Product analytics function, not marketing/measurement science</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -1948,11 +1948,11 @@
         </is>
       </c>
       <c r="Q20" t="n">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>'Leader' title and comp band read as Director/VP-equivalent, roughly matching level, but function is GTM/technical-success, not measurement science. This looks like applied DS embedded in OpenAI's go-to-market and technical customer-success org - closer to the candidate's #2 career goal (Field CTO/Head of AI Solutions) than to core measurement work. The Samsung $100M enterprise account-segmentation program is a real, if partial, credential, but OpenAI's bar for this kind of GTM-intelligence leadership likely wants someone with deeper enterprise sales-analytics or solutions pedigree. Gaps: No direct GTM/sales-analytics leadership experience at this scale; Role scope ambiguous - could be more solutions-strategy than DS leadership</t>
+          <t>"Leader" + comp band reads Director-equivalent or above — level is plausible, but the track (GTM intelligence/technical success) is more solutions-architecture than measurement science. This looks like it wants someone who bridges data science with GTM/solutions delivery — close to your "bridge between causal inference and commercial impact" positioning and your Field CTO/Applied AI Architect goals, not your Marketing Science Lead goal. The JD not mentioning GTM/product explicitly is a real signal, not a coincidence — it may be scoped more toward internal enterprise-customer technical success than measurement per se. Gaps: No direct GTM/solutions-engineering or customer-facing technical delivery experience; No AI/LLM product background; Unclear if role is people-manager or senior IC</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2018,11 +2018,11 @@
         </is>
       </c>
       <c r="Q21" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>Sr Director matches level, but 'Data' is a broad generalist mandate, not measurement-specific. Already flagged as closing due to gaps. Navan's Sr Director Data role is likely a general data-leadership seat spanning product analytics, platform, and growth, without the causal/MMM specialization the candidate is positioned around, and SF adds relocation friction. Gaps: Broad generalist data leadership mandate, not measurement-specific; SF location vs NY-based candidate</t>
+          <t>Title matches Director-plus level, but you've already flagged this as a gaps-close — trust that read. Navan Sr Director, Data is a broad data/analytics leadership role for a travel/expense SaaS company, with no visible marketing measurement or causal-inference core — it's DS leadership generically, not your specialization. Gaps: No B2B SaaS product-data domain experience; Broad data-org leadership scope beyond measurement science</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
@@ -2090,11 +2090,11 @@
         </is>
       </c>
       <c r="Q22" t="n">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>Director title matches level, but this is product-embedded DS/ML for healthcare RCM, not marketing measurement. Adonis is a healthcare revenue-cycle AI startup; 'Director of DS/ML' almost certainly means owning ML models embedded in their product. No MMM/attribution/clean-room overlap, and startup product-ML leadership is a different skill emphasis than measurement science. Gaps: Healthcare RCM product domain, no marketing measurement component; Startup product-ML engineering focus vs measurement-science specialization</t>
+          <t>Director title matches your current level. Adonis is healthcare revenue-cycle automation — the JD title suggests general DS/ML leadership, not marketing or measurement science, and there's no indication this role touches causal inference, MMM, or attribution. Level is right but domain is a real stretch from your marketing-science core. Gaps: No healthcare revenue-cycle domain experience; Role reads as general ML/product DS, not measurement science</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
@@ -2168,11 +2168,11 @@
         </is>
       </c>
       <c r="Q23" t="n">
-        <v>18</v>
+        <v>28</v>
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>Research-scientist IC track; candidate is an applied-measurement people-manager - mismatched on both track and function. ML Scientist roles at this level are research-track and typically expect a research/publication background. Candidate's decade of experience is applied measurement leadership, not ads-understanding research science. Already deprioritized in favor of other applications. Gaps: Research-scientist track vs candidate's applied-leadership track; No research/publication background in ads modeling</t>
+          <t>ML Scientist is a senior IC research-scientist track — a real track change and step down from your Director/people-manager seat, regardless of the level number. This is a research-scientist role (ads member understanding) requiring deep applied ML research chops, not a measurement-science leadership role. You manage teams that build forecasting and segmentation systems — you're not positioned as a hands-on research scientist competing against PhD-track candidates. Gaps: IC research-scientist track vs. your management track; No published/deep applied-research ML portfolio for this level</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
@@ -2238,11 +2238,11 @@
         </is>
       </c>
       <c r="Q24" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>Unmodified 'Data Scientist' title is a clear IC step down from candidate's Director/Senior Director level. Generic mid-level IC title; deprioritized since candidate already applied to the Lead-level OpenAI role, and taking this would be a real level regression. Gaps: Title level is a step down from Director; Redundant with the Lead-level OpenAI application already in flight</t>
+          <t>"Data Scientist" with no Staff/Lead/Senior qualifier is a junior-to-mid IC title — several levels below your Director/Senior Director track. This is a straightforward IC data scientist opening; taking it would be a significant title and scope downgrade from your current Senior Director seat leading a team of 5. You've correctly deprioritized this in favor of the Lead-level opening. Gaps: Level mismatch — IC vs. your management track; Ads demand forecasting is adjacent but not your specialization</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
@@ -2308,11 +2308,11 @@
         </is>
       </c>
       <c r="Q25" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>Generic IC-level 'Data Scientist' title, a step down from current seniority. Deprioritized in favor of the Lead-level application. 'Business' DS is a generalist scope with no called-out measurement/causal specialization. Gaps: IC level below candidate's current title; Generic scope, unclear measurement relevance</t>
+          <t>Same as above — unqualified "Data Scientist" title is IC-level, well below your current scope. Generic business data scientist role with no measurement/marketing-science specificity in the title; a clear downgrade from Senior Director managing a team. You've already applied to the Lead-level OpenAI role, which is the right call. Gaps: Level mismatch; No stated marketing/measurement focus</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
@@ -2378,11 +2378,11 @@
         </is>
       </c>
       <c r="Q26" t="n">
-        <v>22</v>
+        <v>15</v>
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>IC-level title, a step down; SMB growth analytics is product/growth-metrics work, not causal measurement. Deprioritized already. Growth analytics for SMB ads is adjacent but not the causal/MMM measurement specialization the candidate is positioned around. Gaps: IC title, step down from Director; SMB growth analytics vs measurement-science specialization</t>
+          <t>IC-level title, well below your Director track. SMB ads growth DS is a hands-on growth-analytics IC role; correctly deprioritized in favor of the Lead opening you already applied to. Gaps: Level mismatch; SMB growth-analytics is a narrower function than your measurement-science remit</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
@@ -2520,11 +2520,11 @@
         </is>
       </c>
       <c r="Q28" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>'ML Data Scientist' IC title is a step down from Director, despite forecasting being a genuine strength. Deprioritized in favor of the Lead-level OpenAI application. Forecasting is one of the candidate's strongest proven areas (Gap Inc. revenue forecasting suite), but the title doesn't match current seniority. Gaps: IC-level title, step down from Director/Senior Director; Redundant with the Lead-level OpenAI application</t>
+          <t>Title is unqualified IC ("ML Data Scientist"), a track/level step down from Director even though comp implies a senior-leaning band at OpenAI. Forecasting is genuinely your strongest technical match — you built the revenue forecasting model suite at OMD — but the title reads as IC, not a leadership seat, and you've already applied to the Lead-level role instead. Worth noting the domain overlap is real even if this particular req isn't the right seat. Gaps: IC title vs. your management track; Already pursuing the Lead-level equivalent</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
@@ -2598,7 +2598,7 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>Currently a people-manager; Pinterest Staff DS is a senior IC role, a different track and likely a step down in title. Staff DS is a deep IC track, and the candidate has been managing teams since 2020 with a resume built around leadership, not hands-on IC modeling depth. Already deprioritized in favor of other applications. Gaps: IC track vs candidate's management track; Ads product domain one step removed from marketing measurement</t>
+          <t>Staff DS is a senior IC ladder, not a manager ladder — taking this would be a track change and a step down from Senior Director leading a team of 5. Ads Product at Pinterest is closer to product-embedded data science than measurement/causal science, and Staff DS means going back to individual contribution after several years managing teams. You've correctly deprioritized this. Gaps: IC track vs. management track; Ads product function is product-embedded DS, not core measurement science</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
@@ -2668,11 +2668,11 @@
         </is>
       </c>
       <c r="Q30" t="n">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>Same IC/manager track mismatch as the other Pinterest Staff DS postings; marketing domain is closer to candidate's background but the track issue remains. Of the three Pinterest Staff DS postings, marketing is domain-closest to the candidate's expertise, but it's still a senior-IC seat, not a leadership seat, and the candidate's own notes already rank it below the other Pinterest options. Gaps: IC track vs candidate's management track; Comp band lower than comparable Pinterest DS postings</t>
+          <t>Staff DS is still IC-track — same management-to-IC step down as the other Pinterest Staff DS roles, domain fit slightly better. Marketing is the right domain, closer to your MMM/attribution core than the Ads Product or Notifications variants, but it's still a Staff (senior IC) ladder position, not a leadership seat matching your current scope. Gaps: IC track vs. management track; Would require stepping back from team leadership</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
@@ -2742,11 +2742,11 @@
         </is>
       </c>
       <c r="Q31" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>Same IC/manager track mismatch, and notifications/growth is further from measurement science than the other Pinterest postings. Notifications is a lifecycle/growth-engagement domain, not causal measurement work; combined with the Staff IC track mismatch, this is the weakest of the three Pinterest Staff DS roles. Gaps: IC track vs candidate's management track; Notifications/lifecycle domain has little measurement-science overlap</t>
+          <t>Staff DS IC track — track/level mismatch, plus weakest domain fit of the three Pinterest DS roles. Notifications is lifecycle/engagement optimization, not marketing measurement or causal inference — the weakest domain match of the Pinterest set on top of the same IC track-change problem. Gaps: IC track vs. management track; Notifications/engagement domain is furthest from measurement science</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
@@ -2818,11 +2818,11 @@
         </is>
       </c>
       <c r="Q32" t="n">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>'Lead' scope for a dedicated measurement product aligns well with candidate's measurement-science specialization and current level. This is a genuine domain match - measurement leadership tied to Pinterest's tvScientific streaming-TV incrementality partnership, squarely in the candidate's incrementality/geo-lift/MTA wheelhouse. The 'Lead' framing fits a senior seat rather than a pure research or engineering track. Gaps: Streaming/CTV incrementality specifics vs candidate's linear/digital MMM background; Unclear from title whether scope is IC or people-manager</t>
+          <t>"Measurement Lead" reads senior and domain-matched — this is close to a direct hit on your #1 target role (Measurement/Marketing Science Lead at a platform org). This is measurement leadership for a TV/streaming attribution integration on Pinterest's platform — squarely your causal-inference/attribution/measurement wheelhouse, and platform-side exposure would directly close your agency-vs-platform gap. Your MMM/attribution reconciliation work at OMD and Zenith is directly relevant experience to lead with. Gaps: No prior platform-side (vs. agency-side) measurement experience; No streaming/TV-specific attribution experience; Clean rooms gap still applies if this touches ADH-style infrastructure</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
@@ -2896,11 +2896,11 @@
         </is>
       </c>
       <c r="Q33" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>'Measurement Lead' matches candidate's specialization, and comp/scope look like a credible fit for a Senior Director stepping into a high-prestige lead seat. Directly in the core domain - ads measurement leadership for Netflix's scaled/SMB advertiser segment - drawing on the candidate's MMM, attribution, and incrementality background. This is one of the strongest matches in the batch on domain and level both. Gaps: No direct streaming/CTV ads measurement experience specifically; Scaled Solutions (SMB) client sophistication differs from candidate's enterprise/Fortune 500 experience</t>
+          <t>"Lead" plus scope (regional ads measurement) matches your Director-level management track well. This is close to verbatim your #1 target role — ads measurement leadership at a major platform. Your background in MTA, MMM, and geo-lift design translates directly, and the "Scaled Solutions" framing (serving many advertisers efficiently) echoes your self-serve tooling work at OMD. Gaps: Agency-side background, not platform ad-sales measurement experience; No streaming/video-specific measurement portfolio; Clean rooms gap (Netflix ads likely touches ADH-style clean room infra)</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
@@ -2970,7 +2970,7 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>Director level matches candidate's current Senior Director/Director track — right level, right track. Zocdoc needs forecasting/attribution/MMM leadership for marketing spend decisions; candidate's OMD revenue forecasting suite and prior agency attribution/MMM work map directly onto this. Team-leadership scope matches candidate's management track. Gaps: No healthcare/marketplace vertical experience; Comp range ($220-300k) may sit below what a Senior Director title commands if leveled as pure Director</t>
+          <t>Director title is an exact level match to your current Senior Director seat — no track or level question here. Marketing DS at Director level is the most literal title-and-function match in this batch — MMM, attribution, and segmentation for a consumer marketplace maps directly onto your OMD/Zenith/Merkle experience. Main open question is company-stage fit (Zocdoc scale vs. holding-company agency scale) but that's a lesser gap than domain or track mismatches elsewhere. Gaps: No healthcare-marketplace domain experience; Unclear team size/scope vs. your current team of 5</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
@@ -3036,11 +3036,11 @@
         </is>
       </c>
       <c r="Q35" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>EVP is a stretch above candidate's current Senior Director title, but same track (agency analytics leadership) with a direct warm contact already in play. Deep agency analytics pedigree across three prior agency roles (Zenith, Merkle, Tinuiti) plus current OMD measurement leadership is exactly the resume for an agency EVP Analytics seat. A warm contact (Kasper) is already engaged. Gaps: Never held an EVP/VP-level title — will need to sell Senior Director scope as equivalent; No public track record running an org at EVP headcount scale</t>
+          <t>EVP is a level up from current Senior Director, but it's a natural next rung on the exact same agency-measurement ladder — not a track change. Direct continuation of the Zenith/OMD/Merkle/Tinuiti agency-measurement career line, just at a bigger title and presumably bigger book of business. Candidate has already run MMM, MTA, and segmentation practices inside agencies at this scale. Gaps: EVP is untested title level — need to confirm scope (staff size, P&amp;L) matches what agencies mean by EVP vs. what candidate has run; No confirmed relationship yet beyond initial LI outreach</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
@@ -3106,11 +3106,11 @@
         </is>
       </c>
       <c r="Q36" t="n">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>Principal DS is a senior IC seat; candidate has been a people manager since 2020 — a track change likely read as a step down. Ads measurement has some overlap with attribution/MTA work, but Reddit is hiring a technical IC to ship models hands-on, not to lead a team or own agency-style client relationships. Gaps: No recent hands-on IC modeling — resume is team-lead/owner framing since 2020; No large-scale ads-platform or ranking-model experience</t>
+          <t>Principal DS is a senior IC technical role; candidate is currently a people-manager (team of 5) — this is a track change and likely a step down in scope of influence even if title reads 'senior'. Domain (ads measurement) is adjacent to candidate's marketing-science background, but Reddit's ads DS org wants deep hands-on causal/ML IC work at platform scale, not agency-side MMM/attribution leadership. No evidence in the resume of platform-scale ads ranking or auction data science. Gaps: No production ads-platform DS experience (auction, ranking, incrementality at platform scale); Manager-to-senior-IC track change not addressed</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
@@ -3176,11 +3176,11 @@
         </is>
       </c>
       <c r="Q37" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>Senior Staff is IC-ladder; track mismatch against candidate's manager career, compounded by a privacy/signals focus outside candidate's stack. "Signals, Privacy" points to identity/measurement infrastructure engineering for a post-cookie world, a different specialty than candidate's MMM/attribution/segmentation background. Gaps: No privacy-engineering or identity-signal infrastructure experience; IC track vs. candidate's manager track</t>
+          <t>Sr Staff DS is a senior IC track; candidate's current track is people-management. Also a specialized technical niche (privacy-preserving signals) outside candidate's experience. The 'signals, privacy' focus (differential privacy, signal loss, MMP-style measurement under platform tracking restrictions) is a distinct technical specialty candidate hasn't worked in. Agency-side MTA experience doesn't transfer directly to privacy-engineering-adjacent measurement work. Gaps: No privacy-preserving measurement / signal-loss experience; IC track vs. current manager track</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
@@ -3320,11 +3320,11 @@
         </is>
       </c>
       <c r="Q39" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>Manager-level customer-programs role, several levels below candidate's Senior Director scope, and a different function. This is a marketing operations/partnerships role that happens to have "measurement" in the title; it isn't a data science or causal measurement leadership seat, and the level is a clear downgrade. Gaps: Function is co-marketing/partner programs, not measurement science; Title level (Manager) is well below Senior Director</t>
+          <t>Plain 'Manager' title is a step down from Senior Director, and the function (customer/co-marketing program management) is not data science or measurement leadership. This is a marketing operations/partnerships role that happens to touch measurement, not a role that owns measurement methodology or a data science team. Function drift from candidate's actual expertise. Gaps: Not a DS/analytics leadership role — program management function; Title level below current role</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
@@ -3402,7 +3402,7 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>Software engineering IC role; candidate has no software engineering background — not adjacent to candidate's career at all. This role builds experimentation infrastructure/tooling and requires production software engineering skills the resume doesn't show anywhere. Gaps: No software engineering title or experience; Not a data science or measurement leadership function</t>
+          <t>Software engineering IC role — candidate has no software engineering track record; this is a different profession, not just a different level. Candidate is a data science/analytics leader, not an engineer. Building experimentation platform infrastructure requires production software engineering skills not evidenced anywhere in the resume. Gaps: No software engineering background; Wrong function entirely</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
@@ -3480,7 +3480,7 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Partner II is a junior/associate-level client-facing title, multiple levels below candidate's Senior Director role. This is an entry-to-mid analyst/client-partner role bolted onto Pinterest's tvScientific product — a significant step down in scope for someone currently leading a measurement team at a holding-company agency. Gaps: Title/level (II) is junior relative to a decade of director-level experience; Role is client-facing partner support, not measurement science leadership</t>
+          <t>'Partner II' is a junior individual-contributor client-facing role — several levels below candidate's current Senior Director scope. This is a junior measurement-partner role, likely early-career or associate-level client support work. Massive level mismatch against a decade of director-level leadership. Gaps: Level mismatch (junior IC vs. Senior Director); Would be a significant step backward in scope and compensation</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
@@ -3558,11 +3558,11 @@
         </is>
       </c>
       <c r="Q42" t="n">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>Senior Manager is a step down from candidate's Senior Director title, and Singapore is a major relocation ask. Domain and management track both fit reasonably, but the title downgrade plus international relocation make this a compromised match regardless of skill overlap. Gaps: Requires relocation to Singapore with no signal candidate is pursuing this; Title level (Senior Manager) is below current Senior Director</t>
+          <t>Senior Manager is roughly comparable level/track to current Senior Director, but the role is based in Singapore — a hard geographic mismatch, not a fixable gap. Domain and level are a reasonable match on paper, but this is an APAC regional leadership seat requiring relocation to Singapore, which isn't a resume gap so much as a life/logistics blocker that should dominate the verdict. Gaps: Requires relocation to Singapore; APAC market/regulatory context is unfamiliar territory</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
@@ -3636,11 +3636,11 @@
         </is>
       </c>
       <c r="Q43" t="n">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>Staff DS is a senior IC role; candidate has been a people manager since 2020 — a track change despite strong forecasting domain overlap. Forecasting domain overlap is real (candidate built the exact revenue forecasting suite OMD uses for Gap budget allocation), but the role is IC-only at a large internal platform, a different context than candidate's agency/brand-side career. Gaps: IC vs manager track mismatch; No large-scale internal platform/consumer-tech company experience</t>
+          <t>Currently a people-manager; Staff Data Scientist is a senior IC role — a track change and likely a step down in scope of authority even though the title sounds senior. Candidate has real forecasting experience (OMD revenue forecasting suite) but as a builder-and-owner of a team's output, not as a deep hands-on IC statistician. Staff DS roles at this level expect heavier applied-stats/ML depth than the resume's scikit-learn/statsmodels stack suggests. Gaps: Manager-to-senior-IC track change; Depth of applied statistical forecasting methods (vs. team-managed output) untested</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
@@ -3714,11 +3714,11 @@
         </is>
       </c>
       <c r="Q44" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>Product manager function — candidate has no PM background or title; this is a function drift, not a level issue. Requires product management skills (roadmapping, spec-writing, cross-functional PM ownership) not evidenced anywhere in a career that is entirely data science and analytics leadership. Gaps: No product management experience or title; Function mismatch: PM vs. data science/measurement leadership</t>
+          <t>Product management track, not data science/analytics — function drift regardless of level. This is a PM role that happens to sit on ads measurement; it requires product roadmap ownership and cross-functional PM skills, not causal inference or measurement science expertise. No PM experience on the resume. Gaps: No product management track record; Different core skill set (roadmap/prioritization vs. modeling/measurement)</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
@@ -3796,7 +3796,7 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>Software engineering IC role; entirely outside candidate's function. Requires production software/data engineering skills for measurement signal infrastructure; candidate's stack is Python/SQL/Snowflake for modeling and analysis, not systems engineering. Gaps: No software engineering title or experience; Not a data science/measurement leadership function</t>
+          <t>Software engineering IC role — wrong profession, not just wrong level. Same mismatch as the Anthropic SWE role: candidate has no software engineering background to build measurement signal infrastructure. Gaps: No software engineering background</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
@@ -3870,11 +3870,11 @@
         </is>
       </c>
       <c r="Q46" t="n">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>Senior Staff is IC-ladder, still a track mismatch against candidate's manager career; remote-Ontario adds a cross-border employment question. Experimentation is a genuine strength, but this is a deep technical IC seat, and the consumer-platform context plus Canadian location/work-authorization logistics compound the fit problem. Gaps: IC vs manager track mismatch; Remote-Canada location raises work authorization questions for a US-based candidate</t>
+          <t>Senior Staff DS is a high-bar IC track; candidate's track is people-management, and the domain (consumer/product growth experimentation) is a step away from marketing measurement. This role is about product experimentation (feature-level A/B testing, growth metrics) rather than marketing science (MMM, attribution, media incrementality). Candidate's causal-inference experience is marketing-specific, not product-growth-specific. Gaps: Domain drift: product/growth experimentation vs. marketing measurement; IC track vs. manager track</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
@@ -3956,7 +3956,7 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>IC-ladder role based in Toronto; track mismatch plus relocation/work-authorization issue on top of privacy/signals function drift. Same core issues as the sibling US posting — privacy/signals infra skew and IC track — plus a Toronto location requiring relocation or Canadian work authorization. Gaps: IC vs manager track mismatch; Toronto location requires relocation/Canadian work authorization</t>
+          <t>Same as the other Reddit 'Ads Measurement, Signals, Privacy' postings — senior IC role in a privacy-engineering-adjacent niche outside candidate's track and specialty. Duplicate posting (Toronto) of the same specialized signals/privacy measurement role; assessment is identical to the US/remote version. Gaps: No privacy-preserving measurement experience; IC track vs. manager track</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
@@ -4034,11 +4034,11 @@
         </is>
       </c>
       <c r="Q48" t="n">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>Currently Senior Director managing a team of 5; Staff DS is a senior IC role — a track reversal, not a lateral move, and a step down in title trajectory. The measurement/causal-inference/attribution domain vocabulary overlaps with the candidate's background, but this is a platform-side ads-signals-and-privacy engineering role (conversion signals, privacy-preserving measurement infra) rather than agency/brand-side marketing science. Candidate's MMM and MTA work has been client-facing and strategy-adjacent, not building measurement infrastructure for an ad platform's own advertiser base. Gaps: No clean-rooms or privacy-preserving measurement infrastructure experience (candidate's own notes flag this as a critical gap); Track mismatch: would move from people-manager (Senior Director, team of 5) into a senior IC seat; No ad-platform-side experience — background is entirely agency/brand-side measurement, not building signals/attribution products for advertisers on a platform</t>
+          <t>Duplicate posting (Toronto) of the same Staff-level signals/privacy measurement role — same verdict as the US/remote listing. Identical role/specialty mismatch as the other postings in this family. Gaps: No privacy-preserving measurement experience; IC track vs. manager track</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
@@ -4116,11 +4116,11 @@
         </is>
       </c>
       <c r="Q49" t="n">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Candidate is a people-manager (Senior Director leading a team of 5); Staff DS is a senior IC seat — a track change and likely a step down in scope of authority even if titles look comparable on paper. Domain overlaps genuinely (ads measurement is adjacent to marketing science), but this is a hands-on IC role at an ads platform requiring deep signals/privacy engineering work, not the team-leadership and vendor-adjudication work the candidate has been doing since 2021. The 'Signals, Privacy' framing points to post-cookie/clean-room measurement infrastructure, which the candidate's own notes flag as a gap. Gaps: No clean-room or privacy-preserving measurement experience (explicitly named in the JD; explicitly flagged as a gap in candidate's own positioning notes); Track mismatch: candidate has been a people-manager for 5+ years, this is a senior individual-contributor seat; Toronto location vs. NY-based candidate — likely relocation/visa friction</t>
+          <t>Duplicate posting (Toronto) of the same Staff-level signals/privacy measurement role — same verdict as the US/remote listing. Identical role/specialty mismatch as the other postings in this family. Gaps: No privacy-preserving measurement experience; IC track vs. manager track</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
@@ -4188,16 +4188,16 @@
         </is>
       </c>
       <c r="Q50" t="n">
-        <v>42</v>
+        <v>64</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Track mismatch: candidate has been on a people-manager/Director track since 2021 (Senior Director at OMD managing 5, prior Director roles at Zenith/Merkle); this is an IC 'Staff Data Scientist' seat with no direct reports and an expectation of hands-on coding/pipeline-building, not a management role. Domain fit is about as close as it gets — MMM, MTA, geo-holdout incrementality, causal inference for marketing spend — this is literally the candidate's stated target keyword list. But the role is an IC title after four-plus years of manager/Director titles, and the JD wants someone who personally codes production pipelines rather than directs a team that does; that's a track and title step-down even though the strategic scope described (set 2-3yr roadmap, influence leadership) sounds Director-equivalent. Gaps: IC 'Staff' title vs. current and recent Director/Senior Director people-manager titles — reads as a downgrade on paper regardless of actual scope; JD requires an advanced degree (MS/PhD) in a quantitative field — not evident on the resume; JD wants hands-on production ML pipeline building day-to-day; candidate's last several roles are oversight/leadership of teams that build, not hands-on IC coding at that level</t>
+          <t>Staff DS is a senior IC role — mentors junior scientists but doesn't manage a team, which is a track change from candidate's current Senior Director (team of 5) role. Level itself is comparable seniority, just a different track. The domain is a near-perfect bullseye: MMM, MTA, incrementality testing, geo-holdout, marketing budget allocation — literally the candidate's core keyword list and recent OMD work. The compromise is track (IC vs. manager) and an unconfirmed advanced-degree requirement (MS/PhD) that the resume doesn't establish. Gaps: Role is IC (mentors, doesn't manage) — step back from current people-manager scope; Minimum quals ask for an advanced degree in a quantitative field, not evidenced on the resume</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>research</t>
+          <t>apply</t>
         </is>
       </c>
       <c r="T50" t="inlineStr">
@@ -4258,11 +4258,11 @@
         </is>
       </c>
       <c r="Q51" t="n">
-        <v>55</v>
+        <v>66</v>
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>Director + people-manager track matches current level exactly, but this is product/growth analytics, not marketing measurement. Deep causal inference and experimentation chops transfer directly, and leading a DS team is exactly what this candidate does now. But the domain is product analytics for a marketplace vertical (grocery/alcohol/retail ops), not marketing science — no MMM, attribution, or media measurement in scope at all. Gaps: No consumer marketplace/product-analytics background (vs. media/marketing measurement); JD wants 0→1 product experimentation, not brand/channel measurement</t>
+          <t>Director level managing a team of DS/analytics leaders — same level and same people-manager track as candidate's current Senior Director role. Strong level and track match: leading a team, experimentation and causal inference as core tools, cross-functional influence with Product/Eng/Finance. The gap is domain — this is general consumer/product analytics for a delivery vertical, not marketing measurement/MMM/attribution, so the specific marketing-science expertise is underused here. Gaps: Domain is product/consumer analytics, not marketing measurement — MMM/MTA background is largely irrelevant here; No consumer marketplace/delivery industry experience</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
@@ -4394,11 +4394,11 @@
         </is>
       </c>
       <c r="Q53" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>VP at a bank is a mid-level IC/manager title, roughly a step below the candidate's current Senior Director seat — comp range (130-195k) confirms it. Marketing data science is the right domain, but the level and comp band both signal this sits below where the candidate is already operating. Taking this would be a step down in scope and title, not a lateral move. Gaps: Title/level is below current Senior Director seniority; Comp ceiling (195k) is below likely current comp</t>
+          <t>Banking 'VP' is a mid-level title, not equivalent to corporate VP — likely a step down from current Senior Director seat. No JD excerpt to confirm scope, so this is judged on title and comp band alone. Marketing data science domain is directionally right, but the title tier and the 130-195k range both sit below where the candidate is already operating. Gaps: No JD detail on scope/seniority to confirm it's not a step down; Comp band below current trajectory</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
@@ -4468,11 +4468,11 @@
         </is>
       </c>
       <c r="Q54" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>Partner at a strategy consultancy is a sales-and-firm-equity role; candidate is a Senior Director / Principal Consultant with ~10 years leadership, not the 15+ years and BD/P&amp;L track record this title implies. This is fundamentally a rainmaker role — selling engagements, owning commercial targets, and overseeing (not doing) technical work across DCM, qualitative research, and brand tracking. Candidate's strength is hands-on causal/measurement science and shipping production systems, which is explicitly not what this JD wants ("without requiring direct coding or model deployment"). Gaps: No demonstrated business-development / sales quota ownership at a consultancy — candidate's agency roles were delivery-focused, not rainmaking; No discrete choice modeling, brand tracking, or qualitative/primary research experience — core methods listed in the JD; 15+ years leadership required; candidate has ~10, and none of it at Partner-equivalent title in a consultancy</t>
+          <t>Equity Partner with firm-wide P&amp;L and 15+ years consulting-specific leadership — a different track than anything on the resume. This is a market-research/consulting practice-leadership role (segmentation, DCMs, brand tracking, qualitative) overseeing specialists without touching models directly — not causal inference or measurement science. Candidate has consultancy exposure via Arjentic as a principal, not partner-level firm leadership at a major consultancy with vendor/qual research oversight. Gaps: No track record as an equity partner or P&amp;L owner at a professional-services firm; Core expertise is causal/measurement, not discrete-choice/qualitative market research</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
@@ -4612,11 +4612,11 @@
         </is>
       </c>
       <c r="Q56" t="n">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>Title-for-title match: Senior Director, Marketing Science is the candidate's current exact title and level. This is squarely in-lane — marketing science leadership at the Senior Director level, same as the current OMD role. Comp (150-200k) is lower than current band, likely reflecting sports/entertainment budgets rather than agency holding-co scale, but the role itself is a real match. Gaps: Comp likely below current level; Sports/entertainment measurement maturity may be less developed than agency-side MMM work — could mean more building-from-scratch</t>
+          <t>Title parity with current role (Senior Director) — same level, same track. Exact title and function match to what the candidate does today and to career goal #1. Sports/media marketing science plausibly touches attribution, fan segmentation, and media measurement, all core strengths. Gaps: No JD detail yet on whether it's attribution/MMM-heavy or more reporting-focused; Sports-specific domain knowledge unproven</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
@@ -4686,11 +4686,11 @@
         </is>
       </c>
       <c r="Q57" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>Director level matches, but track is applied ML/ads science (ranking, ad systems), not measurement/causal inference leadership. This is an ads ML science role — building ranking and ad-serving models — not marketing measurement. The candidate has no applied ML/ads infrastructure background; the overlap is keyword-level ("ads", "director") not substantive. Gaps: No ad-ranking/ad-serving ML systems experience; Function is applied ML engineering leadership, not causal measurement</t>
+          <t>Director level matches, but the track is applied ML/ads-infrastructure science, not marketing/measurement science. This reads as an ads-ranking/auction ML leadership role (large-scale model systems for an ads marketplace), a different technical center of gravity than causal inference and measurement. Candidate has shipped propensity/recommendation models, but not ads-serving ML at this scale or specificity. Gaps: No large-scale ads ranking/auction ML experience; Domain is applied ML engineering leadership, not measurement/causal science</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
@@ -4760,16 +4760,16 @@
         </is>
       </c>
       <c r="Q58" t="n">
-        <v>40</v>
+        <v>52</v>
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>Title is vague ("Applied Science / Data Science Leader") and skews toward a research/ML IC-adjacent track rather than a clear people-management measurement seat. Attentive is a marketing/messaging platform, so there's plausible domain adjacency, but "Applied Science" framing plus the high comp band suggests they want deep ML/research depth (likely for their own product's ML models) rather than a marketing measurement strategist. Gaps: Unclear if role is measurement-facing or product-ML-facing; "Applied Science" track typically wants hands-on modeling depth beyond marketing science scope</t>
+          <t>Title is ambiguous ('leader' could mean senior IC or people-manager) — needs clarification before assuming level parity. Attentive is an SMS/email marketing platform, and the candidate directly built production propensity and recommendation models for Email, SMS, and Push at Samsung — a real, specific overlap. But the vague title makes it unclear if this is a management seat or a senior IC seat, which matters given the candidate's current people-manager track. Gaps: Title doesn't confirm people-manager vs. IC track; No JD detail on whether it's measurement-focused or pure applied ML</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>skip</t>
+          <t>research</t>
         </is>
       </c>
       <c r="T58" t="inlineStr">
@@ -4830,11 +4830,11 @@
         </is>
       </c>
       <c r="Q59" t="n">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>Head of DS level is right, but domain is healthcare AI/clinical documentation — total function drift from marketing science. Abridge builds clinical documentation AI. There is no marketing, measurement, or causal-inference-for-commercial-decisions angle here; this would require an entirely different domain expertise (healthcare NLP/ML). Gaps: Zero healthcare/clinical domain experience; No NLP/LLM applied research background</t>
+          <t>Head of Data Science title level is fine, but the domain is a hard break from marketing/measurement science. Abridge builds clinical documentation AI — this is healthcare NLP/ML, with none of the marketing measurement, attribution, or causal inference DNA the candidate has built a career on. Nothing on the resume speaks to clinical data science. Gaps: No healthcare or clinical NLP experience; Zero overlap with measurement/marketing science domain</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
@@ -4904,7 +4904,7 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>Level matches exactly (Senior Director), but the generic "Data Science" title leaves the actual scope (subscriber/content analytics vs. marketing measurement) unclear. Media/entertainment is a plausible adjacent industry and the level is right, but without JD detail on whether this is marketing measurement, streaming subscriber analytics, or content ML, it's a bet on title alone. Worth researching before committing. Gaps: JD doesn't confirm marketing/measurement scope vs. broader subscriber or content data science; No streaming/media subscription analytics track record</t>
+          <t>Title parity with current Senior Director role — level and track match. Media/entertainment company at the right seniority level, and if this role touches ad measurement, content/subscriber analytics, or MMM it would be a strong match. Without JD detail on scope, this is a plausible but unconfirmed fit. Gaps: No JD detail confirming measurement/attribution focus vs. general subscriber/content DS; Media vertical experience not on resume (agency-side media measurement is adjacent but not the same as in-house media company DS)</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
@@ -26994,11 +26994,11 @@
         </is>
       </c>
       <c r="Q387" t="n">
-        <v>90</v>
+        <v>80</v>
       </c>
       <c r="R387" t="inlineStr">
         <is>
-          <t>SVP at a bank is a senior leadership title (roughly Director/Senior Director equivalent in tech) and matches current level and trajectory exactly. This is close to a direct restatement of the candidate's resume: attribution, MMM, incrementality testing, vendor management, cross-channel measurement narrative for senior stakeholders. Rare case where domain, level, and function all line up. Gaps: No banking/regulated-industry experience (compliance, legal, procurement rigor called out in JD); Clean rooms/adtech tool depth (DSP/SSP, identity solutions) is a stated gap vs. the candidate's agency-side background</t>
+          <t>SVP is a genuine step up from Senior Director — right direction, and the JD's scope (attribution, MMM, incrementality, team leadership) matches current-level responsibilities. This is squarely the candidate's core domain — attribution, MMM, incrementality testing, vendor evaluation, and translating measurement into stakeholder narratives — all things done at OMD and Zenith. The explicit call-out of MMM and incrementality testing lines up with career goal #1 almost exactly. Gaps: No client-side big-bank/regulated-industry experience (compliance, legal, procurement rigor called out in JD); Clean rooms experience gap not addressed by this JD but may surface in interview</t>
         </is>
       </c>
       <c r="S387" t="inlineStr">
@@ -32472,7 +32472,7 @@
       </c>
       <c r="R468" t="inlineStr">
         <is>
-          <t>Completely different function — hardware/GPU infrastructure program management, not data science or measurement at any level. No overlap whatsoever: this role is about physical GPU cluster bring-up, networking, power, and cooling logistics. Nothing in the candidate's background — marketing science, causal inference, team leadership in analytics — applies here. Gaps: No infrastructure/hardware program management experience; No compute/datacenter operations background</t>
+          <t>Irrelevant — this is a hardware/infrastructure TPM role, not a data science or measurement track at any level. This is GPU cluster bring-up program management (networking, power, cooling, hyperscaler ops) — a completely different discipline from marketing science and causal measurement. Nothing on the resume speaks to this. Gaps: No infrastructure/hardware program management background; No technical program management track record at all</t>
         </is>
       </c>
       <c r="S468" t="inlineStr">
@@ -32538,11 +32538,11 @@
         </is>
       </c>
       <c r="Q469" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="R469" t="inlineStr">
         <is>
-          <t>Title-senior but a deep ML/RL research IC-track role requiring a PhD — different track entirely from marketing science leadership. This wants a hands-on RL/LLM post-training researcher building environment-and-reward systems for agent training. The candidate's causal inference and marketing measurement background doesn't translate to this research agenda. Gaps: No PhD or RL/LLM post-training research background; No agent environment/eval engineering experience</t>
+          <t>Requires a PhD-level RL/LLM post-training research track record — a different career entirely from applied marketing measurement leadership. This is a hands-on research role building RL environments and post-training methods for agentic models at a frontier AI startup. Nothing in the candidate's background (marketing science, causal inference, MMM) touches RL, LLM post-training, or agent evaluation research. Gaps: No PhD or research publication track record in ML/RL; No LLM post-training or agent environment engineering experience</t>
         </is>
       </c>
       <c r="S469" t="inlineStr">

</xml_diff>